<commit_message>
added doc table, modal create return
</commit_message>
<xml_diff>
--- a/client/public/Sorce/balanceDP.xlsx
+++ b/client/public/Sorce/balanceDP.xlsx
@@ -14,12 +14,12 @@
 </file>
 
 <file path=xl/SharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="421">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="436">
   <si>
     <t>Формирвоание отчета</t>
   </si>
   <si>
-    <t>Период: на 16.01.2026 15:05:13</t>
+    <t>Период: на 30.01.2026 8:15:13</t>
   </si>
   <si>
     <t>Показатели: Свободный остаток(В ед. хранения);</t>
@@ -71,21 +71,27 @@
     <t>Lacmi Гарячий шоколад УБ 20г /90шт</t>
   </si>
   <si>
+    <t>Lacmi Гарячий шоколад УБ 20г /90шт АКЦІЯ ВІП</t>
+  </si>
+  <si>
     <t>Желе ананас УБ 78г /56шт</t>
   </si>
   <si>
+    <t>Желе ананас УБ 78г /56шт АКЦІЯ ВІП</t>
+  </si>
+  <si>
     <t>Желе ананас УБ 78г /56шт АКЦІЯ ОПТ</t>
   </si>
   <si>
     <t>Желе апельсин УБ 78г /56шт</t>
   </si>
   <si>
-    <t>Желе апельсин УБ 78г /56шт АКЦІЯ</t>
-  </si>
-  <si>
     <t>Желе вишня УБ 78г /56шт</t>
   </si>
   <si>
+    <t>Желе вишня УБ 78г /56шт АКЦІЯ ВІП</t>
+  </si>
+  <si>
     <t>Желе вишня УБ 78г /56шт АКЦІЯ ОПТ</t>
   </si>
   <si>
@@ -95,16 +101,25 @@
     <t>Желе ківі УБ 78г /56шт АКЦІЯ</t>
   </si>
   <si>
+    <t>Желе ківі УБ 78г /56шт АКЦІЯ ВІП</t>
+  </si>
+  <si>
     <t>Желе ківі УБ 78г /56шт АКЦІЯ ОПТ</t>
   </si>
   <si>
+    <t>Желе Лісова ягода УБ 78г /56шт</t>
+  </si>
+  <si>
+    <t>Желе Лісова ягода УБ 78г /56шт АКЦІЯ ВІП</t>
+  </si>
+  <si>
     <t>Желе Лісова ягода УБ 78г /56шт АКЦІЯ ОПТ</t>
   </si>
   <si>
     <t>Желе полуниця УБ 78г /56шт</t>
   </si>
   <si>
-    <t>Желе полуниця УБ 78г /56шт АКЦІЯ ОПТ</t>
+    <t>Желе полуниця УБ 78г /56шт АКЦІЯ ВІП</t>
   </si>
   <si>
     <t>Какао-порошок 22% УБ 60г /26шт</t>
@@ -137,9 +152,18 @@
     <t>Лимонна кислота УБ 25г /55шт</t>
   </si>
   <si>
+    <t>Суміш для приготування Грибного соусу УБ 36г /34шт</t>
+  </si>
+  <si>
     <t>Суміш для приготування Грибного соусу УБ 36г /34шт /</t>
   </si>
   <si>
+    <t>Суміш для приготування Грибного соусу УБ 36г /34шт /АКЦІЯ</t>
+  </si>
+  <si>
+    <t>Суміш для приготування Грибного соусу УБ 36г /34шт /АКЦІЯ ВІП</t>
+  </si>
+  <si>
     <t>Суміш для приготування Грибного соусу УБ 36г /34шт АКЦІЯ ВІП</t>
   </si>
   <si>
@@ -149,12 +173,21 @@
     <t>Суміш для приготування соусу Болоньєзе УБ 40г /32шт /</t>
   </si>
   <si>
+    <t>Суміш для приготування соусу Болоньєзе УБ 40г /32шт /АКЦІЯ ВІП</t>
+  </si>
+  <si>
     <t>Суміш для приготування соусу Болоньєзе УБ 40г /32шт АКЦІЯ ВІП</t>
   </si>
   <si>
     <t>Суміш для приготування соусу Карбонара УБ 36г /34шт</t>
   </si>
   <si>
+    <t>Суміш для приготування соусу Карбонара УБ 36г /34шт /</t>
+  </si>
+  <si>
+    <t>Суміш для приготування соусу Карбонара УБ 36г /34шт /АКЦІЯ ВІП</t>
+  </si>
+  <si>
     <t>Суміш для приготування соусу Карбонара УБ 36г /34шт АКЦІЯ ВІП</t>
   </si>
   <si>
@@ -281,9 +314,6 @@
     <t>Перець чорний мелений УБ 20г /38шт</t>
   </si>
   <si>
-    <t>Перець чорний мелений УБ 20г /38шт АКЦІЯ</t>
-  </si>
-  <si>
     <t>Перець чорний мелений УБ 20г /38шт АКЦІЯ ВІП</t>
   </si>
   <si>
@@ -296,9 +326,6 @@
     <t>Суміш перців Класична УБ 30г /24шт</t>
   </si>
   <si>
-    <t>Суміш перців Класична УБ 30г /24шт АКЦІЯ ВІП</t>
-  </si>
-  <si>
     <t>РОШЕН</t>
   </si>
   <si>
@@ -308,9 +335,15 @@
     <t>Батон ROSHEN "Double peanuts" мол-шок з арахісом та арахісовим кремом ВКФ 39г /180шт UA TP</t>
   </si>
   <si>
+    <t>Батон ROSHEN "Double peanuts" мол-шок з арахісом та арахісовим кремом ВКФ 39г /180шт UA TP АКЦІЯ ОПТ</t>
+  </si>
+  <si>
     <t>Батон ROSHEN з начинкою ВКФ 43г /180шт /</t>
   </si>
   <si>
+    <t>Батон ROSHEN з начинкою ВКФ 43г /180шт /АКЦІЯ ОПТ</t>
+  </si>
+  <si>
     <t>Батон ROSHEN з начинкою ВКФ 43г /180шт /АКЦІЯ Цінова</t>
   </si>
   <si>
@@ -320,27 +353,30 @@
     <t>Батон ROSHEN мол-шок з карамельною начинкою ВКФ 40г /180шт /</t>
   </si>
   <si>
-    <t>Батон ROSHEN мол-шок з карамельною начинкою ВКФ 40г /180шт /АКЦІЯ Цінова</t>
-  </si>
-  <si>
-    <t>Батон ROSHEN мол-шок з кокосом та мигдалем ВКФ 38г /180шт /</t>
-  </si>
-  <si>
-    <t>Батон ROSHEN мол-шок з кокосом та мигдалем ВКФ 38г /180шт /АКЦІЯ Цінова</t>
+    <t>Батон ROSHEN мол-шок з карамельною начинкою ВКФ 40г /180шт /АКЦІЯ ОПТ</t>
   </si>
   <si>
     <t>Батон ROSHEN мол-шок з кокосом та мигдалем ВКФ 38г /180шт UA TP</t>
   </si>
   <si>
+    <t>Батон ROSHEN мол-шок з кокосом та мигдалем ВКФ 38г /180шт UA TP АКЦІЯ ОПТ</t>
+  </si>
+  <si>
     <t>Батон ROSHEN молочно-шоколадний з арахісовою начинкою ВКФ 38г /180шт UA TP</t>
   </si>
   <si>
+    <t>Батон ROSHEN молочно-шоколадний з арахісовою начинкою ВКФ 38г /180шт UA TP АКЦІЯ ОПТ</t>
+  </si>
+  <si>
     <t>Батон ROSHEN молочно-шоколадний з начинкою крем-брюле ВКФ 43г /180шт /АКЦІЯ Цінова</t>
   </si>
   <si>
     <t>Батон ROSHEN молочно-шоколадний з начинкою крем-брюле ВКФ 43г /180шт UA TP</t>
   </si>
   <si>
+    <t>Батон ROSHEN молочно-шоколадний з начинкою крем-брюле ВКФ 43г /180шт UA TP АКЦІЯ ОПТ</t>
+  </si>
+  <si>
     <t>БІСКВІТИ</t>
   </si>
   <si>
@@ -395,6 +431,9 @@
     <t>Roshetto milk ВКФ 34г /200шт</t>
   </si>
   <si>
+    <t>Roshetto milk ВКФ 34г /200шт АКЦІЯ</t>
+  </si>
+  <si>
     <t>Roshetto Peanut ВКФ 34г /200шт</t>
   </si>
   <si>
@@ -509,9 +548,6 @@
     <t>Yummi Gummi Cherry ВКФ 70г /22шт</t>
   </si>
   <si>
-    <t>Yummi Gummi Cherry ВКФ 70г /22шт АКЦІЯ Цінова</t>
-  </si>
-  <si>
     <t>Yummi Gummi CupCakes ВКФ 70г /22шт</t>
   </si>
   <si>
@@ -530,9 +566,6 @@
     <t>Yummi Gummi Duo Mix ВКФ 70г /22шт</t>
   </si>
   <si>
-    <t>Yummi Gummi Duo Mix ВКФ 70г /22шт АКЦІЯ Цінова</t>
-  </si>
-  <si>
     <t>Yummi Gummi Fizzy Worms ВКФ 70г /22шт</t>
   </si>
   <si>
@@ -542,6 +575,9 @@
     <t>Yummi Gummi Fluffi Barbecue ВКФ 200г /7шт</t>
   </si>
   <si>
+    <t>Yummi Gummi Fluffi Barbecue ВКФ 200г /7шт АКЦІЯ Цінова</t>
+  </si>
+  <si>
     <t>Yummi Gummi Fluffi Barbecue ВКФ 200г /7шт АКЦІЯ Цінова UA</t>
   </si>
   <si>
@@ -551,6 +587,9 @@
     <t>Yummi Gummi Fluffi Rainbow Turbines ВКФ 65г /11шт</t>
   </si>
   <si>
+    <t>Yummi Gummi Fluffi Rainbow Turbines ВКФ 65г /11шт АКЦІЯ Цінова UA</t>
+  </si>
+  <si>
     <t>Yummi Gummi Fluffi Soft Hearts ВКФ 65г /11шт</t>
   </si>
   <si>
@@ -560,6 +599,12 @@
     <t>Yummi Gummi Fluffi Soft Hearts ВКФ 65г /11шт АКЦІЯ Цінова накладна UA</t>
   </si>
   <si>
+    <t>Yummi Gummi Fluffi Teeny Tiny Bits ВКФ 65г /11шт</t>
+  </si>
+  <si>
+    <t>Yummi Gummi Fluffi Teeny Tiny Bits ВКФ 65г /11шт АКЦІЯ Цінова UA</t>
+  </si>
+  <si>
     <t>Yummi Gummi Fluffy Sheep ВКФ 70г /22шт</t>
   </si>
   <si>
@@ -575,9 +620,6 @@
     <t>Yummi Gummi Funny Cola ВКФ 70г /22шт</t>
   </si>
   <si>
-    <t>Yummi Gummi Funny Cola ВКФ 70г /22шт АКЦІЯ Цінова</t>
-  </si>
-  <si>
     <t>Yummi Gummi Galaxy Life ВКФ 70г /22шт</t>
   </si>
   <si>
@@ -593,12 +635,12 @@
     <t>Yummi Gummi Mini Bear Mix ВКФ 70г /22шт АКЦІЯ Цінова накладна</t>
   </si>
   <si>
+    <t>Yummi Gummi Pasta ВКФ 70г /22шт</t>
+  </si>
+  <si>
     <t>Yummi Gummi Smile Mix ВКФ 70г /22шт</t>
   </si>
   <si>
-    <t>Yummi Gummi Smile Mix ВКФ 70г /22шт АКЦІЯ Цінова</t>
-  </si>
-  <si>
     <t>Yummi Gummi Sour Belts ВКФ 70г /40шт</t>
   </si>
   <si>
@@ -608,9 +650,6 @@
     <t>Yummi Gummi Sour Sticks ВКФ 70г /40шт</t>
   </si>
   <si>
-    <t>Yummi Gummi Sour Sticks ВКФ 70г /40шт АКЦІЯ Цінова</t>
-  </si>
-  <si>
     <t>Yummi Gummi Sour Strawberries ВКФ 70г /22шт</t>
   </si>
   <si>
@@ -761,9 +800,15 @@
     <t>Assortment Classic 154г/8</t>
   </si>
   <si>
+    <t>Assortment Classic ВКФ 154г /8шт АКЦІЯ</t>
+  </si>
+  <si>
     <t>Assortment Elegant 145г/8</t>
   </si>
   <si>
+    <t>Cherry Queen heart РЦ 122г /8шт</t>
+  </si>
+  <si>
     <t>Cherry Queen heart РЦ 122г /8шт АКЦІЯ ВІП</t>
   </si>
   <si>
@@ -776,10 +821,13 @@
     <t>Roshen Compliment ВКФ 145г /8шт</t>
   </si>
   <si>
+    <t>Roshen Compliment ВКФ 145г /8шт АКЦІЯ ВІП</t>
+  </si>
+  <si>
     <t>Roshen вишня з вишневим лікером ВКФ 155г /10шт /</t>
   </si>
   <si>
-    <t>Shooters віски-лікер ВКФ 150г /10шт /</t>
+    <t>Shooters віски-лікер ВКФ 150г /10шт /АКЦІЯ ВІП 1</t>
   </si>
   <si>
     <t>Shooters з бренді-лікером ВКФ 150г /10шт /</t>
@@ -788,9 +836,15 @@
     <t>Shooters з ромовим лікером ВКФ 150г /10шт /</t>
   </si>
   <si>
+    <t>Shooters з ромовим лікером ВКФ 150г /10шт /АКЦІЯ ВІП 1</t>
+  </si>
+  <si>
     <t>Київ вечірній ВКФ 176г /7шт</t>
   </si>
   <si>
+    <t>Київ вечірній ВКФ 176г /7шт АКЦІЯ</t>
+  </si>
+  <si>
     <t>Київ вечірній ВКФ 352г /7шт</t>
   </si>
   <si>
@@ -806,6 +860,9 @@
     <t>2 CRACK з молочно-ванільною начинкою ККФ 190г /26шт</t>
   </si>
   <si>
+    <t>2 CRACK з начинкою какао-горіх ККФ 190г /26шт</t>
+  </si>
+  <si>
     <t>2 CRACK з шоколадною начинкою ККФ 190г /26шт</t>
   </si>
   <si>
@@ -947,9 +1004,6 @@
     <t>Johnny Krocker choco ВКФ 1кг /4шт PL</t>
   </si>
   <si>
-    <t>Johnny Krocker choco ВКФ 1кг /4шт АКЦІЯ ВІП 1</t>
-  </si>
-  <si>
     <t>Johnny Krocker coconut ВКФ 1кг /4шт</t>
   </si>
   <si>
@@ -962,9 +1016,6 @@
     <t>Johnny Krocker milk ВКФ 1кг /4шт АКЦІЯ ВІП 1</t>
   </si>
   <si>
-    <t>Ko-Ko Choco White ВКФ 1кг /5пак АКЦІЯ ВІП</t>
-  </si>
-  <si>
     <t>KONAFETTO blanc ККФ 1кг /5пак /</t>
   </si>
   <si>
@@ -986,9 +1037,6 @@
     <t>Sorrento ВКФ 1кг /9пак</t>
   </si>
   <si>
-    <t>Sorrento ВКФ 1кг /9пак АКЦІЯ ВІП 1</t>
-  </si>
-  <si>
     <t>Кара-Кум ВКФ 1кг /7пак</t>
   </si>
   <si>
@@ -998,9 +1046,6 @@
     <t>Ліщина 1кг/6 ВКФ</t>
   </si>
   <si>
-    <t>Ліщина ВКФ 1кг /6пак АКЦІЯ ВІП 1</t>
-  </si>
-  <si>
     <t>Монблан з карамелізованим мигдалем ВКФ 1кг /4пак</t>
   </si>
   <si>
@@ -1022,6 +1067,9 @@
     <t>Ромашка ВКФ 1кг /9пак</t>
   </si>
   <si>
+    <t>Ромашка ВКФ 1кг /9пак АКЦІЯ ВІП</t>
+  </si>
+  <si>
     <t>Сливки-Ленивки 1кг ВКФ</t>
   </si>
   <si>
@@ -1037,9 +1085,6 @@
     <t>Шоколапки ВКФ 1кг /7пак</t>
   </si>
   <si>
-    <t>Шоколапки ВКФ 1кг /7пак АКЦІЯ ВІП 1</t>
-  </si>
-  <si>
     <t>ЦУКЕРКИ ШОКОЛАДНІ ФАСОВАНІ</t>
   </si>
   <si>
@@ -1055,6 +1100,9 @@
     <t>ШОКОЛАД</t>
   </si>
   <si>
+    <t>Lacmi Big Bite молочний ВКФ 200г /17шт</t>
+  </si>
+  <si>
     <t>Lacmi Big Bite молочний ВКФ 260г /15шт /АКЦІЯ ВІП 1</t>
   </si>
   <si>
@@ -1064,18 +1112,15 @@
     <t>Lacmi Black, White &amp; Caramel молочний з молочною начинкою, карамеллю та печивом з какао ВКФ 100г /18шт</t>
   </si>
   <si>
-    <t>Lacmi Black, White &amp; Caramel молочний з молочною начинкою, карамеллю та печивом з какао ВКФ 100г /18шт АКЦІЯ Цінова</t>
-  </si>
-  <si>
-    <t>Lacmi Black, White &amp; Caramel молочний з молочною начинкою, карамеллю та печивом з какао ВКФ 100г /18шт АКЦІЯ Цінова UA</t>
-  </si>
-  <si>
     <t>Lacmi Cool-Nut-Coconut молочний з мигдалем та кокосом ВКФ 280г /12шт</t>
   </si>
   <si>
     <t>Lacmi Crumble-Bumble ВКФ 83г /22шт</t>
   </si>
   <si>
+    <t>Lacmi Crumble-Bumble ВКФ 83г /22шт АКЦІЯ ОПТ</t>
+  </si>
+  <si>
     <t>Lacmi Fun&amp;Crispy молочний пористий з молочною начинкою з кріспі ВКФ 85г /17шт</t>
   </si>
   <si>
@@ -1124,18 +1169,15 @@
     <t>Lacmi молочний з мигдалем та кокосовим кремом ВКФ 84г /22шт</t>
   </si>
   <si>
-    <t>Lacmi молочний з мигдалем та кокосовим кремом ВКФ 84г /22шт АКЦІЯ ОПТ</t>
-  </si>
-  <si>
-    <t>Lacmi молочний з мигдалем та кокосовим кремом ВКФ 84г /22шт АКЦІЯ Цінова</t>
-  </si>
-  <si>
     <t>Lacmi молочний з молочною начинкою та вафлею ВКФ 90г /18шт</t>
   </si>
   <si>
     <t>Lacmi молочний з молочною начинкою та вафлею ВКФ 90г /18шт UA TP</t>
   </si>
   <si>
+    <t>Lacmi молочний з молочною начинкою та вафлею ВКФ 90г /18шт UA TP АКЦІЯ ОПТ</t>
+  </si>
+  <si>
     <t>Lacmi молочний з молочною начинкою та вафлею ВКФ 90г /18шт АКЦІЯ ОПТ</t>
   </si>
   <si>
@@ -1145,12 +1187,15 @@
     <t>Lacmi молочний з молочною начинкою та печивом ВКФ 100г /18шт UA TP</t>
   </si>
   <si>
-    <t>Lacmi молочний з молочною начинкою та печивом ВКФ 100г /18шт UA TP АКЦІЯ ОПТ</t>
+    <t>Lacmi молочний з молочною начинкою та печивом ВКФ 100г /18шт АКЦІЯ ОПТ</t>
   </si>
   <si>
     <t>Lacmi молочний з молочною та шоколадною начинками, вафлею з какао ВКФ 235г /12шт</t>
   </si>
   <si>
+    <t>Lacmi молочний з молочною та шоколадною начинками, вафлею з какао ВКФ 235г /12шт АКЦІЯ ОПТ</t>
+  </si>
+  <si>
     <t>Lacmi молочний з начинкою зі смаком "Полунична панакота" ВКФ 90г /22шт</t>
   </si>
   <si>
@@ -1166,7 +1211,7 @@
     <t>Lacmi молочний з начинкою зі смаком "Тірамісу" та печивом ВКФ 270г /12шт UA TP АКЦІЯ ОПТ</t>
   </si>
   <si>
-    <t>Lacmi молочний з начинкою зі смаком "Тірамісу" та печивом ВКФ 270г /12шт АКЦІЯ Цінова</t>
+    <t>Lacmi молочний з цілим мигдалем ВКФ 90г /20шт</t>
   </si>
   <si>
     <t>Lacmi молочний з цілими лісовими горіхами ВКФ 90г /16шт</t>
@@ -1196,21 +1241,21 @@
     <t>Lacmi молочний з шоколадною начинкою та вафлею ВКФ 90г /18шт UA TP АКЦІЯ ОПТ</t>
   </si>
   <si>
-    <t>Lacmi молочний з шоколадною начинкою та вафлею ВКФ 90г /18шт АКЦІЯ Цінова</t>
-  </si>
-  <si>
     <t>Roshen Nut молочний з цілим мигдалем ВКФ 90г /20шт</t>
   </si>
   <si>
-    <t>Roshen Nut молочний з цілим мигдалем ВКФ 90г /20шт АКЦІЯ Цінова</t>
-  </si>
-  <si>
     <t>Roshen Nut молочний з цілим фундуком ВКФ 90г /18шт</t>
   </si>
   <si>
+    <t>Roshen Nut молочний з цілим фундуком ВКФ 90г /18шт АКЦІЯ Цінова</t>
+  </si>
+  <si>
     <t>Roshen Nut чорний з цілим мигдалем ВКФ 90г /20шт</t>
   </si>
   <si>
+    <t>Roshen Nut чорний з цілим мигдалем ВКФ 90г /20шт АКЦІЯ Цінова UA</t>
+  </si>
+  <si>
     <t>Roshen Nut чорний з цілим фундуком ВКФ 90г /18шт</t>
   </si>
   <si>
@@ -1220,7 +1265,7 @@
     <t>Roshen пористий БІЛИЙ ВКФ 80г /20шт Aerated UA АКЦІЯ ОПТ</t>
   </si>
   <si>
-    <t>Roshen пористий БІЛИЙ ВКФ 80г /20шт FP АКЦІЯ Цінова UA</t>
+    <t>Roshen пористий БІЛИЙ ВКФ 80г /20шт Aerated АКЦІЯ Цінова</t>
   </si>
   <si>
     <t>Roshen пористий білий карамельний ВКФ 80г /20шт Aerated UA</t>
@@ -1256,13 +1301,13 @@
     <t>Roshen чорний Bitter 80% ВКФ 85г /35шт АКЦІЯ ОПТ</t>
   </si>
   <si>
-    <t>Roshen Чорний Brut 80% ВКФ 85г /35шт /</t>
-  </si>
-  <si>
     <t>Roshen чорний Special 56% ВКФ 85г /35шт /</t>
   </si>
   <si>
     <t>Roshen чорний Special 56% ВКФ 85г /35шт /АКЦІЯ ОПТ</t>
+  </si>
+  <si>
+    <t>Roshen чорний з підсоленим подрібн. мигдалем ВКФ 85г /35шт /</t>
   </si>
   <si>
     <t>Roshen чорний термостійкий РЦ 80г /13шт HAL</t>
@@ -1535,7 +1580,7 @@
     <outlinePr summaryBelow="false" summaryRight="false"/>
     <pageSetUpPr autoPageBreaks="false"/>
   </sheetPr>
-  <dimension ref="C421"/>
+  <dimension ref="C436"/>
   <sheetFormatPr defaultColWidth="10.5" customHeight="true" defaultRowHeight="11.429"/>
   <cols>
     <col min="1" max="1" width="2.33203125" style="1" customWidth="true"/>
@@ -1600,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="C11" s="11" t="n">
-        <v>594</v>
+        <v>551</v>
       </c>
     </row>
     <row r="12" ht="11" customHeight="true">
@@ -1608,7 +1653,7 @@
         <v>11</v>
       </c>
       <c r="C12" s="12" t="n">
-        <v>675310</v>
+        <v>575316</v>
       </c>
     </row>
     <row r="13" ht="11" customHeight="true" outlineLevel="1">
@@ -1632,7 +1677,7 @@
         <v>14</v>
       </c>
       <c r="C15" s="12" t="n">
-        <v>157301</v>
+        <v>157685</v>
       </c>
     </row>
     <row r="16" ht="11" customHeight="true" outlineLevel="2">
@@ -1640,7 +1685,7 @@
         <v>15</v>
       </c>
       <c r="C16" s="12" t="n">
-        <v>26151</v>
+        <v>27876</v>
       </c>
     </row>
     <row r="17" ht="11" customHeight="true" outlineLevel="3">
@@ -1648,23 +1693,23 @@
         <v>16</v>
       </c>
       <c r="C17" s="18" t="n">
-        <v>7453</v>
+        <v>3983</v>
       </c>
     </row>
     <row r="18" ht="11" customHeight="true" outlineLevel="3">
       <c r="B18" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="C18" s="18" t="n">
-        <v>2694</v>
+      <c r="C18" s="11" t="n">
+        <v>607</v>
       </c>
     </row>
     <row r="19" ht="11" customHeight="true" outlineLevel="3">
       <c r="B19" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="C19" s="11" t="n">
-        <v>340</v>
+      <c r="C19" s="18" t="n">
+        <v>4706</v>
       </c>
     </row>
     <row r="20" ht="11" customHeight="true" outlineLevel="3">
@@ -1672,7 +1717,7 @@
         <v>19</v>
       </c>
       <c r="C20" s="11" t="n">
-        <v>539</v>
+        <v>640</v>
       </c>
     </row>
     <row r="21" ht="11" customHeight="true" outlineLevel="3">
@@ -1680,7 +1725,7 @@
         <v>20</v>
       </c>
       <c r="C21" s="11" t="n">
-        <v>496</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22" ht="11" customHeight="true" outlineLevel="3">
@@ -1688,39 +1733,39 @@
         <v>21</v>
       </c>
       <c r="C22" s="18" t="n">
-        <v>2348</v>
+        <v>3545</v>
       </c>
     </row>
     <row r="23" ht="11" customHeight="true" outlineLevel="3">
       <c r="B23" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="C23" s="11" t="n">
-        <v>929</v>
+      <c r="C23" s="18" t="n">
+        <v>5474</v>
       </c>
     </row>
     <row r="24" ht="11" customHeight="true" outlineLevel="3">
       <c r="B24" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="C24" s="18" t="n">
-        <v>3425</v>
+      <c r="C24" s="11" t="n">
+        <v>230</v>
       </c>
     </row>
     <row r="25" ht="11" customHeight="true" outlineLevel="3">
       <c r="B25" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="C25" s="18" t="n">
-        <v>1456</v>
+      <c r="C25" s="11" t="n">
+        <v>313</v>
       </c>
     </row>
     <row r="26" ht="11" customHeight="true" outlineLevel="3">
       <c r="B26" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="C26" s="11" t="n">
-        <v>920</v>
+      <c r="C26" s="18" t="n">
+        <v>5647</v>
       </c>
     </row>
     <row r="27" ht="11" customHeight="true" outlineLevel="3">
@@ -1728,7 +1773,7 @@
         <v>26</v>
       </c>
       <c r="C27" s="11" t="n">
-        <v>375</v>
+        <v>40</v>
       </c>
     </row>
     <row r="28" ht="11" customHeight="true" outlineLevel="3">
@@ -1736,7 +1781,7 @@
         <v>27</v>
       </c>
       <c r="C28" s="11" t="n">
-        <v>280</v>
+        <v>227</v>
       </c>
     </row>
     <row r="29" ht="11" customHeight="true" outlineLevel="3">
@@ -1744,7 +1789,7 @@
         <v>28</v>
       </c>
       <c r="C29" s="11" t="n">
-        <v>394</v>
+        <v>248</v>
       </c>
     </row>
     <row r="30" ht="11" customHeight="true" outlineLevel="3">
@@ -1752,23 +1797,23 @@
         <v>29</v>
       </c>
       <c r="C30" s="11" t="n">
-        <v>232</v>
+        <v>783</v>
       </c>
     </row>
     <row r="31" ht="11" customHeight="true" outlineLevel="3">
       <c r="B31" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="C31" s="18" t="n">
-        <v>4270</v>
-      </c>
-    </row>
-    <row r="32" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B32" s="16" t="s">
+      <c r="C31" s="11" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="32" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B32" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="C32" s="12" t="n">
-        <v>61965</v>
+      <c r="C32" s="11" t="n">
+        <v>95</v>
       </c>
     </row>
     <row r="33" ht="11" customHeight="true" outlineLevel="3">
@@ -1776,39 +1821,39 @@
         <v>32</v>
       </c>
       <c r="C33" s="18" t="n">
-        <v>4252</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="34" ht="11" customHeight="true" outlineLevel="3">
       <c r="B34" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="C34" s="18" t="n">
-        <v>39962</v>
+      <c r="C34" s="11" t="n">
+        <v>76</v>
       </c>
     </row>
     <row r="35" ht="11" customHeight="true" outlineLevel="3">
       <c r="B35" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="C35" s="18" t="n">
-        <v>4794</v>
+      <c r="C35" s="11" t="n">
+        <v>48</v>
       </c>
     </row>
     <row r="36" ht="11" customHeight="true" outlineLevel="3">
       <c r="B36" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="C36" s="18" t="n">
-        <v>1201</v>
-      </c>
-    </row>
-    <row r="37" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B37" s="17" t="s">
+      <c r="C36" s="11" t="n">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="37" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B37" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="C37" s="11" t="n">
-        <v>608</v>
+      <c r="C37" s="12" t="n">
+        <v>73485</v>
       </c>
     </row>
     <row r="38" ht="11" customHeight="true" outlineLevel="3">
@@ -1816,23 +1861,23 @@
         <v>37</v>
       </c>
       <c r="C38" s="18" t="n">
-        <v>6504</v>
+        <v>4395</v>
       </c>
     </row>
     <row r="39" ht="11" customHeight="true" outlineLevel="3">
       <c r="B39" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="C39" s="11" t="n">
-        <v>938</v>
+      <c r="C39" s="18" t="n">
+        <v>54325</v>
       </c>
     </row>
     <row r="40" ht="11" customHeight="true" outlineLevel="3">
       <c r="B40" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="C40" s="11" t="n">
-        <v>901</v>
+      <c r="C40" s="18" t="n">
+        <v>4794</v>
       </c>
     </row>
     <row r="41" ht="11" customHeight="true" outlineLevel="3">
@@ -1840,7 +1885,7 @@
         <v>40</v>
       </c>
       <c r="C41" s="11" t="n">
-        <v>120</v>
+        <v>482</v>
       </c>
     </row>
     <row r="42" ht="11" customHeight="true" outlineLevel="3">
@@ -1848,23 +1893,23 @@
         <v>41</v>
       </c>
       <c r="C42" s="11" t="n">
-        <v>811</v>
+        <v>24</v>
       </c>
     </row>
     <row r="43" ht="11" customHeight="true" outlineLevel="3">
       <c r="B43" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="C43" s="11" t="n">
-        <v>919</v>
-      </c>
-    </row>
-    <row r="44" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C43" s="18" t="n">
+        <v>4208</v>
+      </c>
+    </row>
+    <row r="44" ht="11" customHeight="true" outlineLevel="3">
       <c r="B44" s="17" t="s">
         <v>43</v>
       </c>
       <c r="C44" s="11" t="n">
-        <v>80</v>
+        <v>272</v>
       </c>
     </row>
     <row r="45" ht="11" customHeight="true" outlineLevel="3">
@@ -1872,31 +1917,31 @@
         <v>44</v>
       </c>
       <c r="C45" s="11" t="n">
-        <v>741</v>
-      </c>
-    </row>
-    <row r="46" ht="22" customHeight="true" outlineLevel="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="46" ht="11" customHeight="true" outlineLevel="3">
       <c r="B46" s="17" t="s">
         <v>45</v>
       </c>
       <c r="C46" s="11" t="n">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="47" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B47" s="16" t="s">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="47" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B47" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="C47" s="12" t="n">
-        <v>20914</v>
-      </c>
-    </row>
-    <row r="48" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C47" s="18" t="n">
+        <v>1338</v>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="true" outlineLevel="3">
       <c r="B48" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="C48" s="18" t="n">
-        <v>1233</v>
+      <c r="C48" s="11" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="49" ht="11" customHeight="true" outlineLevel="3">
@@ -1904,7 +1949,7 @@
         <v>48</v>
       </c>
       <c r="C49" s="11" t="n">
-        <v>532</v>
+        <v>140</v>
       </c>
     </row>
     <row r="50" ht="11" customHeight="true" outlineLevel="3">
@@ -1912,7 +1957,7 @@
         <v>49</v>
       </c>
       <c r="C50" s="11" t="n">
-        <v>658</v>
+        <v>10</v>
       </c>
     </row>
     <row r="51" ht="11" customHeight="true" outlineLevel="3">
@@ -1920,31 +1965,31 @@
         <v>50</v>
       </c>
       <c r="C51" s="18" t="n">
-        <v>1233</v>
-      </c>
-    </row>
-    <row r="52" ht="11" customHeight="true" outlineLevel="3">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="true" outlineLevel="3">
       <c r="B52" s="17" t="s">
         <v>51</v>
       </c>
       <c r="C52" s="11" t="n">
-        <v>924</v>
-      </c>
-    </row>
-    <row r="53" ht="11" customHeight="true" outlineLevel="3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="53" ht="22" customHeight="true" outlineLevel="3">
       <c r="B53" s="17" t="s">
         <v>52</v>
       </c>
       <c r="C53" s="11" t="n">
-        <v>723</v>
+        <v>100</v>
       </c>
     </row>
     <row r="54" ht="11" customHeight="true" outlineLevel="3">
       <c r="B54" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="C54" s="18" t="n">
-        <v>1439</v>
+      <c r="C54" s="11" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="55" ht="11" customHeight="true" outlineLevel="3">
@@ -1952,31 +1997,31 @@
         <v>54</v>
       </c>
       <c r="C55" s="11" t="n">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="56" ht="11" customHeight="true" outlineLevel="3">
+        <v>987</v>
+      </c>
+    </row>
+    <row r="56" ht="22" customHeight="true" outlineLevel="3">
       <c r="B56" s="17" t="s">
         <v>55</v>
       </c>
       <c r="C56" s="11" t="n">
-        <v>845</v>
-      </c>
-    </row>
-    <row r="57" ht="11" customHeight="true" outlineLevel="3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="57" ht="22" customHeight="true" outlineLevel="3">
       <c r="B57" s="17" t="s">
         <v>56</v>
       </c>
       <c r="C57" s="11" t="n">
-        <v>775</v>
-      </c>
-    </row>
-    <row r="58" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B58" s="17" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="58" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B58" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="C58" s="18" t="n">
-        <v>1333</v>
+      <c r="C58" s="12" t="n">
+        <v>13919</v>
       </c>
     </row>
     <row r="59" ht="11" customHeight="true" outlineLevel="3">
@@ -1984,7 +2029,7 @@
         <v>58</v>
       </c>
       <c r="C59" s="11" t="n">
-        <v>785</v>
+        <v>229</v>
       </c>
     </row>
     <row r="60" ht="11" customHeight="true" outlineLevel="3">
@@ -1992,7 +2037,7 @@
         <v>59</v>
       </c>
       <c r="C60" s="11" t="n">
-        <v>795</v>
+        <v>136</v>
       </c>
     </row>
     <row r="61" ht="11" customHeight="true" outlineLevel="3">
@@ -2000,15 +2045,15 @@
         <v>60</v>
       </c>
       <c r="C61" s="11" t="n">
-        <v>361</v>
+        <v>337</v>
       </c>
     </row>
     <row r="62" ht="11" customHeight="true" outlineLevel="3">
       <c r="B62" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="C62" s="18" t="n">
-        <v>1015</v>
+      <c r="C62" s="11" t="n">
+        <v>329</v>
       </c>
     </row>
     <row r="63" ht="11" customHeight="true" outlineLevel="3">
@@ -2016,15 +2061,15 @@
         <v>62</v>
       </c>
       <c r="C63" s="11" t="n">
-        <v>800</v>
+        <v>893</v>
       </c>
     </row>
     <row r="64" ht="11" customHeight="true" outlineLevel="3">
       <c r="B64" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="C64" s="18" t="n">
-        <v>1221</v>
+      <c r="C64" s="11" t="n">
+        <v>655</v>
       </c>
     </row>
     <row r="65" ht="11" customHeight="true" outlineLevel="3">
@@ -2032,7 +2077,7 @@
         <v>64</v>
       </c>
       <c r="C65" s="11" t="n">
-        <v>337</v>
+        <v>493</v>
       </c>
     </row>
     <row r="66" ht="11" customHeight="true" outlineLevel="3">
@@ -2040,7 +2085,7 @@
         <v>65</v>
       </c>
       <c r="C66" s="11" t="n">
-        <v>149</v>
+        <v>260</v>
       </c>
     </row>
     <row r="67" ht="11" customHeight="true" outlineLevel="3">
@@ -2048,15 +2093,15 @@
         <v>66</v>
       </c>
       <c r="C67" s="11" t="n">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="68" ht="22" customHeight="true" outlineLevel="3">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="68" ht="11" customHeight="true" outlineLevel="3">
       <c r="B68" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="C68" s="18" t="n">
-        <v>1000</v>
+      <c r="C68" s="11" t="n">
+        <v>643</v>
       </c>
     </row>
     <row r="69" ht="11" customHeight="true" outlineLevel="3">
@@ -2064,15 +2109,15 @@
         <v>68</v>
       </c>
       <c r="C69" s="11" t="n">
-        <v>319</v>
+        <v>678</v>
       </c>
     </row>
     <row r="70" ht="11" customHeight="true" outlineLevel="3">
       <c r="B70" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="C70" s="18" t="n">
-        <v>1172</v>
+      <c r="C70" s="11" t="n">
+        <v>755</v>
       </c>
     </row>
     <row r="71" ht="11" customHeight="true" outlineLevel="3">
@@ -2080,7 +2125,7 @@
         <v>70</v>
       </c>
       <c r="C71" s="11" t="n">
-        <v>737</v>
+        <v>111</v>
       </c>
     </row>
     <row r="72" ht="11" customHeight="true" outlineLevel="3">
@@ -2088,7 +2133,7 @@
         <v>71</v>
       </c>
       <c r="C72" s="11" t="n">
-        <v>557</v>
+        <v>565</v>
       </c>
     </row>
     <row r="73" ht="11" customHeight="true" outlineLevel="3">
@@ -2096,7 +2141,7 @@
         <v>72</v>
       </c>
       <c r="C73" s="11" t="n">
-        <v>233</v>
+        <v>630</v>
       </c>
     </row>
     <row r="74" ht="11" customHeight="true" outlineLevel="3">
@@ -2104,15 +2149,15 @@
         <v>73</v>
       </c>
       <c r="C74" s="11" t="n">
-        <v>848</v>
-      </c>
-    </row>
-    <row r="75" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B75" s="16" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="75" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B75" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="C75" s="12" t="n">
-        <v>48271</v>
+      <c r="C75" s="11" t="n">
+        <v>99</v>
       </c>
     </row>
     <row r="76" ht="11" customHeight="true" outlineLevel="3">
@@ -2120,31 +2165,31 @@
         <v>75</v>
       </c>
       <c r="C76" s="11" t="n">
-        <v>410</v>
+        <v>37</v>
       </c>
     </row>
     <row r="77" ht="11" customHeight="true" outlineLevel="3">
       <c r="B77" s="17" t="s">
         <v>76</v>
       </c>
-      <c r="C77" s="18" t="n">
-        <v>1518</v>
+      <c r="C77" s="11" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="78" ht="11" customHeight="true" outlineLevel="3">
       <c r="B78" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="C78" s="18" t="n">
-        <v>1805</v>
-      </c>
-    </row>
-    <row r="79" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C78" s="11" t="n">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="79" ht="22" customHeight="true" outlineLevel="3">
       <c r="B79" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="C79" s="18" t="n">
-        <v>1972</v>
+      <c r="C79" s="11" t="n">
+        <v>582</v>
       </c>
     </row>
     <row r="80" ht="11" customHeight="true" outlineLevel="3">
@@ -2152,55 +2197,55 @@
         <v>79</v>
       </c>
       <c r="C80" s="18" t="n">
-        <v>8091</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="81" ht="11" customHeight="true" outlineLevel="3">
       <c r="B81" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="C81" s="18" t="n">
-        <v>1441</v>
+      <c r="C81" s="11" t="n">
+        <v>564</v>
       </c>
     </row>
     <row r="82" ht="11" customHeight="true" outlineLevel="3">
       <c r="B82" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="C82" s="18" t="n">
-        <v>1744</v>
+      <c r="C82" s="11" t="n">
+        <v>681</v>
       </c>
     </row>
     <row r="83" ht="11" customHeight="true" outlineLevel="3">
       <c r="B83" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="C83" s="18" t="n">
-        <v>2889</v>
+      <c r="C83" s="11" t="n">
+        <v>437</v>
       </c>
     </row>
     <row r="84" ht="11" customHeight="true" outlineLevel="3">
       <c r="B84" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="C84" s="11" t="n">
-        <v>617</v>
+      <c r="C84" s="18" t="n">
+        <v>1403</v>
       </c>
     </row>
     <row r="85" ht="11" customHeight="true" outlineLevel="3">
       <c r="B85" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="C85" s="18" t="n">
-        <v>6400</v>
-      </c>
-    </row>
-    <row r="86" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B86" s="17" t="s">
+      <c r="C85" s="11" t="n">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="86" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B86" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="C86" s="18" t="n">
-        <v>1783</v>
+      <c r="C86" s="12" t="n">
+        <v>42405</v>
       </c>
     </row>
     <row r="87" ht="11" customHeight="true" outlineLevel="3">
@@ -2208,79 +2253,79 @@
         <v>86</v>
       </c>
       <c r="C87" s="18" t="n">
-        <v>12613</v>
+        <v>1980</v>
       </c>
     </row>
     <row r="88" ht="11" customHeight="true" outlineLevel="3">
       <c r="B88" s="17" t="s">
         <v>87</v>
       </c>
-      <c r="C88" s="11" t="n">
-        <v>10</v>
+      <c r="C88" s="18" t="n">
+        <v>1323</v>
       </c>
     </row>
     <row r="89" ht="11" customHeight="true" outlineLevel="3">
       <c r="B89" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="C89" s="18" t="n">
-        <v>4503</v>
+      <c r="C89" s="11" t="n">
+        <v>419</v>
       </c>
     </row>
     <row r="90" ht="11" customHeight="true" outlineLevel="3">
       <c r="B90" s="17" t="s">
         <v>89</v>
       </c>
-      <c r="C90" s="11" t="n">
-        <v>959</v>
+      <c r="C90" s="18" t="n">
+        <v>2011</v>
       </c>
     </row>
     <row r="91" ht="11" customHeight="true" outlineLevel="3">
       <c r="B91" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="C91" s="11" t="n">
-        <v>607</v>
+      <c r="C91" s="18" t="n">
+        <v>8928</v>
       </c>
     </row>
     <row r="92" ht="11" customHeight="true" outlineLevel="3">
       <c r="B92" s="17" t="s">
         <v>91</v>
       </c>
-      <c r="C92" s="11" t="n">
-        <v>838</v>
+      <c r="C92" s="18" t="n">
+        <v>1211</v>
       </c>
     </row>
     <row r="93" ht="11" customHeight="true" outlineLevel="3">
       <c r="B93" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="C93" s="11" t="n">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="94" ht="11" customHeight="true" outlineLevel="1">
-      <c r="B94" s="13" t="s">
+      <c r="C93" s="18" t="n">
+        <v>3388</v>
+      </c>
+    </row>
+    <row r="94" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B94" s="17" t="s">
         <v>93</v>
       </c>
-      <c r="C94" s="12" t="n">
-        <v>517958</v>
-      </c>
-    </row>
-    <row r="95" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B95" s="16" t="s">
+      <c r="C94" s="18" t="n">
+        <v>1776</v>
+      </c>
+    </row>
+    <row r="95" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B95" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="C95" s="12" t="n">
-        <v>148563</v>
-      </c>
-    </row>
-    <row r="96" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C95" s="18" t="n">
+        <v>1434</v>
+      </c>
+    </row>
+    <row r="96" ht="11" customHeight="true" outlineLevel="3">
       <c r="B96" s="17" t="s">
         <v>95</v>
       </c>
       <c r="C96" s="18" t="n">
-        <v>12593</v>
+        <v>4197</v>
       </c>
     </row>
     <row r="97" ht="11" customHeight="true" outlineLevel="3">
@@ -2288,7 +2333,7 @@
         <v>96</v>
       </c>
       <c r="C97" s="18" t="n">
-        <v>20589</v>
+        <v>1687</v>
       </c>
     </row>
     <row r="98" ht="11" customHeight="true" outlineLevel="3">
@@ -2296,55 +2341,55 @@
         <v>97</v>
       </c>
       <c r="C98" s="18" t="n">
-        <v>5730</v>
-      </c>
-    </row>
-    <row r="99" ht="22" customHeight="true" outlineLevel="3">
+        <v>10418</v>
+      </c>
+    </row>
+    <row r="99" ht="11" customHeight="true" outlineLevel="3">
       <c r="B99" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="C99" s="11" t="n">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="100" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C99" s="18" t="n">
+        <v>2071</v>
+      </c>
+    </row>
+    <row r="100" ht="11" customHeight="true" outlineLevel="3">
       <c r="B100" s="17" t="s">
         <v>99</v>
       </c>
-      <c r="C100" s="18" t="n">
-        <v>14427</v>
-      </c>
-    </row>
-    <row r="101" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C100" s="11" t="n">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="101" ht="11" customHeight="true" outlineLevel="3">
       <c r="B101" s="17" t="s">
         <v>100</v>
       </c>
-      <c r="C101" s="18" t="n">
-        <v>3530</v>
-      </c>
-    </row>
-    <row r="102" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C101" s="11" t="n">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="102" ht="11" customHeight="true" outlineLevel="3">
       <c r="B102" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="C102" s="18" t="n">
-        <v>15042</v>
-      </c>
-    </row>
-    <row r="103" ht="22" customHeight="true" outlineLevel="3">
-      <c r="B103" s="17" t="s">
+      <c r="C102" s="11" t="n">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="103" ht="11" customHeight="true" outlineLevel="1">
+      <c r="B103" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="C103" s="18" t="n">
-        <v>7421</v>
-      </c>
-    </row>
-    <row r="104" ht="22" customHeight="true" outlineLevel="3">
-      <c r="B104" s="17" t="s">
+      <c r="C103" s="12" t="n">
+        <v>417580</v>
+      </c>
+    </row>
+    <row r="104" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B104" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="C104" s="18" t="n">
-        <v>12043</v>
+      <c r="C104" s="12" t="n">
+        <v>78296</v>
       </c>
     </row>
     <row r="105" ht="22" customHeight="true" outlineLevel="3">
@@ -2352,7 +2397,7 @@
         <v>104</v>
       </c>
       <c r="C105" s="18" t="n">
-        <v>22937</v>
+        <v>3592</v>
       </c>
     </row>
     <row r="106" ht="22" customHeight="true" outlineLevel="3">
@@ -2360,127 +2405,127 @@
         <v>105</v>
       </c>
       <c r="C106" s="18" t="n">
-        <v>3410</v>
-      </c>
-    </row>
-    <row r="107" ht="22" customHeight="true" outlineLevel="3">
+        <v>3420</v>
+      </c>
+    </row>
+    <row r="107" ht="11" customHeight="true" outlineLevel="3">
       <c r="B107" s="17" t="s">
         <v>106</v>
       </c>
       <c r="C107" s="18" t="n">
-        <v>30550</v>
-      </c>
-    </row>
-    <row r="108" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B108" s="16" t="s">
+        <v>11318</v>
+      </c>
+    </row>
+    <row r="108" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B108" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="C108" s="12" t="n">
-        <v>5081</v>
+      <c r="C108" s="18" t="n">
+        <v>2700</v>
       </c>
     </row>
     <row r="109" ht="11" customHeight="true" outlineLevel="3">
       <c r="B109" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="C109" s="11" t="n">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="110" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C109" s="18" t="n">
+        <v>3081</v>
+      </c>
+    </row>
+    <row r="110" ht="22" customHeight="true" outlineLevel="3">
       <c r="B110" s="17" t="s">
         <v>109</v>
       </c>
       <c r="C110" s="11" t="n">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="111" ht="11" customHeight="true" outlineLevel="3">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="111" ht="22" customHeight="true" outlineLevel="3">
       <c r="B111" s="17" t="s">
         <v>110</v>
       </c>
-      <c r="C111" s="11" t="n">
-        <v>586</v>
-      </c>
-    </row>
-    <row r="112" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C111" s="18" t="n">
+        <v>5577</v>
+      </c>
+    </row>
+    <row r="112" ht="22" customHeight="true" outlineLevel="3">
       <c r="B112" s="17" t="s">
         <v>111</v>
       </c>
       <c r="C112" s="18" t="n">
-        <v>1239</v>
-      </c>
-    </row>
-    <row r="113" ht="11" customHeight="true" outlineLevel="3">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="113" ht="22" customHeight="true" outlineLevel="3">
       <c r="B113" s="17" t="s">
         <v>112</v>
       </c>
       <c r="C113" s="18" t="n">
-        <v>1082</v>
-      </c>
-    </row>
-    <row r="114" ht="11" customHeight="true" outlineLevel="3">
+        <v>2891</v>
+      </c>
+    </row>
+    <row r="114" ht="22" customHeight="true" outlineLevel="3">
       <c r="B114" s="17" t="s">
         <v>113</v>
       </c>
-      <c r="C114" s="11" t="n">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="115" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C114" s="18" t="n">
+        <v>2700</v>
+      </c>
+    </row>
+    <row r="115" ht="22" customHeight="true" outlineLevel="3">
       <c r="B115" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="C115" s="11" t="n">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="116" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C115" s="18" t="n">
+        <v>6977</v>
+      </c>
+    </row>
+    <row r="116" ht="22" customHeight="true" outlineLevel="3">
       <c r="B116" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="C116" s="11" t="n">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="117" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C116" s="18" t="n">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="117" ht="22" customHeight="true" outlineLevel="3">
       <c r="B117" s="17" t="s">
         <v>116</v>
       </c>
-      <c r="C117" s="11" t="n">
-        <v>617</v>
-      </c>
-    </row>
-    <row r="118" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B118" s="16" t="s">
+      <c r="C117" s="18" t="n">
+        <v>1269</v>
+      </c>
+    </row>
+    <row r="118" ht="22" customHeight="true" outlineLevel="3">
+      <c r="B118" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="C118" s="12" t="n">
-        <v>81395</v>
-      </c>
-    </row>
-    <row r="119" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C118" s="18" t="n">
+        <v>20980</v>
+      </c>
+    </row>
+    <row r="119" ht="22" customHeight="true" outlineLevel="3">
       <c r="B119" s="17" t="s">
         <v>118</v>
       </c>
-      <c r="C119" s="11" t="n">
-        <v>460</v>
-      </c>
-    </row>
-    <row r="120" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B120" s="17" t="s">
+      <c r="C119" s="18" t="n">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="120" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B120" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="C120" s="11" t="n">
-        <v>199</v>
+      <c r="C120" s="12" t="n">
+        <v>6653</v>
       </c>
     </row>
     <row r="121" ht="11" customHeight="true" outlineLevel="3">
       <c r="B121" s="17" t="s">
         <v>120</v>
       </c>
-      <c r="C121" s="11" t="n">
-        <v>553</v>
+      <c r="C121" s="18" t="n">
+        <v>1133</v>
       </c>
     </row>
     <row r="122" ht="11" customHeight="true" outlineLevel="3">
@@ -2488,15 +2533,15 @@
         <v>121</v>
       </c>
       <c r="C122" s="11" t="n">
-        <v>735</v>
+        <v>490</v>
       </c>
     </row>
     <row r="123" ht="11" customHeight="true" outlineLevel="3">
       <c r="B123" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="C123" s="18" t="n">
-        <v>1718</v>
+      <c r="C123" s="11" t="n">
+        <v>687</v>
       </c>
     </row>
     <row r="124" ht="11" customHeight="true" outlineLevel="3">
@@ -2504,15 +2549,15 @@
         <v>123</v>
       </c>
       <c r="C124" s="18" t="n">
-        <v>23734</v>
+        <v>1726</v>
       </c>
     </row>
     <row r="125" ht="11" customHeight="true" outlineLevel="3">
       <c r="B125" s="17" t="s">
         <v>124</v>
       </c>
-      <c r="C125" s="18" t="n">
-        <v>27230</v>
+      <c r="C125" s="11" t="n">
+        <v>459</v>
       </c>
     </row>
     <row r="126" ht="11" customHeight="true" outlineLevel="3">
@@ -2520,7 +2565,7 @@
         <v>125</v>
       </c>
       <c r="C126" s="18" t="n">
-        <v>11753</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="127" ht="11" customHeight="true" outlineLevel="3">
@@ -2528,7 +2573,7 @@
         <v>126</v>
       </c>
       <c r="C127" s="11" t="n">
-        <v>439</v>
+        <v>272</v>
       </c>
     </row>
     <row r="128" ht="11" customHeight="true" outlineLevel="3">
@@ -2536,7 +2581,7 @@
         <v>127</v>
       </c>
       <c r="C128" s="11" t="n">
-        <v>105</v>
+        <v>410</v>
       </c>
     </row>
     <row r="129" ht="11" customHeight="true" outlineLevel="3">
@@ -2544,15 +2589,15 @@
         <v>128</v>
       </c>
       <c r="C129" s="11" t="n">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="130" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B130" s="17" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="130" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B130" s="16" t="s">
         <v>129</v>
       </c>
-      <c r="C130" s="11" t="n">
-        <v>659</v>
+      <c r="C130" s="12" t="n">
+        <v>107219</v>
       </c>
     </row>
     <row r="131" ht="11" customHeight="true" outlineLevel="3">
@@ -2560,7 +2605,7 @@
         <v>130</v>
       </c>
       <c r="C131" s="11" t="n">
-        <v>231</v>
+        <v>301</v>
       </c>
     </row>
     <row r="132" ht="11" customHeight="true" outlineLevel="3">
@@ -2568,15 +2613,15 @@
         <v>131</v>
       </c>
       <c r="C132" s="11" t="n">
-        <v>500</v>
+        <v>394</v>
       </c>
     </row>
     <row r="133" ht="11" customHeight="true" outlineLevel="3">
       <c r="B133" s="17" t="s">
         <v>132</v>
       </c>
-      <c r="C133" s="18" t="n">
-        <v>1284</v>
+      <c r="C133" s="11" t="n">
+        <v>578</v>
       </c>
     </row>
     <row r="134" ht="11" customHeight="true" outlineLevel="3">
@@ -2584,15 +2629,15 @@
         <v>133</v>
       </c>
       <c r="C134" s="11" t="n">
-        <v>985</v>
+        <v>545</v>
       </c>
     </row>
     <row r="135" ht="11" customHeight="true" outlineLevel="3">
       <c r="B135" s="17" t="s">
         <v>134</v>
       </c>
-      <c r="C135" s="11" t="n">
-        <v>2</v>
+      <c r="C135" s="18" t="n">
+        <v>3579</v>
       </c>
     </row>
     <row r="136" ht="11" customHeight="true" outlineLevel="3">
@@ -2600,31 +2645,31 @@
         <v>135</v>
       </c>
       <c r="C136" s="18" t="n">
-        <v>1888</v>
+        <v>22358</v>
       </c>
     </row>
     <row r="137" ht="11" customHeight="true" outlineLevel="3">
       <c r="B137" s="17" t="s">
         <v>136</v>
       </c>
-      <c r="C137" s="11" t="n">
-        <v>10</v>
+      <c r="C137" s="18" t="n">
+        <v>45757</v>
       </c>
     </row>
     <row r="138" ht="11" customHeight="true" outlineLevel="3">
       <c r="B138" s="17" t="s">
         <v>137</v>
       </c>
-      <c r="C138" s="11" t="n">
-        <v>981</v>
+      <c r="C138" s="18" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="139" ht="11" customHeight="true" outlineLevel="3">
       <c r="B139" s="17" t="s">
         <v>138</v>
       </c>
-      <c r="C139" s="11" t="n">
-        <v>254</v>
+      <c r="C139" s="18" t="n">
+        <v>21079</v>
       </c>
     </row>
     <row r="140" ht="11" customHeight="true" outlineLevel="3">
@@ -2632,7 +2677,7 @@
         <v>139</v>
       </c>
       <c r="C140" s="11" t="n">
-        <v>374</v>
+        <v>178</v>
       </c>
     </row>
     <row r="141" ht="11" customHeight="true" outlineLevel="3">
@@ -2640,55 +2685,55 @@
         <v>140</v>
       </c>
       <c r="C141" s="11" t="n">
-        <v>762</v>
+        <v>325</v>
       </c>
     </row>
     <row r="142" ht="11" customHeight="true" outlineLevel="3">
       <c r="B142" s="17" t="s">
         <v>141</v>
       </c>
-      <c r="C142" s="18" t="n">
-        <v>1876</v>
+      <c r="C142" s="11" t="n">
+        <v>219</v>
       </c>
     </row>
     <row r="143" ht="11" customHeight="true" outlineLevel="3">
       <c r="B143" s="17" t="s">
         <v>142</v>
       </c>
-      <c r="C143" s="18" t="n">
-        <v>1081</v>
+      <c r="C143" s="11" t="n">
+        <v>863</v>
       </c>
     </row>
     <row r="144" ht="11" customHeight="true" outlineLevel="3">
       <c r="B144" s="17" t="s">
         <v>143</v>
       </c>
-      <c r="C144" s="18" t="n">
-        <v>2085</v>
+      <c r="C144" s="11" t="n">
+        <v>146</v>
       </c>
     </row>
     <row r="145" ht="11" customHeight="true" outlineLevel="3">
       <c r="B145" s="17" t="s">
         <v>144</v>
       </c>
-      <c r="C145" s="18" t="n">
-        <v>1262</v>
-      </c>
-    </row>
-    <row r="146" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B146" s="16" t="s">
+      <c r="C145" s="11" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="146" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B146" s="17" t="s">
         <v>145</v>
       </c>
-      <c r="C146" s="12" t="n">
-        <v>98835</v>
+      <c r="C146" s="11" t="n">
+        <v>533</v>
       </c>
     </row>
     <row r="147" ht="11" customHeight="true" outlineLevel="3">
       <c r="B147" s="17" t="s">
         <v>146</v>
       </c>
-      <c r="C147" s="18" t="n">
-        <v>1269</v>
+      <c r="C147" s="11" t="n">
+        <v>319</v>
       </c>
     </row>
     <row r="148" ht="11" customHeight="true" outlineLevel="3">
@@ -2696,7 +2741,7 @@
         <v>147</v>
       </c>
       <c r="C148" s="11" t="n">
-        <v>402</v>
+        <v>1</v>
       </c>
     </row>
     <row r="149" ht="11" customHeight="true" outlineLevel="3">
@@ -2704,7 +2749,7 @@
         <v>148</v>
       </c>
       <c r="C149" s="11" t="n">
-        <v>317</v>
+        <v>742</v>
       </c>
     </row>
     <row r="150" ht="11" customHeight="true" outlineLevel="3">
@@ -2712,7 +2757,7 @@
         <v>149</v>
       </c>
       <c r="C150" s="11" t="n">
-        <v>344</v>
+        <v>9</v>
       </c>
     </row>
     <row r="151" ht="11" customHeight="true" outlineLevel="3">
@@ -2720,15 +2765,15 @@
         <v>150</v>
       </c>
       <c r="C151" s="18" t="n">
-        <v>1793</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="152" ht="11" customHeight="true" outlineLevel="3">
       <c r="B152" s="17" t="s">
         <v>151</v>
       </c>
-      <c r="C152" s="18" t="n">
-        <v>1180</v>
+      <c r="C152" s="11" t="n">
+        <v>165</v>
       </c>
     </row>
     <row r="153" ht="11" customHeight="true" outlineLevel="3">
@@ -2736,63 +2781,63 @@
         <v>152</v>
       </c>
       <c r="C153" s="11" t="n">
-        <v>250</v>
+        <v>449</v>
       </c>
     </row>
     <row r="154" ht="11" customHeight="true" outlineLevel="3">
       <c r="B154" s="17" t="s">
         <v>153</v>
       </c>
-      <c r="C154" s="11" t="n">
-        <v>43</v>
+      <c r="C154" s="18" t="n">
+        <v>1019</v>
       </c>
     </row>
     <row r="155" ht="11" customHeight="true" outlineLevel="3">
       <c r="B155" s="17" t="s">
         <v>154</v>
       </c>
-      <c r="C155" s="11" t="n">
-        <v>224</v>
+      <c r="C155" s="18" t="n">
+        <v>1416</v>
       </c>
     </row>
     <row r="156" ht="11" customHeight="true" outlineLevel="3">
       <c r="B156" s="17" t="s">
         <v>155</v>
       </c>
-      <c r="C156" s="11" t="n">
-        <v>19</v>
+      <c r="C156" s="18" t="n">
+        <v>1392</v>
       </c>
     </row>
     <row r="157" ht="11" customHeight="true" outlineLevel="3">
       <c r="B157" s="17" t="s">
         <v>156</v>
       </c>
-      <c r="C157" s="18" t="n">
-        <v>3332</v>
+      <c r="C157" s="11" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="158" ht="11" customHeight="true" outlineLevel="3">
       <c r="B158" s="17" t="s">
         <v>157</v>
       </c>
-      <c r="C158" s="11" t="n">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="159" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B159" s="17" t="s">
+      <c r="C158" s="18" t="n">
+        <v>1395</v>
+      </c>
+    </row>
+    <row r="159" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B159" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="C159" s="18" t="n">
-        <v>2722</v>
+      <c r="C159" s="12" t="n">
+        <v>73708</v>
       </c>
     </row>
     <row r="160" ht="11" customHeight="true" outlineLevel="3">
       <c r="B160" s="17" t="s">
         <v>159</v>
       </c>
-      <c r="C160" s="11" t="n">
-        <v>149</v>
+      <c r="C160" s="18" t="n">
+        <v>1328</v>
       </c>
     </row>
     <row r="161" ht="11" customHeight="true" outlineLevel="3">
@@ -2800,15 +2845,15 @@
         <v>160</v>
       </c>
       <c r="C161" s="11" t="n">
-        <v>636</v>
+        <v>245</v>
       </c>
     </row>
     <row r="162" ht="11" customHeight="true" outlineLevel="3">
       <c r="B162" s="17" t="s">
         <v>161</v>
       </c>
-      <c r="C162" s="18" t="n">
-        <v>5018</v>
+      <c r="C162" s="11" t="n">
+        <v>172</v>
       </c>
     </row>
     <row r="163" ht="11" customHeight="true" outlineLevel="3">
@@ -2816,7 +2861,7 @@
         <v>162</v>
       </c>
       <c r="C163" s="11" t="n">
-        <v>403</v>
+        <v>155</v>
       </c>
     </row>
     <row r="164" ht="11" customHeight="true" outlineLevel="3">
@@ -2824,7 +2869,7 @@
         <v>163</v>
       </c>
       <c r="C164" s="18" t="n">
-        <v>1463</v>
+        <v>2791</v>
       </c>
     </row>
     <row r="165" ht="11" customHeight="true" outlineLevel="3">
@@ -2832,23 +2877,23 @@
         <v>164</v>
       </c>
       <c r="C165" s="11" t="n">
-        <v>244</v>
+        <v>991</v>
       </c>
     </row>
     <row r="166" ht="11" customHeight="true" outlineLevel="3">
       <c r="B166" s="17" t="s">
         <v>165</v>
       </c>
-      <c r="C166" s="18" t="n">
-        <v>7023</v>
+      <c r="C166" s="11" t="n">
+        <v>269</v>
       </c>
     </row>
     <row r="167" ht="11" customHeight="true" outlineLevel="3">
       <c r="B167" s="17" t="s">
         <v>166</v>
       </c>
-      <c r="C167" s="18" t="n">
-        <v>1303</v>
+      <c r="C167" s="11" t="n">
+        <v>255</v>
       </c>
     </row>
     <row r="168" ht="11" customHeight="true" outlineLevel="3">
@@ -2856,7 +2901,7 @@
         <v>167</v>
       </c>
       <c r="C168" s="11" t="n">
-        <v>18</v>
+        <v>488</v>
       </c>
     </row>
     <row r="169" ht="11" customHeight="true" outlineLevel="3">
@@ -2864,39 +2909,39 @@
         <v>168</v>
       </c>
       <c r="C169" s="11" t="n">
-        <v>978</v>
+        <v>19</v>
       </c>
     </row>
     <row r="170" ht="11" customHeight="true" outlineLevel="3">
       <c r="B170" s="17" t="s">
         <v>169</v>
       </c>
-      <c r="C170" s="11" t="n">
-        <v>437</v>
+      <c r="C170" s="18" t="n">
+        <v>3892</v>
       </c>
     </row>
     <row r="171" ht="11" customHeight="true" outlineLevel="3">
       <c r="B171" s="17" t="s">
         <v>170</v>
       </c>
-      <c r="C171" s="18" t="n">
-        <v>2114</v>
+      <c r="C171" s="11" t="n">
+        <v>505</v>
       </c>
     </row>
     <row r="172" ht="11" customHeight="true" outlineLevel="3">
       <c r="B172" s="17" t="s">
         <v>171</v>
       </c>
-      <c r="C172" s="18" t="n">
-        <v>2653</v>
+      <c r="C172" s="11" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="173" ht="11" customHeight="true" outlineLevel="3">
       <c r="B173" s="17" t="s">
         <v>172</v>
       </c>
-      <c r="C173" s="18" t="n">
-        <v>1094</v>
+      <c r="C173" s="11" t="n">
+        <v>232</v>
       </c>
     </row>
     <row r="174" ht="11" customHeight="true" outlineLevel="3">
@@ -2904,15 +2949,15 @@
         <v>173</v>
       </c>
       <c r="C174" s="11" t="n">
-        <v>173</v>
+        <v>289</v>
       </c>
     </row>
     <row r="175" ht="11" customHeight="true" outlineLevel="3">
       <c r="B175" s="17" t="s">
         <v>174</v>
       </c>
-      <c r="C175" s="11" t="n">
-        <v>135</v>
+      <c r="C175" s="18" t="n">
+        <v>1640</v>
       </c>
     </row>
     <row r="176" ht="11" customHeight="true" outlineLevel="3">
@@ -2920,7 +2965,7 @@
         <v>175</v>
       </c>
       <c r="C176" s="11" t="n">
-        <v>215</v>
+        <v>259</v>
       </c>
     </row>
     <row r="177" ht="11" customHeight="true" outlineLevel="3">
@@ -2928,31 +2973,31 @@
         <v>176</v>
       </c>
       <c r="C177" s="11" t="n">
-        <v>308</v>
+        <v>685</v>
       </c>
     </row>
     <row r="178" ht="11" customHeight="true" outlineLevel="3">
       <c r="B178" s="17" t="s">
         <v>177</v>
       </c>
-      <c r="C178" s="11" t="n">
-        <v>11</v>
+      <c r="C178" s="18" t="n">
+        <v>3354</v>
       </c>
     </row>
     <row r="179" ht="11" customHeight="true" outlineLevel="3">
       <c r="B179" s="17" t="s">
         <v>178</v>
       </c>
-      <c r="C179" s="18" t="n">
-        <v>1543</v>
-      </c>
-    </row>
-    <row r="180" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C179" s="11" t="n">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="180" ht="11" customHeight="true" outlineLevel="3">
       <c r="B180" s="17" t="s">
         <v>179</v>
       </c>
-      <c r="C180" s="18" t="n">
-        <v>1184</v>
+      <c r="C180" s="11" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="181" ht="11" customHeight="true" outlineLevel="3">
@@ -2960,31 +3005,31 @@
         <v>180</v>
       </c>
       <c r="C181" s="11" t="n">
-        <v>454</v>
+        <v>906</v>
       </c>
     </row>
     <row r="182" ht="11" customHeight="true" outlineLevel="3">
       <c r="B182" s="17" t="s">
         <v>181</v>
       </c>
-      <c r="C182" s="11" t="n">
-        <v>119</v>
+      <c r="C182" s="18" t="n">
+        <v>1026</v>
       </c>
     </row>
     <row r="183" ht="11" customHeight="true" outlineLevel="3">
       <c r="B183" s="17" t="s">
         <v>182</v>
       </c>
-      <c r="C183" s="11" t="n">
-        <v>333</v>
+      <c r="C183" s="18" t="n">
+        <v>2470</v>
       </c>
     </row>
     <row r="184" ht="11" customHeight="true" outlineLevel="3">
       <c r="B184" s="17" t="s">
         <v>183</v>
       </c>
-      <c r="C184" s="18" t="n">
-        <v>6812</v>
+      <c r="C184" s="11" t="n">
+        <v>104</v>
       </c>
     </row>
     <row r="185" ht="11" customHeight="true" outlineLevel="3">
@@ -2992,23 +3037,23 @@
         <v>184</v>
       </c>
       <c r="C185" s="11" t="n">
-        <v>176</v>
+        <v>254</v>
       </c>
     </row>
     <row r="186" ht="11" customHeight="true" outlineLevel="3">
       <c r="B186" s="17" t="s">
         <v>185</v>
       </c>
-      <c r="C186" s="18" t="n">
-        <v>1040</v>
+      <c r="C186" s="11" t="n">
+        <v>770</v>
       </c>
     </row>
     <row r="187" ht="11" customHeight="true" outlineLevel="3">
       <c r="B187" s="17" t="s">
         <v>186</v>
       </c>
-      <c r="C187" s="11" t="n">
-        <v>170</v>
+      <c r="C187" s="18" t="n">
+        <v>1483</v>
       </c>
     </row>
     <row r="188" ht="11" customHeight="true" outlineLevel="3">
@@ -3016,31 +3061,31 @@
         <v>187</v>
       </c>
       <c r="C188" s="11" t="n">
-        <v>372</v>
+        <v>204</v>
       </c>
     </row>
     <row r="189" ht="11" customHeight="true" outlineLevel="3">
       <c r="B189" s="17" t="s">
         <v>188</v>
       </c>
-      <c r="C189" s="18" t="n">
-        <v>3684</v>
-      </c>
-    </row>
-    <row r="190" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C189" s="11" t="n">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="190" ht="22" customHeight="true" outlineLevel="3">
       <c r="B190" s="17" t="s">
         <v>189</v>
       </c>
       <c r="C190" s="11" t="n">
-        <v>888</v>
+        <v>257</v>
       </c>
     </row>
     <row r="191" ht="11" customHeight="true" outlineLevel="3">
       <c r="B191" s="17" t="s">
         <v>190</v>
       </c>
-      <c r="C191" s="18" t="n">
-        <v>1635</v>
+      <c r="C191" s="11" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="192" ht="11" customHeight="true" outlineLevel="3">
@@ -3048,55 +3093,55 @@
         <v>191</v>
       </c>
       <c r="C192" s="11" t="n">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="193" ht="11" customHeight="true" outlineLevel="3">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="193" ht="22" customHeight="true" outlineLevel="3">
       <c r="B193" s="17" t="s">
         <v>192</v>
       </c>
       <c r="C193" s="11" t="n">
-        <v>424</v>
+        <v>322</v>
       </c>
     </row>
     <row r="194" ht="11" customHeight="true" outlineLevel="3">
       <c r="B194" s="17" t="s">
         <v>193</v>
       </c>
-      <c r="C194" s="18" t="n">
-        <v>2417</v>
-      </c>
-    </row>
-    <row r="195" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C194" s="11" t="n">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="195" ht="22" customHeight="true" outlineLevel="3">
       <c r="B195" s="17" t="s">
         <v>194</v>
       </c>
-      <c r="C195" s="18" t="n">
-        <v>1913</v>
+      <c r="C195" s="11" t="n">
+        <v>43</v>
       </c>
     </row>
     <row r="196" ht="11" customHeight="true" outlineLevel="3">
       <c r="B196" s="17" t="s">
         <v>195</v>
       </c>
-      <c r="C196" s="18" t="n">
-        <v>1058</v>
+      <c r="C196" s="11" t="n">
+        <v>413</v>
       </c>
     </row>
     <row r="197" ht="11" customHeight="true" outlineLevel="3">
       <c r="B197" s="17" t="s">
         <v>196</v>
       </c>
-      <c r="C197" s="18" t="n">
-        <v>1414</v>
+      <c r="C197" s="11" t="n">
+        <v>119</v>
       </c>
     </row>
     <row r="198" ht="11" customHeight="true" outlineLevel="3">
       <c r="B198" s="17" t="s">
         <v>197</v>
       </c>
-      <c r="C198" s="18" t="n">
-        <v>1776</v>
+      <c r="C198" s="11" t="n">
+        <v>157</v>
       </c>
     </row>
     <row r="199" ht="11" customHeight="true" outlineLevel="3">
@@ -3104,7 +3149,7 @@
         <v>198</v>
       </c>
       <c r="C199" s="18" t="n">
-        <v>19209</v>
+        <v>3712</v>
       </c>
     </row>
     <row r="200" ht="11" customHeight="true" outlineLevel="3">
@@ -3112,23 +3157,23 @@
         <v>199</v>
       </c>
       <c r="C200" s="11" t="n">
-        <v>302</v>
+        <v>7</v>
       </c>
     </row>
     <row r="201" ht="11" customHeight="true" outlineLevel="3">
       <c r="B201" s="17" t="s">
         <v>200</v>
       </c>
-      <c r="C201" s="18" t="n">
-        <v>2923</v>
+      <c r="C201" s="11" t="n">
+        <v>888</v>
       </c>
     </row>
     <row r="202" ht="11" customHeight="true" outlineLevel="3">
       <c r="B202" s="17" t="s">
         <v>201</v>
       </c>
-      <c r="C202" s="18" t="n">
-        <v>1868</v>
+      <c r="C202" s="11" t="n">
+        <v>190</v>
       </c>
     </row>
     <row r="203" ht="11" customHeight="true" outlineLevel="3">
@@ -3136,7 +3181,7 @@
         <v>202</v>
       </c>
       <c r="C203" s="18" t="n">
-        <v>1646</v>
+        <v>3460</v>
       </c>
     </row>
     <row r="204" ht="11" customHeight="true" outlineLevel="3">
@@ -3144,55 +3189,55 @@
         <v>203</v>
       </c>
       <c r="C204" s="11" t="n">
-        <v>522</v>
+        <v>274</v>
       </c>
     </row>
     <row r="205" ht="11" customHeight="true" outlineLevel="3">
       <c r="B205" s="17" t="s">
         <v>204</v>
       </c>
-      <c r="C205" s="11" t="n">
-        <v>252</v>
+      <c r="C205" s="18" t="n">
+        <v>1437</v>
       </c>
     </row>
     <row r="206" ht="11" customHeight="true" outlineLevel="3">
       <c r="B206" s="17" t="s">
         <v>205</v>
       </c>
-      <c r="C206" s="18" t="n">
-        <v>2771</v>
+      <c r="C206" s="11" t="n">
+        <v>95</v>
       </c>
     </row>
     <row r="207" ht="11" customHeight="true" outlineLevel="3">
       <c r="B207" s="17" t="s">
         <v>206</v>
       </c>
-      <c r="C207" s="18" t="n">
-        <v>4457</v>
+      <c r="C207" s="11" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="208" ht="11" customHeight="true" outlineLevel="3">
       <c r="B208" s="17" t="s">
         <v>207</v>
       </c>
-      <c r="C208" s="11" t="n">
-        <v>819</v>
+      <c r="C208" s="18" t="n">
+        <v>1963</v>
       </c>
     </row>
     <row r="209" ht="11" customHeight="true" outlineLevel="3">
       <c r="B209" s="17" t="s">
         <v>208</v>
       </c>
-      <c r="C209" s="11" t="n">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="210" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B210" s="16" t="s">
+      <c r="C209" s="18" t="n">
+        <v>2443</v>
+      </c>
+    </row>
+    <row r="210" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B210" s="17" t="s">
         <v>209</v>
       </c>
-      <c r="C210" s="12" t="n">
-        <v>64595</v>
+      <c r="C210" s="11" t="n">
+        <v>186</v>
       </c>
     </row>
     <row r="211" ht="11" customHeight="true" outlineLevel="3">
@@ -3200,23 +3245,23 @@
         <v>210</v>
       </c>
       <c r="C211" s="18" t="n">
-        <v>1127</v>
+        <v>1581</v>
       </c>
     </row>
     <row r="212" ht="11" customHeight="true" outlineLevel="3">
       <c r="B212" s="17" t="s">
         <v>211</v>
       </c>
-      <c r="C212" s="11" t="n">
-        <v>945</v>
+      <c r="C212" s="18" t="n">
+        <v>18770</v>
       </c>
     </row>
     <row r="213" ht="11" customHeight="true" outlineLevel="3">
       <c r="B213" s="17" t="s">
         <v>212</v>
       </c>
-      <c r="C213" s="18" t="n">
-        <v>2260</v>
+      <c r="C213" s="11" t="n">
+        <v>562</v>
       </c>
     </row>
     <row r="214" ht="11" customHeight="true" outlineLevel="3">
@@ -3224,31 +3269,31 @@
         <v>213</v>
       </c>
       <c r="C214" s="11" t="n">
-        <v>7</v>
+        <v>396</v>
       </c>
     </row>
     <row r="215" ht="11" customHeight="true" outlineLevel="3">
       <c r="B215" s="17" t="s">
         <v>214</v>
       </c>
-      <c r="C215" s="11" t="n">
-        <v>741</v>
+      <c r="C215" s="18" t="n">
+        <v>1276</v>
       </c>
     </row>
     <row r="216" ht="11" customHeight="true" outlineLevel="3">
       <c r="B216" s="17" t="s">
         <v>215</v>
       </c>
-      <c r="C216" s="11" t="n">
-        <v>484</v>
+      <c r="C216" s="18" t="n">
+        <v>1318</v>
       </c>
     </row>
     <row r="217" ht="11" customHeight="true" outlineLevel="3">
       <c r="B217" s="17" t="s">
         <v>216</v>
       </c>
-      <c r="C217" s="18" t="n">
-        <v>5794</v>
+      <c r="C217" s="11" t="n">
+        <v>639</v>
       </c>
     </row>
     <row r="218" ht="11" customHeight="true" outlineLevel="3">
@@ -3256,23 +3301,23 @@
         <v>217</v>
       </c>
       <c r="C218" s="11" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
     </row>
     <row r="219" ht="11" customHeight="true" outlineLevel="3">
       <c r="B219" s="17" t="s">
         <v>218</v>
       </c>
-      <c r="C219" s="11" t="n">
-        <v>187</v>
+      <c r="C219" s="18" t="n">
+        <v>1756</v>
       </c>
     </row>
     <row r="220" ht="11" customHeight="true" outlineLevel="3">
       <c r="B220" s="17" t="s">
         <v>219</v>
       </c>
-      <c r="C220" s="11" t="n">
-        <v>159</v>
+      <c r="C220" s="18" t="n">
+        <v>2951</v>
       </c>
     </row>
     <row r="221" ht="11" customHeight="true" outlineLevel="3">
@@ -3280,7 +3325,7 @@
         <v>220</v>
       </c>
       <c r="C221" s="18" t="n">
-        <v>1458</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="222" ht="11" customHeight="true" outlineLevel="3">
@@ -3288,31 +3333,31 @@
         <v>221</v>
       </c>
       <c r="C222" s="11" t="n">
-        <v>592</v>
-      </c>
-    </row>
-    <row r="223" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B223" s="17" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="223" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B223" s="16" t="s">
         <v>222</v>
       </c>
-      <c r="C223" s="18" t="n">
-        <v>2272</v>
+      <c r="C223" s="12" t="n">
+        <v>42245</v>
       </c>
     </row>
     <row r="224" ht="11" customHeight="true" outlineLevel="3">
       <c r="B224" s="17" t="s">
         <v>223</v>
       </c>
-      <c r="C224" s="18" t="n">
-        <v>2730</v>
+      <c r="C224" s="11" t="n">
+        <v>870</v>
       </c>
     </row>
     <row r="225" ht="11" customHeight="true" outlineLevel="3">
       <c r="B225" s="17" t="s">
         <v>224</v>
       </c>
-      <c r="C225" s="18" t="n">
-        <v>1983</v>
+      <c r="C225" s="11" t="n">
+        <v>694</v>
       </c>
     </row>
     <row r="226" ht="11" customHeight="true" outlineLevel="3">
@@ -3320,15 +3365,15 @@
         <v>225</v>
       </c>
       <c r="C226" s="18" t="n">
-        <v>1154</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="227" ht="11" customHeight="true" outlineLevel="3">
       <c r="B227" s="17" t="s">
         <v>226</v>
       </c>
-      <c r="C227" s="18" t="n">
-        <v>1178</v>
+      <c r="C227" s="11" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="228" ht="11" customHeight="true" outlineLevel="3">
@@ -3336,15 +3381,15 @@
         <v>227</v>
       </c>
       <c r="C228" s="11" t="n">
-        <v>725</v>
+        <v>598</v>
       </c>
     </row>
     <row r="229" ht="11" customHeight="true" outlineLevel="3">
       <c r="B229" s="17" t="s">
         <v>228</v>
       </c>
-      <c r="C229" s="18" t="n">
-        <v>1801</v>
+      <c r="C229" s="11" t="n">
+        <v>652</v>
       </c>
     </row>
     <row r="230" ht="11" customHeight="true" outlineLevel="3">
@@ -3352,7 +3397,7 @@
         <v>229</v>
       </c>
       <c r="C230" s="18" t="n">
-        <v>1371</v>
+        <v>3823</v>
       </c>
     </row>
     <row r="231" ht="11" customHeight="true" outlineLevel="3">
@@ -3360,23 +3405,23 @@
         <v>230</v>
       </c>
       <c r="C231" s="11" t="n">
-        <v>377</v>
+        <v>50</v>
       </c>
     </row>
     <row r="232" ht="11" customHeight="true" outlineLevel="3">
       <c r="B232" s="17" t="s">
         <v>231</v>
       </c>
-      <c r="C232" s="18" t="n">
-        <v>1855</v>
+      <c r="C232" s="11" t="n">
+        <v>96</v>
       </c>
     </row>
     <row r="233" ht="11" customHeight="true" outlineLevel="3">
       <c r="B233" s="17" t="s">
         <v>232</v>
       </c>
-      <c r="C233" s="18" t="n">
-        <v>2873</v>
+      <c r="C233" s="11" t="n">
+        <v>173</v>
       </c>
     </row>
     <row r="234" ht="11" customHeight="true" outlineLevel="3">
@@ -3384,15 +3429,15 @@
         <v>233</v>
       </c>
       <c r="C234" s="18" t="n">
-        <v>2673</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="235" ht="11" customHeight="true" outlineLevel="3">
       <c r="B235" s="17" t="s">
         <v>234</v>
       </c>
-      <c r="C235" s="18" t="n">
-        <v>2807</v>
+      <c r="C235" s="11" t="n">
+        <v>443</v>
       </c>
     </row>
     <row r="236" ht="11" customHeight="true" outlineLevel="3">
@@ -3400,7 +3445,7 @@
         <v>235</v>
       </c>
       <c r="C236" s="18" t="n">
-        <v>2567</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="237" ht="11" customHeight="true" outlineLevel="3">
@@ -3408,39 +3453,39 @@
         <v>236</v>
       </c>
       <c r="C237" s="18" t="n">
-        <v>2778</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="238" ht="11" customHeight="true" outlineLevel="3">
       <c r="B238" s="17" t="s">
         <v>237</v>
       </c>
-      <c r="C238" s="11" t="n">
-        <v>824</v>
+      <c r="C238" s="18" t="n">
+        <v>1024</v>
       </c>
     </row>
     <row r="239" ht="11" customHeight="true" outlineLevel="3">
       <c r="B239" s="17" t="s">
         <v>238</v>
       </c>
-      <c r="C239" s="18" t="n">
-        <v>1004</v>
+      <c r="C239" s="11" t="n">
+        <v>791</v>
       </c>
     </row>
     <row r="240" ht="11" customHeight="true" outlineLevel="3">
       <c r="B240" s="17" t="s">
         <v>239</v>
       </c>
-      <c r="C240" s="18" t="n">
-        <v>4038</v>
+      <c r="C240" s="11" t="n">
+        <v>483</v>
       </c>
     </row>
     <row r="241" ht="11" customHeight="true" outlineLevel="3">
       <c r="B241" s="17" t="s">
         <v>240</v>
       </c>
-      <c r="C241" s="18" t="n">
-        <v>1833</v>
+      <c r="C241" s="11" t="n">
+        <v>515</v>
       </c>
     </row>
     <row r="242" ht="11" customHeight="true" outlineLevel="3">
@@ -3448,79 +3493,79 @@
         <v>241</v>
       </c>
       <c r="C242" s="18" t="n">
-        <v>1714</v>
+        <v>1169</v>
       </c>
     </row>
     <row r="243" ht="11" customHeight="true" outlineLevel="3">
       <c r="B243" s="17" t="s">
         <v>242</v>
       </c>
-      <c r="C243" s="18" t="n">
-        <v>2695</v>
+      <c r="C243" s="11" t="n">
+        <v>903</v>
       </c>
     </row>
     <row r="244" ht="11" customHeight="true" outlineLevel="3">
       <c r="B244" s="17" t="s">
         <v>243</v>
       </c>
-      <c r="C244" s="18" t="n">
-        <v>7807</v>
+      <c r="C244" s="11" t="n">
+        <v>206</v>
       </c>
     </row>
     <row r="245" ht="11" customHeight="true" outlineLevel="3">
       <c r="B245" s="17" t="s">
         <v>244</v>
       </c>
-      <c r="C245" s="18" t="n">
-        <v>1731</v>
-      </c>
-    </row>
-    <row r="246" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B246" s="16" t="s">
+      <c r="C245" s="11" t="n">
+        <v>865</v>
+      </c>
+    </row>
+    <row r="246" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B246" s="17" t="s">
         <v>245</v>
       </c>
-      <c r="C246" s="12" t="n">
-        <v>6194</v>
+      <c r="C246" s="18" t="n">
+        <v>1891</v>
       </c>
     </row>
     <row r="247" ht="11" customHeight="true" outlineLevel="3">
       <c r="B247" s="17" t="s">
         <v>246</v>
       </c>
-      <c r="C247" s="11" t="n">
-        <v>868</v>
+      <c r="C247" s="18" t="n">
+        <v>2328</v>
       </c>
     </row>
     <row r="248" ht="11" customHeight="true" outlineLevel="3">
       <c r="B248" s="17" t="s">
         <v>247</v>
       </c>
-      <c r="C248" s="11" t="n">
-        <v>711</v>
+      <c r="C248" s="18" t="n">
+        <v>2005</v>
       </c>
     </row>
     <row r="249" ht="11" customHeight="true" outlineLevel="3">
       <c r="B249" s="17" t="s">
         <v>248</v>
       </c>
-      <c r="C249" s="11" t="n">
-        <v>93</v>
+      <c r="C249" s="18" t="n">
+        <v>1539</v>
       </c>
     </row>
     <row r="250" ht="11" customHeight="true" outlineLevel="3">
       <c r="B250" s="17" t="s">
         <v>249</v>
       </c>
-      <c r="C250" s="11" t="n">
-        <v>508</v>
+      <c r="C250" s="18" t="n">
+        <v>2028</v>
       </c>
     </row>
     <row r="251" ht="11" customHeight="true" outlineLevel="3">
       <c r="B251" s="17" t="s">
         <v>250</v>
       </c>
-      <c r="C251" s="11" t="n">
-        <v>70</v>
+      <c r="C251" s="18" t="n">
+        <v>1521</v>
       </c>
     </row>
     <row r="252" ht="11" customHeight="true" outlineLevel="3">
@@ -3528,47 +3573,47 @@
         <v>251</v>
       </c>
       <c r="C252" s="11" t="n">
-        <v>615</v>
+        <v>115</v>
       </c>
     </row>
     <row r="253" ht="11" customHeight="true" outlineLevel="3">
       <c r="B253" s="17" t="s">
         <v>252</v>
       </c>
-      <c r="C253" s="11" t="n">
-        <v>663</v>
+      <c r="C253" s="18" t="n">
+        <v>2015</v>
       </c>
     </row>
     <row r="254" ht="11" customHeight="true" outlineLevel="3">
       <c r="B254" s="17" t="s">
         <v>253</v>
       </c>
-      <c r="C254" s="11" t="n">
-        <v>384</v>
+      <c r="C254" s="18" t="n">
+        <v>1351</v>
       </c>
     </row>
     <row r="255" ht="11" customHeight="true" outlineLevel="3">
       <c r="B255" s="17" t="s">
         <v>254</v>
       </c>
-      <c r="C255" s="11" t="n">
-        <v>304</v>
+      <c r="C255" s="18" t="n">
+        <v>2080</v>
       </c>
     </row>
     <row r="256" ht="11" customHeight="true" outlineLevel="3">
       <c r="B256" s="17" t="s">
         <v>255</v>
       </c>
-      <c r="C256" s="11" t="n">
-        <v>693</v>
+      <c r="C256" s="18" t="n">
+        <v>1532</v>
       </c>
     </row>
     <row r="257" ht="11" customHeight="true" outlineLevel="3">
       <c r="B257" s="17" t="s">
         <v>256</v>
       </c>
-      <c r="C257" s="11" t="n">
-        <v>953</v>
+      <c r="C257" s="18" t="n">
+        <v>4315</v>
       </c>
     </row>
     <row r="258" ht="11" customHeight="true" outlineLevel="3">
@@ -3576,15 +3621,15 @@
         <v>257</v>
       </c>
       <c r="C258" s="11" t="n">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="259" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B259" s="17" t="s">
+        <v>951</v>
+      </c>
+    </row>
+    <row r="259" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B259" s="16" t="s">
         <v>258</v>
       </c>
-      <c r="C259" s="11" t="n">
-        <v>7</v>
+      <c r="C259" s="12" t="n">
+        <v>5702</v>
       </c>
     </row>
     <row r="260" ht="11" customHeight="true" outlineLevel="3">
@@ -3592,15 +3637,15 @@
         <v>259</v>
       </c>
       <c r="C260" s="11" t="n">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="261" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B261" s="16" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="261" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B261" s="17" t="s">
         <v>260</v>
       </c>
-      <c r="C261" s="12" t="n">
-        <v>28446</v>
+      <c r="C261" s="11" t="n">
+        <v>251</v>
       </c>
     </row>
     <row r="262" ht="11" customHeight="true" outlineLevel="3">
@@ -3608,7 +3653,7 @@
         <v>261</v>
       </c>
       <c r="C262" s="11" t="n">
-        <v>352</v>
+        <v>625</v>
       </c>
     </row>
     <row r="263" ht="11" customHeight="true" outlineLevel="3">
@@ -3616,7 +3661,7 @@
         <v>262</v>
       </c>
       <c r="C263" s="11" t="n">
-        <v>353</v>
+        <v>25</v>
       </c>
     </row>
     <row r="264" ht="11" customHeight="true" outlineLevel="3">
@@ -3624,7 +3669,7 @@
         <v>263</v>
       </c>
       <c r="C264" s="11" t="n">
-        <v>459</v>
+        <v>777</v>
       </c>
     </row>
     <row r="265" ht="11" customHeight="true" outlineLevel="3">
@@ -3632,7 +3677,7 @@
         <v>264</v>
       </c>
       <c r="C265" s="11" t="n">
-        <v>461</v>
+        <v>201</v>
       </c>
     </row>
     <row r="266" ht="11" customHeight="true" outlineLevel="3">
@@ -3640,7 +3685,7 @@
         <v>265</v>
       </c>
       <c r="C266" s="11" t="n">
-        <v>315</v>
+        <v>64</v>
       </c>
     </row>
     <row r="267" ht="11" customHeight="true" outlineLevel="3">
@@ -3648,7 +3693,7 @@
         <v>266</v>
       </c>
       <c r="C267" s="11" t="n">
-        <v>394</v>
+        <v>336</v>
       </c>
     </row>
     <row r="268" ht="11" customHeight="true" outlineLevel="3">
@@ -3656,15 +3701,15 @@
         <v>267</v>
       </c>
       <c r="C268" s="11" t="n">
-        <v>717</v>
-      </c>
-    </row>
-    <row r="269" ht="22" customHeight="true" outlineLevel="3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="269" ht="11" customHeight="true" outlineLevel="3">
       <c r="B269" s="17" t="s">
         <v>268</v>
       </c>
       <c r="C269" s="11" t="n">
-        <v>39</v>
+        <v>292</v>
       </c>
     </row>
     <row r="270" ht="11" customHeight="true" outlineLevel="3">
@@ -3672,7 +3717,7 @@
         <v>269</v>
       </c>
       <c r="C270" s="11" t="n">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="271" ht="11" customHeight="true" outlineLevel="3">
@@ -3680,15 +3725,15 @@
         <v>270</v>
       </c>
       <c r="C271" s="11" t="n">
-        <v>435</v>
+        <v>283</v>
       </c>
     </row>
     <row r="272" ht="11" customHeight="true" outlineLevel="3">
       <c r="B272" s="17" t="s">
         <v>271</v>
       </c>
-      <c r="C272" s="18" t="n">
-        <v>1209</v>
+      <c r="C272" s="11" t="n">
+        <v>765</v>
       </c>
     </row>
     <row r="273" ht="11" customHeight="true" outlineLevel="3">
@@ -3696,79 +3741,79 @@
         <v>272</v>
       </c>
       <c r="C273" s="11" t="n">
-        <v>420</v>
+        <v>85</v>
       </c>
     </row>
     <row r="274" ht="11" customHeight="true" outlineLevel="3">
       <c r="B274" s="17" t="s">
         <v>273</v>
       </c>
-      <c r="C274" s="18" t="n">
-        <v>1548</v>
-      </c>
-    </row>
-    <row r="275" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C274" s="11" t="n">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="275" ht="11" customHeight="true" outlineLevel="3">
       <c r="B275" s="17" t="s">
         <v>274</v>
       </c>
       <c r="C275" s="11" t="n">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="276" ht="22" customHeight="true" outlineLevel="3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="276" ht="11" customHeight="true" outlineLevel="3">
       <c r="B276" s="17" t="s">
         <v>275</v>
       </c>
       <c r="C276" s="11" t="n">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="277" ht="22" customHeight="true" outlineLevel="3">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="277" ht="11" customHeight="true" outlineLevel="3">
       <c r="B277" s="17" t="s">
         <v>276</v>
       </c>
       <c r="C277" s="11" t="n">
-        <v>786</v>
-      </c>
-    </row>
-    <row r="278" ht="22" customHeight="true" outlineLevel="3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="278" ht="11" customHeight="true" outlineLevel="3">
       <c r="B278" s="17" t="s">
         <v>277</v>
       </c>
       <c r="C278" s="11" t="n">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="279" ht="22" customHeight="true" outlineLevel="3">
-      <c r="B279" s="17" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="279" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B279" s="16" t="s">
         <v>278</v>
       </c>
-      <c r="C279" s="11" t="n">
-        <v>511</v>
-      </c>
-    </row>
-    <row r="280" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C279" s="12" t="n">
+        <v>32502</v>
+      </c>
+    </row>
+    <row r="280" ht="11" customHeight="true" outlineLevel="3">
       <c r="B280" s="17" t="s">
         <v>279</v>
       </c>
       <c r="C280" s="11" t="n">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="281" ht="22" customHeight="true" outlineLevel="3">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="281" ht="11" customHeight="true" outlineLevel="3">
       <c r="B281" s="17" t="s">
         <v>280</v>
       </c>
       <c r="C281" s="11" t="n">
-        <v>631</v>
-      </c>
-    </row>
-    <row r="282" ht="22" customHeight="true" outlineLevel="3">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="282" ht="11" customHeight="true" outlineLevel="3">
       <c r="B282" s="17" t="s">
         <v>281</v>
       </c>
       <c r="C282" s="11" t="n">
-        <v>133</v>
+        <v>90</v>
       </c>
     </row>
     <row r="283" ht="11" customHeight="true" outlineLevel="3">
@@ -3776,7 +3821,7 @@
         <v>282</v>
       </c>
       <c r="C283" s="11" t="n">
-        <v>817</v>
+        <v>716</v>
       </c>
     </row>
     <row r="284" ht="11" customHeight="true" outlineLevel="3">
@@ -3784,7 +3829,7 @@
         <v>283</v>
       </c>
       <c r="C284" s="11" t="n">
-        <v>599</v>
+        <v>539</v>
       </c>
     </row>
     <row r="285" ht="11" customHeight="true" outlineLevel="3">
@@ -3792,7 +3837,7 @@
         <v>284</v>
       </c>
       <c r="C285" s="11" t="n">
-        <v>500</v>
+        <v>893</v>
       </c>
     </row>
     <row r="286" ht="11" customHeight="true" outlineLevel="3">
@@ -3800,31 +3845,31 @@
         <v>285</v>
       </c>
       <c r="C286" s="11" t="n">
-        <v>227</v>
+        <v>811</v>
       </c>
     </row>
     <row r="287" ht="11" customHeight="true" outlineLevel="3">
       <c r="B287" s="17" t="s">
         <v>286</v>
       </c>
-      <c r="C287" s="18" t="n">
-        <v>2445</v>
-      </c>
-    </row>
-    <row r="288" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C287" s="11" t="n">
+        <v>879</v>
+      </c>
+    </row>
+    <row r="288" ht="22" customHeight="true" outlineLevel="3">
       <c r="B288" s="17" t="s">
         <v>287</v>
       </c>
-      <c r="C288" s="18" t="n">
-        <v>3739</v>
+      <c r="C288" s="11" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="289" ht="11" customHeight="true" outlineLevel="3">
       <c r="B289" s="17" t="s">
         <v>288</v>
       </c>
-      <c r="C289" s="18" t="n">
-        <v>1180</v>
+      <c r="C289" s="11" t="n">
+        <v>44</v>
       </c>
     </row>
     <row r="290" ht="11" customHeight="true" outlineLevel="3">
@@ -3832,7 +3877,7 @@
         <v>289</v>
       </c>
       <c r="C290" s="11" t="n">
-        <v>967</v>
+        <v>235</v>
       </c>
     </row>
     <row r="291" ht="11" customHeight="true" outlineLevel="3">
@@ -3840,15 +3885,15 @@
         <v>290</v>
       </c>
       <c r="C291" s="18" t="n">
-        <v>2559</v>
+        <v>1440</v>
       </c>
     </row>
     <row r="292" ht="11" customHeight="true" outlineLevel="3">
       <c r="B292" s="17" t="s">
         <v>291</v>
       </c>
-      <c r="C292" s="11" t="n">
-        <v>7</v>
+      <c r="C292" s="18" t="n">
+        <v>1164</v>
       </c>
     </row>
     <row r="293" ht="11" customHeight="true" outlineLevel="3">
@@ -3856,95 +3901,95 @@
         <v>292</v>
       </c>
       <c r="C293" s="18" t="n">
-        <v>2170</v>
-      </c>
-    </row>
-    <row r="294" ht="11" customHeight="true" outlineLevel="3">
+        <v>1836</v>
+      </c>
+    </row>
+    <row r="294" ht="22" customHeight="true" outlineLevel="3">
       <c r="B294" s="17" t="s">
         <v>293</v>
       </c>
-      <c r="C294" s="18" t="n">
-        <v>1152</v>
-      </c>
-    </row>
-    <row r="295" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C294" s="11" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="295" ht="22" customHeight="true" outlineLevel="3">
       <c r="B295" s="17" t="s">
         <v>294</v>
       </c>
       <c r="C295" s="11" t="n">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="296" ht="11" customHeight="true" outlineLevel="3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="296" ht="22" customHeight="true" outlineLevel="3">
       <c r="B296" s="17" t="s">
         <v>295</v>
       </c>
       <c r="C296" s="11" t="n">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="297" ht="11" customHeight="true" outlineLevel="3">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="297" ht="22" customHeight="true" outlineLevel="3">
       <c r="B297" s="17" t="s">
         <v>296</v>
       </c>
-      <c r="C297" s="18" t="n">
-        <v>1796</v>
-      </c>
-    </row>
-    <row r="298" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B298" s="16" t="s">
+      <c r="C297" s="11" t="n">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="298" ht="22" customHeight="true" outlineLevel="3">
+      <c r="B298" s="17" t="s">
         <v>297</v>
       </c>
-      <c r="C298" s="12" t="n">
-        <v>52151</v>
-      </c>
-    </row>
-    <row r="299" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C298" s="11" t="n">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="299" ht="22" customHeight="true" outlineLevel="3">
       <c r="B299" s="17" t="s">
         <v>298</v>
       </c>
-      <c r="C299" s="18" t="n">
-        <v>3776</v>
-      </c>
-    </row>
-    <row r="300" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C299" s="11" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="300" ht="22" customHeight="true" outlineLevel="3">
       <c r="B300" s="17" t="s">
         <v>299</v>
       </c>
       <c r="C300" s="11" t="n">
-        <v>910</v>
-      </c>
-    </row>
-    <row r="301" ht="11" customHeight="true" outlineLevel="3">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="301" ht="22" customHeight="true" outlineLevel="3">
       <c r="B301" s="17" t="s">
         <v>300</v>
       </c>
       <c r="C301" s="11" t="n">
-        <v>753</v>
-      </c>
-    </row>
-    <row r="302" ht="22" customHeight="true" outlineLevel="3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="302" ht="11" customHeight="true" outlineLevel="3">
       <c r="B302" s="17" t="s">
         <v>301</v>
       </c>
-      <c r="C302" s="18" t="n">
-        <v>1557</v>
-      </c>
-    </row>
-    <row r="303" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C302" s="11" t="n">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="303" ht="11" customHeight="true" outlineLevel="3">
       <c r="B303" s="17" t="s">
         <v>302</v>
       </c>
-      <c r="C303" s="18" t="n">
-        <v>2312</v>
+      <c r="C303" s="11" t="n">
+        <v>601</v>
       </c>
     </row>
     <row r="304" ht="11" customHeight="true" outlineLevel="3">
       <c r="B304" s="17" t="s">
         <v>303</v>
       </c>
-      <c r="C304" s="18" t="n">
-        <v>1967</v>
+      <c r="C304" s="11" t="n">
+        <v>351</v>
       </c>
     </row>
     <row r="305" ht="11" customHeight="true" outlineLevel="3">
@@ -3952,15 +3997,15 @@
         <v>304</v>
       </c>
       <c r="C305" s="11" t="n">
-        <v>871</v>
+        <v>308</v>
       </c>
     </row>
     <row r="306" ht="11" customHeight="true" outlineLevel="3">
       <c r="B306" s="17" t="s">
         <v>305</v>
       </c>
-      <c r="C306" s="11" t="n">
-        <v>168</v>
+      <c r="C306" s="18" t="n">
+        <v>3323</v>
       </c>
     </row>
     <row r="307" ht="11" customHeight="true" outlineLevel="3">
@@ -3968,15 +4013,15 @@
         <v>306</v>
       </c>
       <c r="C307" s="18" t="n">
-        <v>1056</v>
+        <v>1368</v>
       </c>
     </row>
     <row r="308" ht="11" customHeight="true" outlineLevel="3">
       <c r="B308" s="17" t="s">
         <v>307</v>
       </c>
-      <c r="C308" s="18" t="n">
-        <v>1786</v>
+      <c r="C308" s="11" t="n">
+        <v>971</v>
       </c>
     </row>
     <row r="309" ht="11" customHeight="true" outlineLevel="3">
@@ -3984,15 +4029,15 @@
         <v>308</v>
       </c>
       <c r="C309" s="11" t="n">
-        <v>504</v>
+        <v>634</v>
       </c>
     </row>
     <row r="310" ht="11" customHeight="true" outlineLevel="3">
       <c r="B310" s="17" t="s">
         <v>309</v>
       </c>
-      <c r="C310" s="11" t="n">
-        <v>60</v>
+      <c r="C310" s="18" t="n">
+        <v>3209</v>
       </c>
     </row>
     <row r="311" ht="11" customHeight="true" outlineLevel="3">
@@ -4000,15 +4045,15 @@
         <v>310</v>
       </c>
       <c r="C311" s="11" t="n">
-        <v>217</v>
+        <v>7</v>
       </c>
     </row>
     <row r="312" ht="11" customHeight="true" outlineLevel="3">
       <c r="B312" s="17" t="s">
         <v>311</v>
       </c>
-      <c r="C312" s="11" t="n">
-        <v>300</v>
+      <c r="C312" s="18" t="n">
+        <v>4114</v>
       </c>
     </row>
     <row r="313" ht="11" customHeight="true" outlineLevel="3">
@@ -4016,15 +4061,15 @@
         <v>312</v>
       </c>
       <c r="C313" s="11" t="n">
-        <v>421</v>
+        <v>169</v>
       </c>
     </row>
     <row r="314" ht="11" customHeight="true" outlineLevel="3">
       <c r="B314" s="17" t="s">
         <v>313</v>
       </c>
-      <c r="C314" s="11" t="n">
-        <v>525</v>
+      <c r="C314" s="18" t="n">
+        <v>1475</v>
       </c>
     </row>
     <row r="315" ht="11" customHeight="true" outlineLevel="3">
@@ -4032,63 +4077,63 @@
         <v>314</v>
       </c>
       <c r="C315" s="11" t="n">
-        <v>350</v>
+        <v>194</v>
       </c>
     </row>
     <row r="316" ht="11" customHeight="true" outlineLevel="3">
       <c r="B316" s="17" t="s">
         <v>315</v>
       </c>
-      <c r="C316" s="11" t="n">
-        <v>647</v>
-      </c>
-    </row>
-    <row r="317" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B317" s="17" t="s">
+      <c r="C316" s="18" t="n">
+        <v>3364</v>
+      </c>
+    </row>
+    <row r="317" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B317" s="16" t="s">
         <v>316</v>
       </c>
-      <c r="C317" s="11" t="n">
-        <v>633</v>
+      <c r="C317" s="12" t="n">
+        <v>39803</v>
       </c>
     </row>
     <row r="318" ht="11" customHeight="true" outlineLevel="3">
       <c r="B318" s="17" t="s">
         <v>317</v>
       </c>
-      <c r="C318" s="11" t="n">
-        <v>398</v>
+      <c r="C318" s="18" t="n">
+        <v>3118</v>
       </c>
     </row>
     <row r="319" ht="11" customHeight="true" outlineLevel="3">
       <c r="B319" s="17" t="s">
         <v>318</v>
       </c>
-      <c r="C319" s="18" t="n">
-        <v>1291</v>
+      <c r="C319" s="11" t="n">
+        <v>513</v>
       </c>
     </row>
     <row r="320" ht="11" customHeight="true" outlineLevel="3">
       <c r="B320" s="17" t="s">
         <v>319</v>
       </c>
-      <c r="C320" s="18" t="n">
-        <v>1391</v>
-      </c>
-    </row>
-    <row r="321" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C320" s="11" t="n">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="321" ht="22" customHeight="true" outlineLevel="3">
       <c r="B321" s="17" t="s">
         <v>320</v>
       </c>
       <c r="C321" s="18" t="n">
-        <v>2284</v>
-      </c>
-    </row>
-    <row r="322" ht="11" customHeight="true" outlineLevel="3">
+        <v>1173</v>
+      </c>
+    </row>
+    <row r="322" ht="22" customHeight="true" outlineLevel="3">
       <c r="B322" s="17" t="s">
         <v>321</v>
       </c>
-      <c r="C322" s="11" t="n">
-        <v>737</v>
+      <c r="C322" s="18" t="n">
+        <v>1918</v>
       </c>
     </row>
     <row r="323" ht="11" customHeight="true" outlineLevel="3">
@@ -4096,7 +4141,7 @@
         <v>322</v>
       </c>
       <c r="C323" s="11" t="n">
-        <v>110</v>
+        <v>943</v>
       </c>
     </row>
     <row r="324" ht="11" customHeight="true" outlineLevel="3">
@@ -4104,7 +4149,7 @@
         <v>323</v>
       </c>
       <c r="C324" s="11" t="n">
-        <v>893</v>
+        <v>849</v>
       </c>
     </row>
     <row r="325" ht="11" customHeight="true" outlineLevel="3">
@@ -4112,7 +4157,7 @@
         <v>324</v>
       </c>
       <c r="C325" s="11" t="n">
-        <v>675</v>
+        <v>918</v>
       </c>
     </row>
     <row r="326" ht="11" customHeight="true" outlineLevel="3">
@@ -4120,15 +4165,15 @@
         <v>325</v>
       </c>
       <c r="C326" s="18" t="n">
-        <v>2264</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="327" ht="11" customHeight="true" outlineLevel="3">
       <c r="B327" s="17" t="s">
         <v>326</v>
       </c>
-      <c r="C327" s="11" t="n">
-        <v>164</v>
+      <c r="C327" s="18" t="n">
+        <v>1096</v>
       </c>
     </row>
     <row r="328" ht="11" customHeight="true" outlineLevel="3">
@@ -4136,7 +4181,7 @@
         <v>327</v>
       </c>
       <c r="C328" s="11" t="n">
-        <v>889</v>
+        <v>398</v>
       </c>
     </row>
     <row r="329" ht="11" customHeight="true" outlineLevel="3">
@@ -4144,7 +4189,7 @@
         <v>328</v>
       </c>
       <c r="C329" s="11" t="n">
-        <v>512</v>
+        <v>68</v>
       </c>
     </row>
     <row r="330" ht="11" customHeight="true" outlineLevel="3">
@@ -4152,7 +4197,7 @@
         <v>329</v>
       </c>
       <c r="C330" s="11" t="n">
-        <v>989</v>
+        <v>96</v>
       </c>
     </row>
     <row r="331" ht="11" customHeight="true" outlineLevel="3">
@@ -4160,39 +4205,39 @@
         <v>330</v>
       </c>
       <c r="C331" s="11" t="n">
-        <v>938</v>
+        <v>491</v>
       </c>
     </row>
     <row r="332" ht="11" customHeight="true" outlineLevel="3">
       <c r="B332" s="17" t="s">
         <v>331</v>
       </c>
-      <c r="C332" s="18" t="n">
-        <v>1067</v>
+      <c r="C332" s="11" t="n">
+        <v>321</v>
       </c>
     </row>
     <row r="333" ht="11" customHeight="true" outlineLevel="3">
       <c r="B333" s="17" t="s">
         <v>332</v>
       </c>
-      <c r="C333" s="18" t="n">
-        <v>1133</v>
+      <c r="C333" s="11" t="n">
+        <v>343</v>
       </c>
     </row>
     <row r="334" ht="11" customHeight="true" outlineLevel="3">
       <c r="B334" s="17" t="s">
         <v>333</v>
       </c>
-      <c r="C334" s="18" t="n">
-        <v>9503</v>
+      <c r="C334" s="11" t="n">
+        <v>350</v>
       </c>
     </row>
     <row r="335" ht="11" customHeight="true" outlineLevel="3">
       <c r="B335" s="17" t="s">
         <v>334</v>
       </c>
-      <c r="C335" s="18" t="n">
-        <v>5145</v>
+      <c r="C335" s="11" t="n">
+        <v>398</v>
       </c>
     </row>
     <row r="336" ht="11" customHeight="true" outlineLevel="3">
@@ -4200,7 +4245,7 @@
         <v>335</v>
       </c>
       <c r="C336" s="18" t="n">
-        <v>1135</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="337" ht="11" customHeight="true" outlineLevel="3">
@@ -4208,23 +4253,23 @@
         <v>336</v>
       </c>
       <c r="C337" s="11" t="n">
-        <v>430</v>
+        <v>812</v>
       </c>
     </row>
     <row r="338" ht="11" customHeight="true" outlineLevel="3">
       <c r="B338" s="17" t="s">
         <v>337</v>
       </c>
-      <c r="C338" s="11" t="n">
-        <v>29</v>
+      <c r="C338" s="18" t="n">
+        <v>1215</v>
       </c>
     </row>
     <row r="339" ht="11" customHeight="true" outlineLevel="3">
       <c r="B339" s="17" t="s">
         <v>338</v>
       </c>
-      <c r="C339" s="18" t="n">
-        <v>1360</v>
+      <c r="C339" s="11" t="n">
+        <v>498</v>
       </c>
     </row>
     <row r="340" ht="11" customHeight="true" outlineLevel="3">
@@ -4232,23 +4277,23 @@
         <v>339</v>
       </c>
       <c r="C340" s="11" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="341" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B341" s="16" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="341" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B341" s="17" t="s">
         <v>340</v>
       </c>
-      <c r="C341" s="14" t="n">
-        <v>89</v>
+      <c r="C341" s="11" t="n">
+        <v>403</v>
       </c>
     </row>
     <row r="342" ht="11" customHeight="true" outlineLevel="3">
       <c r="B342" s="17" t="s">
         <v>341</v>
       </c>
-      <c r="C342" s="11" t="n">
-        <v>6</v>
+      <c r="C342" s="18" t="n">
+        <v>1606</v>
       </c>
     </row>
     <row r="343" ht="11" customHeight="true" outlineLevel="3">
@@ -4256,7 +4301,7 @@
         <v>342</v>
       </c>
       <c r="C343" s="11" t="n">
-        <v>67</v>
+        <v>156</v>
       </c>
     </row>
     <row r="344" ht="11" customHeight="true" outlineLevel="3">
@@ -4264,15 +4309,15 @@
         <v>343</v>
       </c>
       <c r="C344" s="11" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="345" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B345" s="16" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="345" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B345" s="17" t="s">
         <v>344</v>
       </c>
-      <c r="C345" s="12" t="n">
-        <v>32609</v>
+      <c r="C345" s="11" t="n">
+        <v>206</v>
       </c>
     </row>
     <row r="346" ht="11" customHeight="true" outlineLevel="3">
@@ -4280,7 +4325,7 @@
         <v>345</v>
       </c>
       <c r="C346" s="11" t="n">
-        <v>90</v>
+        <v>299</v>
       </c>
     </row>
     <row r="347" ht="11" customHeight="true" outlineLevel="3">
@@ -4288,79 +4333,79 @@
         <v>346</v>
       </c>
       <c r="C347" s="11" t="n">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="348" ht="22" customHeight="true" outlineLevel="3">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="348" ht="11" customHeight="true" outlineLevel="3">
       <c r="B348" s="17" t="s">
         <v>347</v>
       </c>
       <c r="C348" s="11" t="n">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="349" ht="22" customHeight="true" outlineLevel="3">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="349" ht="11" customHeight="true" outlineLevel="3">
       <c r="B349" s="17" t="s">
         <v>348</v>
       </c>
-      <c r="C349" s="11" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="350" ht="33" customHeight="true" outlineLevel="3">
+      <c r="C349" s="18" t="n">
+        <v>8027</v>
+      </c>
+    </row>
+    <row r="350" ht="11" customHeight="true" outlineLevel="3">
       <c r="B350" s="17" t="s">
         <v>349</v>
       </c>
       <c r="C350" s="11" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="351" ht="22" customHeight="true" outlineLevel="3">
+        <v>997</v>
+      </c>
+    </row>
+    <row r="351" ht="11" customHeight="true" outlineLevel="3">
       <c r="B351" s="17" t="s">
         <v>350</v>
       </c>
-      <c r="C351" s="11" t="n">
-        <v>87</v>
+      <c r="C351" s="18" t="n">
+        <v>5551</v>
       </c>
     </row>
     <row r="352" ht="11" customHeight="true" outlineLevel="3">
       <c r="B352" s="17" t="s">
         <v>351</v>
       </c>
-      <c r="C352" s="11" t="n">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="353" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C352" s="18" t="n">
+        <v>1581</v>
+      </c>
+    </row>
+    <row r="353" ht="11" customHeight="true" outlineLevel="3">
       <c r="B353" s="17" t="s">
         <v>352</v>
       </c>
       <c r="C353" s="11" t="n">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="354" ht="22" customHeight="true" outlineLevel="3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="354" ht="11" customHeight="true" outlineLevel="3">
       <c r="B354" s="17" t="s">
         <v>353</v>
       </c>
       <c r="C354" s="11" t="n">
-        <v>466</v>
-      </c>
-    </row>
-    <row r="355" ht="22" customHeight="true" outlineLevel="3">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="355" ht="11" customHeight="true" outlineLevel="3">
       <c r="B355" s="17" t="s">
         <v>354</v>
       </c>
-      <c r="C355" s="18" t="n">
-        <v>1392</v>
-      </c>
-    </row>
-    <row r="356" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B356" s="17" t="s">
+      <c r="C355" s="11" t="n">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="356" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B356" s="16" t="s">
         <v>355</v>
       </c>
-      <c r="C356" s="11" t="n">
-        <v>116</v>
+      <c r="C356" s="14" t="n">
+        <v>259</v>
       </c>
     </row>
     <row r="357" ht="11" customHeight="true" outlineLevel="3">
@@ -4368,15 +4413,15 @@
         <v>356</v>
       </c>
       <c r="C357" s="11" t="n">
-        <v>180</v>
+        <v>18</v>
       </c>
     </row>
     <row r="358" ht="11" customHeight="true" outlineLevel="3">
       <c r="B358" s="17" t="s">
         <v>357</v>
       </c>
-      <c r="C358" s="18" t="n">
-        <v>2863</v>
+      <c r="C358" s="11" t="n">
+        <v>90</v>
       </c>
     </row>
     <row r="359" ht="11" customHeight="true" outlineLevel="3">
@@ -4384,39 +4429,39 @@
         <v>358</v>
       </c>
       <c r="C359" s="11" t="n">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="360" ht="22" customHeight="true" outlineLevel="3">
-      <c r="B360" s="17" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="360" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B360" s="16" t="s">
         <v>359</v>
       </c>
-      <c r="C360" s="11" t="n">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="361" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C360" s="12" t="n">
+        <v>31193</v>
+      </c>
+    </row>
+    <row r="361" ht="11" customHeight="true" outlineLevel="3">
       <c r="B361" s="17" t="s">
         <v>360</v>
       </c>
       <c r="C361" s="11" t="n">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="362" ht="22" customHeight="true" outlineLevel="3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="362" ht="11" customHeight="true" outlineLevel="3">
       <c r="B362" s="17" t="s">
         <v>361</v>
       </c>
       <c r="C362" s="11" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="363" ht="22" customHeight="true" outlineLevel="3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="363" ht="11" customHeight="true" outlineLevel="3">
       <c r="B363" s="17" t="s">
         <v>362</v>
       </c>
       <c r="C363" s="11" t="n">
-        <v>515</v>
+        <v>212</v>
       </c>
     </row>
     <row r="364" ht="22" customHeight="true" outlineLevel="3">
@@ -4424,7 +4469,7 @@
         <v>363</v>
       </c>
       <c r="C364" s="11" t="n">
-        <v>266</v>
+        <v>356</v>
       </c>
     </row>
     <row r="365" ht="22" customHeight="true" outlineLevel="3">
@@ -4432,23 +4477,23 @@
         <v>364</v>
       </c>
       <c r="C365" s="11" t="n">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="366" ht="22" customHeight="true" outlineLevel="3">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="366" ht="11" customHeight="true" outlineLevel="3">
       <c r="B366" s="17" t="s">
         <v>365</v>
       </c>
       <c r="C366" s="11" t="n">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="367" ht="22" customHeight="true" outlineLevel="3">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="367" ht="11" customHeight="true" outlineLevel="3">
       <c r="B367" s="17" t="s">
         <v>366</v>
       </c>
-      <c r="C367" s="18" t="n">
-        <v>1159</v>
+      <c r="C367" s="11" t="n">
+        <v>264</v>
       </c>
     </row>
     <row r="368" ht="22" customHeight="true" outlineLevel="3">
@@ -4456,7 +4501,7 @@
         <v>367</v>
       </c>
       <c r="C368" s="11" t="n">
-        <v>616</v>
+        <v>701</v>
       </c>
     </row>
     <row r="369" ht="22" customHeight="true" outlineLevel="3">
@@ -4464,47 +4509,47 @@
         <v>368</v>
       </c>
       <c r="C369" s="11" t="n">
-        <v>122</v>
+        <v>451</v>
       </c>
     </row>
     <row r="370" ht="22" customHeight="true" outlineLevel="3">
       <c r="B370" s="17" t="s">
         <v>369</v>
       </c>
-      <c r="C370" s="11" t="n">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="371" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C370" s="18" t="n">
+        <v>6704</v>
+      </c>
+    </row>
+    <row r="371" ht="11" customHeight="true" outlineLevel="3">
       <c r="B371" s="17" t="s">
         <v>370</v>
       </c>
       <c r="C371" s="11" t="n">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="372" ht="22" customHeight="true" outlineLevel="3">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="372" ht="11" customHeight="true" outlineLevel="3">
       <c r="B372" s="17" t="s">
         <v>371</v>
       </c>
       <c r="C372" s="11" t="n">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="373" ht="22" customHeight="true" outlineLevel="3">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="373" ht="11" customHeight="true" outlineLevel="3">
       <c r="B373" s="17" t="s">
         <v>372</v>
       </c>
-      <c r="C373" s="11" t="n">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="374" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C373" s="18" t="n">
+        <v>1365</v>
+      </c>
+    </row>
+    <row r="374" ht="11" customHeight="true" outlineLevel="3">
       <c r="B374" s="17" t="s">
         <v>373</v>
       </c>
       <c r="C374" s="11" t="n">
-        <v>38</v>
+        <v>261</v>
       </c>
     </row>
     <row r="375" ht="22" customHeight="true" outlineLevel="3">
@@ -4512,7 +4557,7 @@
         <v>374</v>
       </c>
       <c r="C375" s="11" t="n">
-        <v>41</v>
+        <v>460</v>
       </c>
     </row>
     <row r="376" ht="22" customHeight="true" outlineLevel="3">
@@ -4520,7 +4565,7 @@
         <v>375</v>
       </c>
       <c r="C376" s="11" t="n">
-        <v>72</v>
+        <v>90</v>
       </c>
     </row>
     <row r="377" ht="22" customHeight="true" outlineLevel="3">
@@ -4528,15 +4573,15 @@
         <v>376</v>
       </c>
       <c r="C377" s="11" t="n">
-        <v>252</v>
+        <v>1</v>
       </c>
     </row>
     <row r="378" ht="22" customHeight="true" outlineLevel="3">
       <c r="B378" s="17" t="s">
         <v>377</v>
       </c>
-      <c r="C378" s="11" t="n">
-        <v>978</v>
+      <c r="C378" s="18" t="n">
+        <v>1048</v>
       </c>
     </row>
     <row r="379" ht="22" customHeight="true" outlineLevel="3">
@@ -4544,7 +4589,7 @@
         <v>378</v>
       </c>
       <c r="C379" s="11" t="n">
-        <v>320</v>
+        <v>363</v>
       </c>
     </row>
     <row r="380" ht="22" customHeight="true" outlineLevel="3">
@@ -4552,7 +4597,7 @@
         <v>379</v>
       </c>
       <c r="C380" s="11" t="n">
-        <v>87</v>
+        <v>123</v>
       </c>
     </row>
     <row r="381" ht="22" customHeight="true" outlineLevel="3">
@@ -4560,15 +4605,15 @@
         <v>380</v>
       </c>
       <c r="C381" s="11" t="n">
-        <v>2</v>
+        <v>44</v>
       </c>
     </row>
     <row r="382" ht="22" customHeight="true" outlineLevel="3">
       <c r="B382" s="17" t="s">
         <v>381</v>
       </c>
-      <c r="C382" s="11" t="n">
-        <v>180</v>
+      <c r="C382" s="18" t="n">
+        <v>2808</v>
       </c>
     </row>
     <row r="383" ht="22" customHeight="true" outlineLevel="3">
@@ -4576,15 +4621,15 @@
         <v>382</v>
       </c>
       <c r="C383" s="11" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="384" ht="11" customHeight="true" outlineLevel="3">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="384" ht="22" customHeight="true" outlineLevel="3">
       <c r="B384" s="17" t="s">
         <v>383</v>
       </c>
       <c r="C384" s="11" t="n">
-        <v>247</v>
+        <v>137</v>
       </c>
     </row>
     <row r="385" ht="22" customHeight="true" outlineLevel="3">
@@ -4592,7 +4637,7 @@
         <v>384</v>
       </c>
       <c r="C385" s="11" t="n">
-        <v>182</v>
+        <v>106</v>
       </c>
     </row>
     <row r="386" ht="22" customHeight="true" outlineLevel="3">
@@ -4600,7 +4645,7 @@
         <v>385</v>
       </c>
       <c r="C386" s="11" t="n">
-        <v>24</v>
+        <v>162</v>
       </c>
     </row>
     <row r="387" ht="22" customHeight="true" outlineLevel="3">
@@ -4608,7 +4653,7 @@
         <v>386</v>
       </c>
       <c r="C387" s="11" t="n">
-        <v>8</v>
+        <v>36</v>
       </c>
     </row>
     <row r="388" ht="22" customHeight="true" outlineLevel="3">
@@ -4616,7 +4661,7 @@
         <v>387</v>
       </c>
       <c r="C388" s="11" t="n">
-        <v>177</v>
+        <v>358</v>
       </c>
     </row>
     <row r="389" ht="22" customHeight="true" outlineLevel="3">
@@ -4624,7 +4669,7 @@
         <v>388</v>
       </c>
       <c r="C389" s="11" t="n">
-        <v>108</v>
+        <v>5</v>
       </c>
     </row>
     <row r="390" ht="22" customHeight="true" outlineLevel="3">
@@ -4632,7 +4677,7 @@
         <v>389</v>
       </c>
       <c r="C390" s="11" t="n">
-        <v>95</v>
+        <v>108</v>
       </c>
     </row>
     <row r="391" ht="22" customHeight="true" outlineLevel="3">
@@ -4640,7 +4685,7 @@
         <v>390</v>
       </c>
       <c r="C391" s="11" t="n">
-        <v>92</v>
+        <v>143</v>
       </c>
     </row>
     <row r="392" ht="22" customHeight="true" outlineLevel="3">
@@ -4648,7 +4693,7 @@
         <v>391</v>
       </c>
       <c r="C392" s="11" t="n">
-        <v>360</v>
+        <v>133</v>
       </c>
     </row>
     <row r="393" ht="22" customHeight="true" outlineLevel="3">
@@ -4656,15 +4701,15 @@
         <v>392</v>
       </c>
       <c r="C393" s="11" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="394" ht="11" customHeight="true" outlineLevel="3">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="394" ht="22" customHeight="true" outlineLevel="3">
       <c r="B394" s="17" t="s">
         <v>393</v>
       </c>
       <c r="C394" s="11" t="n">
-        <v>281</v>
+        <v>51</v>
       </c>
     </row>
     <row r="395" ht="22" customHeight="true" outlineLevel="3">
@@ -4672,23 +4717,23 @@
         <v>394</v>
       </c>
       <c r="C395" s="11" t="n">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="396" ht="11" customHeight="true" outlineLevel="3">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="396" ht="22" customHeight="true" outlineLevel="3">
       <c r="B396" s="17" t="s">
         <v>395</v>
       </c>
       <c r="C396" s="11" t="n">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="397" ht="11" customHeight="true" outlineLevel="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="397" ht="22" customHeight="true" outlineLevel="3">
       <c r="B397" s="17" t="s">
         <v>396</v>
       </c>
       <c r="C397" s="11" t="n">
-        <v>265</v>
+        <v>157</v>
       </c>
     </row>
     <row r="398" ht="11" customHeight="true" outlineLevel="3">
@@ -4696,7 +4741,7 @@
         <v>397</v>
       </c>
       <c r="C398" s="11" t="n">
-        <v>204</v>
+        <v>330</v>
       </c>
     </row>
     <row r="399" ht="11" customHeight="true" outlineLevel="3">
@@ -4704,31 +4749,31 @@
         <v>398</v>
       </c>
       <c r="C399" s="11" t="n">
-        <v>442</v>
-      </c>
-    </row>
-    <row r="400" ht="11" customHeight="true" outlineLevel="3">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="400" ht="22" customHeight="true" outlineLevel="3">
       <c r="B400" s="17" t="s">
         <v>399</v>
       </c>
       <c r="C400" s="11" t="n">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="401" ht="11" customHeight="true" outlineLevel="3">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="401" ht="22" customHeight="true" outlineLevel="3">
       <c r="B401" s="17" t="s">
         <v>400</v>
       </c>
-      <c r="C401" s="18" t="n">
-        <v>2338</v>
-      </c>
-    </row>
-    <row r="402" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C401" s="11" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="402" ht="22" customHeight="true" outlineLevel="3">
       <c r="B402" s="17" t="s">
         <v>401</v>
       </c>
       <c r="C402" s="11" t="n">
-        <v>660</v>
+        <v>6</v>
       </c>
     </row>
     <row r="403" ht="22" customHeight="true" outlineLevel="3">
@@ -4736,15 +4781,15 @@
         <v>402</v>
       </c>
       <c r="C403" s="11" t="n">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="404" ht="11" customHeight="true" outlineLevel="3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="404" ht="22" customHeight="true" outlineLevel="3">
       <c r="B404" s="17" t="s">
         <v>403</v>
       </c>
       <c r="C404" s="11" t="n">
-        <v>642</v>
+        <v>76</v>
       </c>
     </row>
     <row r="405" ht="22" customHeight="true" outlineLevel="3">
@@ -4752,47 +4797,47 @@
         <v>404</v>
       </c>
       <c r="C405" s="11" t="n">
-        <v>480</v>
+        <v>42</v>
       </c>
     </row>
     <row r="406" ht="22" customHeight="true" outlineLevel="3">
       <c r="B406" s="17" t="s">
         <v>405</v>
       </c>
-      <c r="C406" s="18" t="n">
-        <v>2173</v>
-      </c>
-    </row>
-    <row r="407" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C406" s="11" t="n">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="407" ht="22" customHeight="true" outlineLevel="3">
       <c r="B407" s="17" t="s">
         <v>406</v>
       </c>
       <c r="C407" s="11" t="n">
-        <v>707</v>
-      </c>
-    </row>
-    <row r="408" ht="22" customHeight="true" outlineLevel="3">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="408" ht="11" customHeight="true" outlineLevel="3">
       <c r="B408" s="17" t="s">
         <v>407</v>
       </c>
       <c r="C408" s="11" t="n">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="409" ht="22" customHeight="true" outlineLevel="3">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="409" ht="11" customHeight="true" outlineLevel="3">
       <c r="B409" s="17" t="s">
         <v>408</v>
       </c>
-      <c r="C409" s="18" t="n">
-        <v>1360</v>
-      </c>
-    </row>
-    <row r="410" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C409" s="11" t="n">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="410" ht="22" customHeight="true" outlineLevel="3">
       <c r="B410" s="17" t="s">
         <v>409</v>
       </c>
       <c r="C410" s="11" t="n">
-        <v>48</v>
+        <v>4</v>
       </c>
     </row>
     <row r="411" ht="11" customHeight="true" outlineLevel="3">
@@ -4800,15 +4845,15 @@
         <v>410</v>
       </c>
       <c r="C411" s="11" t="n">
-        <v>645</v>
-      </c>
-    </row>
-    <row r="412" ht="11" customHeight="true" outlineLevel="3">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="412" ht="22" customHeight="true" outlineLevel="3">
       <c r="B412" s="17" t="s">
         <v>411</v>
       </c>
       <c r="C412" s="11" t="n">
-        <v>735</v>
+        <v>488</v>
       </c>
     </row>
     <row r="413" ht="11" customHeight="true" outlineLevel="3">
@@ -4816,15 +4861,15 @@
         <v>412</v>
       </c>
       <c r="C413" s="11" t="n">
-        <v>23</v>
+        <v>381</v>
       </c>
     </row>
     <row r="414" ht="11" customHeight="true" outlineLevel="3">
       <c r="B414" s="17" t="s">
         <v>413</v>
       </c>
-      <c r="C414" s="18" t="n">
-        <v>1868</v>
+      <c r="C414" s="11" t="n">
+        <v>493</v>
       </c>
     </row>
     <row r="415" ht="11" customHeight="true" outlineLevel="3">
@@ -4832,7 +4877,7 @@
         <v>414</v>
       </c>
       <c r="C415" s="11" t="n">
-        <v>385</v>
+        <v>35</v>
       </c>
     </row>
     <row r="416" ht="11" customHeight="true" outlineLevel="3">
@@ -4840,46 +4885,166 @@
         <v>415</v>
       </c>
       <c r="C416" s="11" t="n">
-        <v>324</v>
+        <v>11</v>
       </c>
     </row>
     <row r="417" ht="11" customHeight="true" outlineLevel="3">
       <c r="B417" s="17" t="s">
         <v>416</v>
       </c>
-      <c r="C417" s="18" t="n">
-        <v>2317</v>
-      </c>
-    </row>
-    <row r="418" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C417" s="11" t="n">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="418" ht="22" customHeight="true" outlineLevel="3">
       <c r="B418" s="17" t="s">
         <v>417</v>
       </c>
-      <c r="C418" s="18" t="n">
-        <v>1490</v>
-      </c>
-    </row>
-    <row r="419" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C418" s="11" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="419" ht="11" customHeight="true" outlineLevel="3">
       <c r="B419" s="17" t="s">
         <v>418</v>
       </c>
       <c r="C419" s="11" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="420" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B420" s="19" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="420" ht="22" customHeight="true" outlineLevel="3">
+      <c r="B420" s="17" t="s">
         <v>419</v>
       </c>
-      <c r="C420" s="14" t="n">
+      <c r="C420" s="11" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="421" ht="22" customHeight="true" outlineLevel="3">
+      <c r="B421" s="17" t="s">
+        <v>420</v>
+      </c>
+      <c r="C421" s="18" t="n">
+        <v>1755</v>
+      </c>
+    </row>
+    <row r="422" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B422" s="17" t="s">
+        <v>421</v>
+      </c>
+      <c r="C422" s="11" t="n">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="423" ht="22" customHeight="true" outlineLevel="3">
+      <c r="B423" s="17" t="s">
+        <v>422</v>
+      </c>
+      <c r="C423" s="11" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="424" ht="22" customHeight="true" outlineLevel="3">
+      <c r="B424" s="17" t="s">
+        <v>423</v>
+      </c>
+      <c r="C424" s="11" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="425" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B425" s="17" t="s">
+        <v>424</v>
+      </c>
+      <c r="C425" s="11" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="426" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B426" s="17" t="s">
+        <v>425</v>
+      </c>
+      <c r="C426" s="11" t="n">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="427" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B427" s="17" t="s">
+        <v>426</v>
+      </c>
+      <c r="C427" s="11" t="n">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="428" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B428" s="17" t="s">
+        <v>427</v>
+      </c>
+      <c r="C428" s="18" t="n">
+        <v>1264</v>
+      </c>
+    </row>
+    <row r="429" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B429" s="17" t="s">
+        <v>428</v>
+      </c>
+      <c r="C429" s="11" t="n">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="430" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B430" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="C430" s="11" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="431" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B431" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="C431" s="11" t="n">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="432" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B432" s="17" t="s">
+        <v>431</v>
+      </c>
+      <c r="C432" s="11" t="n">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="433" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B433" s="17" t="s">
+        <v>432</v>
+      </c>
+      <c r="C433" s="11" t="n">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="434" ht="22" customHeight="true" outlineLevel="3">
+      <c r="B434" s="17" t="s">
+        <v>433</v>
+      </c>
+      <c r="C434" s="11" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="435" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B435" s="19" t="s">
+        <v>434</v>
+      </c>
+      <c r="C435" s="14" t="n">
         <v>105</v>
       </c>
     </row>
-    <row r="421" ht="11" customHeight="true" outlineLevel="4">
-      <c r="B421" s="20" t="s">
-        <v>420</v>
-      </c>
-      <c r="C421" s="11" t="n">
+    <row r="436" ht="11" customHeight="true" outlineLevel="4">
+      <c r="B436" s="20" t="s">
+        <v>435</v>
+      </c>
+      <c r="C436" s="11" t="n">
         <v>105</v>
       </c>
     </row>

</xml_diff>

<commit_message>
befor change doc sign
</commit_message>
<xml_diff>
--- a/client/public/Sorce/balanceDP.xlsx
+++ b/client/public/Sorce/balanceDP.xlsx
@@ -14,12 +14,12 @@
 </file>
 
 <file path=xl/SharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="446">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="452">
   <si>
     <t>Формирвоание отчета</t>
   </si>
   <si>
-    <t>Период: на 16.02.2026 7:55:13</t>
+    <t>Период: на 23.02.2026 11:15:12</t>
   </si>
   <si>
     <t>Показатели: Свободный остаток(В ед. хранения);</t>
@@ -92,6 +92,9 @@
     <t>Желе вишня УБ 78г /56шт</t>
   </si>
   <si>
+    <t>Желе вишня УБ 78г /56шт АКЦІЯ ВІП</t>
+  </si>
+  <si>
     <t>Желе вишня УБ 78г /56шт АКЦІЯ ОПТ</t>
   </si>
   <si>
@@ -101,6 +104,9 @@
     <t>Желе ківі УБ 78г /56шт АКЦІЯ</t>
   </si>
   <si>
+    <t>Желе ківі УБ 78г /56шт АКЦІЯ ВІП</t>
+  </si>
+  <si>
     <t>Желе ківі УБ 78г /56шт АКЦІЯ ОПТ</t>
   </si>
   <si>
@@ -110,9 +116,6 @@
     <t>Желе Лісова ягода УБ 78г /56шт АКЦІЯ ВІП</t>
   </si>
   <si>
-    <t>Желе Лісова ягода УБ 78г /56шт АКЦІЯ ОПТ</t>
-  </si>
-  <si>
     <t>Желе полуниця УБ 78г /56шт</t>
   </si>
   <si>
@@ -194,6 +197,9 @@
     <t>Приправа до картоплі УБ 25г /34шт АКЦІЯ ВІП</t>
   </si>
   <si>
+    <t>Приправа до курки УБ 25г /34шт</t>
+  </si>
+  <si>
     <t>Приправа до курки УБ 25г /34шт АКЦІЯ ВІП</t>
   </si>
   <si>
@@ -323,45 +329,48 @@
     <t>Батон ROSHEN "Double peanuts" мол-шок з арахісом та арахісовим кремом ВКФ 39г /180шт /</t>
   </si>
   <si>
+    <t>Батон ROSHEN "Double peanuts" мол-шок з арахісом та арахісовим кремом ВКФ 39г /180шт /АКЦІЯ ВІП</t>
+  </si>
+  <si>
+    <t>Батон ROSHEN "Double peanuts" мол-шок з арахісом та арахісовим кремом ВКФ 39г /180шт /АКЦІЯ ОПТ</t>
+  </si>
+  <si>
     <t>Батон ROSHEN "Double peanuts" мол-шок з арахісом та арахісовим кремом ВКФ 39г /180шт UA TP</t>
   </si>
   <si>
     <t>Батон ROSHEN з начинкою ВКФ 43г /180шт /</t>
   </si>
   <si>
+    <t>Батон ROSHEN з начинкою ВКФ 43г /180шт /АКЦІЯ ВІП</t>
+  </si>
+  <si>
     <t>Батон ROSHEN з начинкою ВКФ 43г /180шт /АКЦІЯ ОПТ</t>
   </si>
   <si>
-    <t>Батон ROSHEN з начинкою ВКФ 43г /180шт /АКЦІЯ Цінова</t>
-  </si>
-  <si>
-    <t>Батон ROSHEN з начинкою ВКФ 43г /180шт /АКЦІЯ Цінова накладна</t>
-  </si>
-  <si>
-    <t>Батон ROSHEN мол-шок з карамельною начинкою ВКФ 40г /180шт /</t>
-  </si>
-  <si>
     <t>Батон ROSHEN мол-шок з карамельною начинкою ВКФ 40г /180шт /АКЦІЯ ОПТ</t>
   </si>
   <si>
-    <t>Батон ROSHEN мол-шок з карамельною начинкою ВКФ 40г /180шт /АКЦІЯ Цінова</t>
-  </si>
-  <si>
     <t>Батон ROSHEN мол-шок з кокосом та мигдалем ВКФ 38г /180шт /</t>
   </si>
   <si>
+    <t>Батон ROSHEN мол-шок з кокосом та мигдалем ВКФ 38г /180шт /АКЦІЯ ВІП</t>
+  </si>
+  <si>
+    <t>Батон ROSHEN мол-шок з кокосом та мигдалем ВКФ 38г /180шт /АКЦІЯ ОПТ</t>
+  </si>
+  <si>
     <t>Батон ROSHEN мол-шок з кокосом та мигдалем ВКФ 38г /180шт UA TP</t>
   </si>
   <si>
     <t>Батон ROSHEN мол-шок з кокосом та мигдалем ВКФ 38г /180шт UA TP АКЦІЯ ОПТ</t>
   </si>
   <si>
-    <t>Батон ROSHEN молочно-шоколадний з арахісовою начинкою ВКФ 38г /180шт /АКЦІЯ Цінова</t>
-  </si>
-  <si>
     <t>Батон ROSHEN молочно-шоколадний з арахісовою начинкою ВКФ 38г /180шт UA TP</t>
   </si>
   <si>
+    <t>Батон ROSHEN молочно-шоколадний з арахісовою начинкою ВКФ 38г /180шт UA TP АКЦІЯ ВІП</t>
+  </si>
+  <si>
     <t>Батон ROSHEN молочно-шоколадний з арахісовою начинкою ВКФ 38г /180шт UA TP АКЦІЯ ОПТ</t>
   </si>
   <si>
@@ -383,9 +392,6 @@
     <t>Бісквіт Рошен П'янка вишня ВКФ 300г /9шт</t>
   </si>
   <si>
-    <t>Бісквіт Рошен Празький ВКФ 300г /9шт</t>
-  </si>
-  <si>
     <t>РУЛЕТ Золотий ключик ВКФ 180г /14шт</t>
   </si>
   <si>
@@ -413,9 +419,6 @@
     <t>Konafetto з ванільною начинкою ВКФ 140г /15шт</t>
   </si>
   <si>
-    <t>Konafetto з горіховою начинкою ВКФ 140г /15шт</t>
-  </si>
-  <si>
     <t>Konafetto з горіховою начинкою ВКФ 140г /15шт АКЦІЯ ВІП 1</t>
   </si>
   <si>
@@ -425,6 +428,9 @@
     <t>Konafetto з молочною начинкою ВКФ 140г /15шт</t>
   </si>
   <si>
+    <t>KONAFETTO з молочною начинкою ВКФ 140г /15шт DE</t>
+  </si>
+  <si>
     <t>Roshetto dark ВКФ 34г /200шт</t>
   </si>
   <si>
@@ -446,15 +452,9 @@
     <t>Wafers Sandwich Crunch горіх ККФ 142г /15шт /</t>
   </si>
   <si>
-    <t>Wafers Sandwich Crunch горіх ККФ 142г /15шт АКЦІЯ Цінова</t>
-  </si>
-  <si>
     <t>Wafers Sandwich Crunch какао ККФ 142г /15шт /</t>
   </si>
   <si>
-    <t>Wafers Sandwich Crunch какао ККФ 142г /15шт АКЦІЯ Цінова</t>
-  </si>
-  <si>
     <t>Wafers Sandwich Crunch лимон ККФ 142г /15шт /</t>
   </si>
   <si>
@@ -479,9 +479,6 @@
     <t>Wafers какао ККФ 216г /16шт</t>
   </si>
   <si>
-    <t>Wafers какао ККФ 216г /16шт АКЦІЯ Цінова</t>
-  </si>
-  <si>
     <t>Wafers какао ККФ 72г /22шт AR /</t>
   </si>
   <si>
@@ -527,9 +524,6 @@
     <t>Korivka Roshen 205г/12</t>
   </si>
   <si>
-    <t>Korivka Roshen ВКФ 205г /12шт EU АКЦІЯ ВІП</t>
-  </si>
-  <si>
     <t>Milky Splash РЦ 150г /12пак</t>
   </si>
   <si>
@@ -563,15 +557,9 @@
     <t>Yummi Gummi Cherry ВКФ 70г /22шт</t>
   </si>
   <si>
-    <t>Yummi Gummi Cherry ВКФ 70г /22шт АКЦІЯ Цінова</t>
-  </si>
-  <si>
     <t>Yummi Gummi CupCakes ВКФ 70г /22шт</t>
   </si>
   <si>
-    <t>Yummi Gummi CupCakes ВКФ 70г /22шт АКЦІЯ Цінова</t>
-  </si>
-  <si>
     <t>Yummi Gummi Daydream ВКФ 70г /22шт</t>
   </si>
   <si>
@@ -584,6 +572,9 @@
     <t>Yummi Gummi Duo Mix ВКФ 70г /22шт</t>
   </si>
   <si>
+    <t>Yummi Gummi Duo Mix ВКФ 70г /22шт АКЦІЯ Цінова</t>
+  </si>
+  <si>
     <t>Yummi Gummi Fizzy Worms ВКФ 70г /22шт</t>
   </si>
   <si>
@@ -605,18 +596,15 @@
     <t>Yummi Gummi Fluffi Rainbow Turbines ВКФ 65г /11шт АКЦІЯ Цінова</t>
   </si>
   <si>
-    <t>Yummi Gummi Fluffi Rainbow Turbines ВКФ 65г /11шт АКЦІЯ Цінова UA</t>
-  </si>
-  <si>
     <t>Yummi Gummi Fluffi Rainbow Turbines ВКФ 65г /11шт АКЦІЯ Цінова накладна</t>
   </si>
   <si>
+    <t>Yummi Gummi Fluffi Soft Hearts ВКФ 65г /11шт</t>
+  </si>
+  <si>
     <t>Yummi Gummi Fluffi Soft Hearts ВКФ 65г /11шт АКЦІЯ Цінова</t>
   </si>
   <si>
-    <t>Yummi Gummi Fluffi Soft Hearts ВКФ 65г /11шт АКЦІЯ Цінова UA</t>
-  </si>
-  <si>
     <t>Yummi Gummi Fluffi Soft Hearts ВКФ 65г /11шт АКЦІЯ Цінова накладна</t>
   </si>
   <si>
@@ -638,6 +626,9 @@
     <t>Yummi Gummi Frozen Yogo ВКФ 70г /22шт</t>
   </si>
   <si>
+    <t>Yummi Gummi Frozen Yogo ВКФ 70г /22шт АКЦІЯ Цінова</t>
+  </si>
+  <si>
     <t>Yummi Gummi Funny Cola ВКФ 70г /22шт</t>
   </si>
   <si>
@@ -671,6 +662,9 @@
     <t>Yummi Gummi Smile Mix ВКФ 70г /22шт</t>
   </si>
   <si>
+    <t>Yummi Gummi Smile Mix ВКФ 70г /22шт АКЦІЯ Цінова</t>
+  </si>
+  <si>
     <t>Yummi Gummi Sour Belts ВКФ 70г /40шт</t>
   </si>
   <si>
@@ -683,6 +677,9 @@
     <t>Yummi Gummi Sour Sticks ВКФ 70г /40шт</t>
   </si>
   <si>
+    <t>Yummi Gummi Sour Sticks ВКФ 70г /40шт АКЦІЯ Цінова</t>
+  </si>
+  <si>
     <t>Yummi Gummi Sour Strawberries ВКФ 70г /22шт</t>
   </si>
   <si>
@@ -692,6 +689,9 @@
     <t>Yummi Gummi Twists ВКФ 70г /40шт</t>
   </si>
   <si>
+    <t>Yummi Gummi Twists ВКФ 70г /40шт АКЦІЯ Цінова</t>
+  </si>
+  <si>
     <t>Yummi Gummi Watermelon Slices ВКФ 70г /22шт</t>
   </si>
   <si>
@@ -848,12 +848,6 @@
     <t>Assortment Elegant ВКФ 145г /8шт АКЦІЯ ВІП</t>
   </si>
   <si>
-    <t>Cherry Queen heart РЦ 122г /8шт</t>
-  </si>
-  <si>
-    <t>Cherry Queen heart РЦ 122г /8шт АКЦІЯ ВІП</t>
-  </si>
-  <si>
     <t>Chocolateria ВКФ 194г /8шт NEW</t>
   </si>
   <si>
@@ -965,6 +959,9 @@
     <t>Lovita Jelly Cookies з желейною начинкою зі смаком полуниці ККФ 135г /21шт /</t>
   </si>
   <si>
+    <t>Lovita Jelly Cookies з желейною начинкою зі смаком полуниці ККФ 420г /7шт</t>
+  </si>
+  <si>
     <t>Lovita Jelly Cookies з желейною начинкою какао + вишня ККФ 135г /21шт /</t>
   </si>
   <si>
@@ -992,9 +989,15 @@
     <t>Multicake з начинкою кокос-крем ККФ 180г /28шт FP</t>
   </si>
   <si>
+    <t>Multicake з начинкою кокос-крем ККФ 180г /28шт FP DE</t>
+  </si>
+  <si>
     <t>Multicake з начинкою лимон-крем ККФ 180г /28шт FP</t>
   </si>
   <si>
+    <t>Multicake з начинкою лимон-крем ККФ 180г /28шт FP DE</t>
+  </si>
+  <si>
     <t>Multicake з начинкою полуниця-крем ККФ 180г /28шт FP</t>
   </si>
   <si>
@@ -1067,9 +1070,6 @@
     <t>KONAFETTO blanc ККФ 1кг /5пак HAL</t>
   </si>
   <si>
-    <t>KONAFETTO nero ККФ 1кг /5пак /</t>
-  </si>
-  <si>
     <t>KONAFETTO nero ККФ 1кг /5пак HAL</t>
   </si>
   <si>
@@ -1100,12 +1100,6 @@
     <t>Монблан з карамелізованим мигдалем ВКФ 1кг /4пак</t>
   </si>
   <si>
-    <t>Монблан з карамелізованим мигдалем ВКФ 1кг /4пак ЗНИЖКА ДИСТР</t>
-  </si>
-  <si>
-    <t>Монблан з мигдалем та кокосовим кремом ВКФ 1кг /4пак ЗНИЖКА ДИСТР</t>
-  </si>
-  <si>
     <t>Монблан з подр. мигдалем та кокосовим кремом ВКФ 1кг /4пак</t>
   </si>
   <si>
@@ -1175,9 +1169,6 @@
     <t>ШОКОЛАД</t>
   </si>
   <si>
-    <t>Lacmi Big Bite молочний ВКФ 200г /17шт</t>
-  </si>
-  <si>
     <t>Lacmi Big Bite молочний ВКФ 260г /15шт /АКЦІЯ ВІП 1</t>
   </si>
   <si>
@@ -1187,6 +1178,12 @@
     <t>Lacmi Black, White &amp; Caramel молочний з молочною начинкою, карамеллю та печивом з какао ВКФ 100г /18шт</t>
   </si>
   <si>
+    <t>Lacmi Black, White &amp; Caramel молочний з молочною начинкою, карамеллю та печивом з какао ВКФ 100г /18шт АКЦІЯ ВІП</t>
+  </si>
+  <si>
+    <t>Lacmi Black, White &amp; Caramel молочний з молочною начинкою, карамеллю та печивом з какао ВКФ 100г /18шт АКЦІЯ ОПТ</t>
+  </si>
+  <si>
     <t>Lacmi Cool-Nut-Coconut молочний з мигдалем та кокосом ВКФ 280г /12шт</t>
   </si>
   <si>
@@ -1202,9 +1199,6 @@
     <t>Lacmi Fun&amp;Crispy молочний пористий з молочною начинкою з кріспі ВКФ 85г /17шт АКЦІЯ ОПТ</t>
   </si>
   <si>
-    <t>Lacmi Fun&amp;Crispy молочний пористий з молочною начинкою з кріспі ВКФ 85г /17шт АКЦІЯ Цінова</t>
-  </si>
-  <si>
     <t>Lacmi молочний Strawberry cake ВКФ 275г /12шт</t>
   </si>
   <si>
@@ -1214,12 +1208,18 @@
     <t>Lacmi молочний ВКФ 90г /22шт</t>
   </si>
   <si>
+    <t>Lacmi молочний ВКФ 90г /22шт АКЦІЯ ВІП 1</t>
+  </si>
+  <si>
     <t>Lacmi молочний ВКФ 90г /22шт АКЦІЯ ОПТ</t>
   </si>
   <si>
     <t>Lacmi молочний з арахісом і карамельно-арахісовою начинкою ВКФ 295г /12шт</t>
   </si>
   <si>
+    <t>Lacmi молочний з арахісом і карамельно-арахісовою начинкою ВКФ 295г /12шт АКЦІЯ ВІП</t>
+  </si>
+  <si>
     <t>Lacmi молочний з арахісом і карамельно-арахісовою начинкою ВКФ 295г /12шт АКЦІЯ ОПТ</t>
   </si>
   <si>
@@ -1229,39 +1229,42 @@
     <t>Lacmi молочний з арахісом, карамельною та арахісовою начинками ВКФ 87г /22шт UA TP</t>
   </si>
   <si>
+    <t>Lacmi молочний з арахісом, карамельною та арахісовою начинками ВКФ 87г /22шт АКЦІЯ ВІП</t>
+  </si>
+  <si>
     <t>Lacmi молочний з арахісом, карамельною та арахісовою начинками ВКФ 87г /22шт АКЦІЯ ОПТ</t>
   </si>
   <si>
     <t>Lacmi молочний з мигдалем та кокосовим кремом ВКФ 84г /22шт</t>
   </si>
   <si>
+    <t>Lacmi молочний з мигдалем та кокосовим кремом ВКФ 84г /22шт АКЦІЯ ОПТ</t>
+  </si>
+  <si>
     <t>Lacmi молочний з молочною начинкою та вафлею ВКФ 90г /18шт</t>
   </si>
   <si>
     <t>Lacmi молочний з молочною начинкою та вафлею ВКФ 90г /18шт UA TP</t>
   </si>
   <si>
-    <t>Lacmi молочний з молочною начинкою та вафлею ВКФ 90г /18шт АКЦІЯ ОПТ</t>
-  </si>
-  <si>
-    <t>Lacmi молочний з молочною начинкою та печивом ВКФ 100г /18шт</t>
-  </si>
-  <si>
-    <t>Lacmi молочний з молочною начинкою та печивом ВКФ 100г /18шт UA TP</t>
-  </si>
-  <si>
-    <t>Lacmi молочний з молочною начинкою та печивом ВКФ 100г /18шт АКЦІЯ ОПТ</t>
+    <t>Lacmi молочний з молочною начинкою та вафлею ВКФ 90г /18шт АКЦІЯ ВІП</t>
   </si>
   <si>
     <t>Lacmi молочний з молочною та шоколадною начинками, вафлею з какао ВКФ 235г /12шт</t>
   </si>
   <si>
+    <t>Lacmi молочний з молочною та шоколадною начинками, вафлею з какао ВКФ 235г /12шт АКЦІЯ ВІП</t>
+  </si>
+  <si>
     <t>Lacmi молочний з молочною та шоколадною начинками, вафлею з какао ВКФ 235г /12шт АКЦІЯ ОПТ</t>
   </si>
   <si>
     <t>Lacmi молочний з начинкою зі смаком "Полунична панакота" ВКФ 90г /22шт</t>
   </si>
   <si>
+    <t>Lacmi молочний з начинкою зі смаком "Полунична панакота" ВКФ 90г /22шт АКЦІЯ ОПТ</t>
+  </si>
+  <si>
     <t>Lacmi молочний з начинкою зі смаком "Тірамісу" та печивом ВКФ 270г /12шт</t>
   </si>
   <si>
@@ -1289,6 +1292,9 @@
     <t>Lacmi молочний з шоколадно-горіховою начинкою та печивом ВКФ 265г /12шт UA TP</t>
   </si>
   <si>
+    <t>Lacmi молочний з шоколадно-горіховою начинкою та печивом ВКФ 265г /12шт АКЦІЯ ВІП</t>
+  </si>
+  <si>
     <t>Lacmi молочний з шоколадно-горіховою начинкою та печивом ВКФ 265г /12шт АКЦІЯ ОПТ</t>
   </si>
   <si>
@@ -1304,27 +1310,33 @@
     <t>Roshen Nut молочний з цілим мигдалем ВКФ 90г /20шт</t>
   </si>
   <si>
+    <t>Roshen Nut молочний з цілим мигдалем ВКФ 90г /20шт АКЦІЯ Цінова UA</t>
+  </si>
+  <si>
     <t>Roshen Nut молочний з цілим фундуком ВКФ 90г /18шт</t>
   </si>
   <si>
     <t>Roshen Nut молочний з цілим фундуком ВКФ 90г /18шт АКЦІЯ Цінова</t>
   </si>
   <si>
+    <t>Roshen Nut чорний з цілим мигдалем ВКФ 90г /20шт</t>
+  </si>
+  <si>
     <t>Roshen Nut чорний з цілим фундуком ВКФ 90г /18шт</t>
   </si>
   <si>
     <t>Roshen пористий БІЛИЙ ВКФ 80г /20шт Aerated UA</t>
   </si>
   <si>
-    <t>Roshen пористий БІЛИЙ ВКФ 80г /20шт FP АКЦІЯ Цінова UA</t>
-  </si>
-  <si>
-    <t>Roshen пористий білий карамельний ВКФ 80г /20шт Aerated UA</t>
+    <t>Roshen пористий БІЛИЙ ВКФ 80г /20шт Aerated АКЦІЯ Цінова</t>
   </si>
   <si>
     <t>Roshen пористий екстрачорний ВКФ 80г /20шт Aerated UA</t>
   </si>
   <si>
+    <t>Roshen пористий екстрачорний ВКФ 80г /20шт Aerated UA АКЦІЯ ОПТ</t>
+  </si>
+  <si>
     <t>Roshen пористий екстрачорний ВКФ 80г /20шт Aerated АКЦІЯ Цінова</t>
   </si>
   <si>
@@ -1340,7 +1352,13 @@
     <t>Roshen чорний Bitter 80% ВКФ 85г /35шт</t>
   </si>
   <si>
+    <t>Roshen чорний Bitter 80% ВКФ 85г /35шт АКЦІЯ ОПТ</t>
+  </si>
+  <si>
     <t>Roshen чорний Special 56% ВКФ 85г /35шт /</t>
+  </si>
+  <si>
+    <t>Roshen чорний Special 56% ВКФ 85г /35шт /АКЦІЯ ОПТ</t>
   </si>
   <si>
     <t>Roshen чорний з підсоленим подрібн. мигдалем ВКФ 85г /35шт /</t>
@@ -1604,7 +1622,7 @@
     <outlinePr summaryBelow="false" summaryRight="false"/>
     <pageSetUpPr autoPageBreaks="false"/>
   </sheetPr>
-  <dimension ref="C446"/>
+  <dimension ref="C452"/>
   <sheetFormatPr defaultColWidth="10.5" customHeight="true" defaultRowHeight="11.429"/>
   <cols>
     <col min="1" max="1" width="2.33203125" style="1" customWidth="true"/>
@@ -1669,7 +1687,7 @@
         <v>10</v>
       </c>
       <c r="C11" s="11" t="n">
-        <v>511</v>
+        <v>628</v>
       </c>
     </row>
     <row r="12" ht="11" customHeight="true">
@@ -1677,7 +1695,7 @@
         <v>11</v>
       </c>
       <c r="C12" s="12" t="n">
-        <v>916750</v>
+        <v>977289</v>
       </c>
     </row>
     <row r="13" ht="11" customHeight="true" outlineLevel="1">
@@ -1701,7 +1719,7 @@
         <v>14</v>
       </c>
       <c r="C15" s="12" t="n">
-        <v>241183</v>
+        <v>267889</v>
       </c>
     </row>
     <row r="16" ht="11" customHeight="true" outlineLevel="2">
@@ -1709,7 +1727,7 @@
         <v>15</v>
       </c>
       <c r="C16" s="12" t="n">
-        <v>35004</v>
+        <v>21453</v>
       </c>
     </row>
     <row r="17" ht="11" customHeight="true" outlineLevel="3">
@@ -1717,15 +1735,15 @@
         <v>16</v>
       </c>
       <c r="C17" s="18" t="n">
-        <v>2347</v>
+        <v>1727</v>
       </c>
     </row>
     <row r="18" ht="11" customHeight="true" outlineLevel="3">
       <c r="B18" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="C18" s="18" t="n">
-        <v>1237</v>
+      <c r="C18" s="11" t="n">
+        <v>907</v>
       </c>
     </row>
     <row r="19" ht="11" customHeight="true" outlineLevel="3">
@@ -1733,7 +1751,7 @@
         <v>18</v>
       </c>
       <c r="C19" s="18" t="n">
-        <v>4193</v>
+        <v>2681</v>
       </c>
     </row>
     <row r="20" ht="11" customHeight="true" outlineLevel="3">
@@ -1741,7 +1759,7 @@
         <v>19</v>
       </c>
       <c r="C20" s="11" t="n">
-        <v>108</v>
+        <v>724</v>
       </c>
     </row>
     <row r="21" ht="11" customHeight="true" outlineLevel="3">
@@ -1756,16 +1774,16 @@
       <c r="B22" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="C22" s="18" t="n">
-        <v>3682</v>
+      <c r="C22" s="11" t="n">
+        <v>206</v>
       </c>
     </row>
     <row r="23" ht="11" customHeight="true" outlineLevel="3">
       <c r="B23" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="C23" s="11" t="n">
-        <v>364</v>
+      <c r="C23" s="18" t="n">
+        <v>1484</v>
       </c>
     </row>
     <row r="24" ht="11" customHeight="true" outlineLevel="3">
@@ -1773,7 +1791,7 @@
         <v>23</v>
       </c>
       <c r="C24" s="18" t="n">
-        <v>5296</v>
+        <v>2863</v>
       </c>
     </row>
     <row r="25" ht="11" customHeight="true" outlineLevel="3">
@@ -1781,23 +1799,23 @@
         <v>24</v>
       </c>
       <c r="C25" s="11" t="n">
-        <v>201</v>
+        <v>896</v>
       </c>
     </row>
     <row r="26" ht="11" customHeight="true" outlineLevel="3">
       <c r="B26" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="C26" s="18" t="n">
-        <v>5064</v>
+      <c r="C26" s="11" t="n">
+        <v>89</v>
       </c>
     </row>
     <row r="27" ht="11" customHeight="true" outlineLevel="3">
       <c r="B27" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="C27" s="11" t="n">
-        <v>36</v>
+      <c r="C27" s="18" t="n">
+        <v>2738</v>
       </c>
     </row>
     <row r="28" ht="11" customHeight="true" outlineLevel="3">
@@ -1805,7 +1823,7 @@
         <v>27</v>
       </c>
       <c r="C28" s="11" t="n">
-        <v>136</v>
+        <v>36</v>
       </c>
     </row>
     <row r="29" ht="11" customHeight="true" outlineLevel="3">
@@ -1813,7 +1831,7 @@
         <v>28</v>
       </c>
       <c r="C29" s="18" t="n">
-        <v>2826</v>
+        <v>1008</v>
       </c>
     </row>
     <row r="30" ht="11" customHeight="true" outlineLevel="3">
@@ -1821,7 +1839,7 @@
         <v>29</v>
       </c>
       <c r="C30" s="11" t="n">
-        <v>812</v>
+        <v>24</v>
       </c>
     </row>
     <row r="31" ht="11" customHeight="true" outlineLevel="3">
@@ -1829,7 +1847,7 @@
         <v>30</v>
       </c>
       <c r="C31" s="11" t="n">
-        <v>39</v>
+        <v>155</v>
       </c>
     </row>
     <row r="32" ht="11" customHeight="true" outlineLevel="3">
@@ -1837,7 +1855,7 @@
         <v>31</v>
       </c>
       <c r="C32" s="18" t="n">
-        <v>2801</v>
+        <v>1372</v>
       </c>
     </row>
     <row r="33" ht="11" customHeight="true" outlineLevel="3">
@@ -1845,7 +1863,7 @@
         <v>32</v>
       </c>
       <c r="C33" s="11" t="n">
-        <v>196</v>
+        <v>292</v>
       </c>
     </row>
     <row r="34" ht="11" customHeight="true" outlineLevel="3">
@@ -1853,7 +1871,7 @@
         <v>33</v>
       </c>
       <c r="C34" s="18" t="n">
-        <v>1322</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="35" ht="11" customHeight="true" outlineLevel="3">
@@ -1861,23 +1879,23 @@
         <v>34</v>
       </c>
       <c r="C35" s="18" t="n">
-        <v>4340</v>
-      </c>
-    </row>
-    <row r="36" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B36" s="16" t="s">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="36" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B36" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="C36" s="12" t="n">
-        <v>108314</v>
-      </c>
-    </row>
-    <row r="37" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B37" s="17" t="s">
+      <c r="C36" s="18" t="n">
+        <v>1985</v>
+      </c>
+    </row>
+    <row r="37" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B37" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="C37" s="18" t="n">
-        <v>7498</v>
+      <c r="C37" s="12" t="n">
+        <v>145597</v>
       </c>
     </row>
     <row r="38" ht="11" customHeight="true" outlineLevel="3">
@@ -1885,7 +1903,7 @@
         <v>37</v>
       </c>
       <c r="C38" s="18" t="n">
-        <v>69457</v>
+        <v>4339</v>
       </c>
     </row>
     <row r="39" ht="11" customHeight="true" outlineLevel="3">
@@ -1893,7 +1911,7 @@
         <v>38</v>
       </c>
       <c r="C39" s="18" t="n">
-        <v>2512</v>
+        <v>96921</v>
       </c>
     </row>
     <row r="40" ht="11" customHeight="true" outlineLevel="3">
@@ -1901,7 +1919,7 @@
         <v>39</v>
       </c>
       <c r="C40" s="18" t="n">
-        <v>4794</v>
+        <v>2213</v>
       </c>
     </row>
     <row r="41" ht="11" customHeight="true" outlineLevel="3">
@@ -1909,71 +1927,71 @@
         <v>40</v>
       </c>
       <c r="C41" s="18" t="n">
-        <v>14432</v>
+        <v>4794</v>
       </c>
     </row>
     <row r="42" ht="11" customHeight="true" outlineLevel="3">
       <c r="B42" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="C42" s="11" t="n">
-        <v>16</v>
+      <c r="C42" s="18" t="n">
+        <v>22427</v>
       </c>
     </row>
     <row r="43" ht="11" customHeight="true" outlineLevel="3">
       <c r="B43" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="C43" s="18" t="n">
-        <v>1710</v>
+      <c r="C43" s="11" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="44" ht="11" customHeight="true" outlineLevel="3">
       <c r="B44" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="C44" s="11" t="n">
-        <v>259</v>
+      <c r="C44" s="18" t="n">
+        <v>3292</v>
       </c>
     </row>
     <row r="45" ht="11" customHeight="true" outlineLevel="3">
       <c r="B45" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="C45" s="11" t="n">
-        <v>2</v>
+      <c r="C45" s="18" t="n">
+        <v>5349</v>
       </c>
     </row>
     <row r="46" ht="11" customHeight="true" outlineLevel="3">
       <c r="B46" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="C46" s="18" t="n">
-        <v>2462</v>
+      <c r="C46" s="11" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="47" ht="11" customHeight="true" outlineLevel="3">
       <c r="B47" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="C47" s="11" t="n">
-        <v>834</v>
-      </c>
-    </row>
-    <row r="48" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C47" s="18" t="n">
+        <v>2075</v>
+      </c>
+    </row>
+    <row r="48" ht="11" customHeight="true" outlineLevel="3">
       <c r="B48" s="17" t="s">
         <v>47</v>
       </c>
       <c r="C48" s="11" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="49" ht="11" customHeight="true" outlineLevel="3">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="true" outlineLevel="3">
       <c r="B49" s="17" t="s">
         <v>48</v>
       </c>
       <c r="C49" s="11" t="n">
-        <v>140</v>
+        <v>26</v>
       </c>
     </row>
     <row r="50" ht="11" customHeight="true" outlineLevel="3">
@@ -1981,63 +1999,63 @@
         <v>49</v>
       </c>
       <c r="C50" s="11" t="n">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="51" ht="11" customHeight="true" outlineLevel="3">
       <c r="B51" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="C51" s="18" t="n">
-        <v>2025</v>
-      </c>
-    </row>
-    <row r="52" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C51" s="11" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="52" ht="11" customHeight="true" outlineLevel="3">
       <c r="B52" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="C52" s="11" t="n">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="53" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C52" s="18" t="n">
+        <v>1640</v>
+      </c>
+    </row>
+    <row r="53" ht="22" customHeight="true" outlineLevel="3">
       <c r="B53" s="17" t="s">
         <v>52</v>
       </c>
       <c r="C53" s="11" t="n">
-        <v>10</v>
+        <v>44</v>
       </c>
     </row>
     <row r="54" ht="11" customHeight="true" outlineLevel="3">
       <c r="B54" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="C54" s="18" t="n">
-        <v>1856</v>
-      </c>
-    </row>
-    <row r="55" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C54" s="11" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="55" ht="11" customHeight="true" outlineLevel="3">
       <c r="B55" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="C55" s="11" t="n">
+      <c r="C55" s="18" t="n">
+        <v>1257</v>
+      </c>
+    </row>
+    <row r="56" ht="22" customHeight="true" outlineLevel="3">
+      <c r="B56" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="C56" s="11" t="n">
         <v>60</v>
       </c>
     </row>
-    <row r="56" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B56" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="C56" s="12" t="n">
-        <v>34417</v>
-      </c>
-    </row>
-    <row r="57" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B57" s="17" t="s">
+    <row r="57" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B57" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="C57" s="18" t="n">
-        <v>3319</v>
+      <c r="C57" s="12" t="n">
+        <v>43065</v>
       </c>
     </row>
     <row r="58" ht="11" customHeight="true" outlineLevel="3">
@@ -2045,7 +2063,7 @@
         <v>57</v>
       </c>
       <c r="C58" s="11" t="n">
-        <v>694</v>
+        <v>886</v>
       </c>
     </row>
     <row r="59" ht="11" customHeight="true" outlineLevel="3">
@@ -2053,15 +2071,15 @@
         <v>58</v>
       </c>
       <c r="C59" s="11" t="n">
-        <v>149</v>
+        <v>655</v>
       </c>
     </row>
     <row r="60" ht="11" customHeight="true" outlineLevel="3">
       <c r="B60" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="C60" s="11" t="n">
-        <v>36</v>
+      <c r="C60" s="18" t="n">
+        <v>1882</v>
       </c>
     </row>
     <row r="61" ht="11" customHeight="true" outlineLevel="3">
@@ -2069,15 +2087,15 @@
         <v>60</v>
       </c>
       <c r="C61" s="11" t="n">
-        <v>587</v>
+        <v>144</v>
       </c>
     </row>
     <row r="62" ht="11" customHeight="true" outlineLevel="3">
       <c r="B62" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="C62" s="11" t="n">
-        <v>443</v>
+      <c r="C62" s="18" t="n">
+        <v>2735</v>
       </c>
     </row>
     <row r="63" ht="11" customHeight="true" outlineLevel="3">
@@ -2085,15 +2103,15 @@
         <v>62</v>
       </c>
       <c r="C63" s="11" t="n">
-        <v>604</v>
+        <v>502</v>
       </c>
     </row>
     <row r="64" ht="11" customHeight="true" outlineLevel="3">
       <c r="B64" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="C64" s="11" t="n">
-        <v>449</v>
+      <c r="C64" s="18" t="n">
+        <v>3394</v>
       </c>
     </row>
     <row r="65" ht="11" customHeight="true" outlineLevel="3">
@@ -2101,15 +2119,15 @@
         <v>64</v>
       </c>
       <c r="C65" s="11" t="n">
-        <v>405</v>
+        <v>554</v>
       </c>
     </row>
     <row r="66" ht="11" customHeight="true" outlineLevel="3">
       <c r="B66" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="C66" s="11" t="n">
-        <v>738</v>
+      <c r="C66" s="18" t="n">
+        <v>2452</v>
       </c>
     </row>
     <row r="67" ht="11" customHeight="true" outlineLevel="3">
@@ -2117,15 +2135,15 @@
         <v>66</v>
       </c>
       <c r="C67" s="11" t="n">
-        <v>605</v>
+        <v>359</v>
       </c>
     </row>
     <row r="68" ht="11" customHeight="true" outlineLevel="3">
       <c r="B68" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="C68" s="18" t="n">
-        <v>1398</v>
+      <c r="C68" s="11" t="n">
+        <v>540</v>
       </c>
     </row>
     <row r="69" ht="11" customHeight="true" outlineLevel="3">
@@ -2133,7 +2151,7 @@
         <v>68</v>
       </c>
       <c r="C69" s="11" t="n">
-        <v>21</v>
+        <v>560</v>
       </c>
     </row>
     <row r="70" ht="11" customHeight="true" outlineLevel="3">
@@ -2141,7 +2159,7 @@
         <v>69</v>
       </c>
       <c r="C70" s="18" t="n">
-        <v>5040</v>
+        <v>3877</v>
       </c>
     </row>
     <row r="71" ht="11" customHeight="true" outlineLevel="3">
@@ -2149,23 +2167,23 @@
         <v>70</v>
       </c>
       <c r="C71" s="11" t="n">
-        <v>100</v>
+        <v>19</v>
       </c>
     </row>
     <row r="72" ht="11" customHeight="true" outlineLevel="3">
       <c r="B72" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="C72" s="11" t="n">
-        <v>894</v>
+      <c r="C72" s="18" t="n">
+        <v>4861</v>
       </c>
     </row>
     <row r="73" ht="11" customHeight="true" outlineLevel="3">
       <c r="B73" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="C73" s="18" t="n">
-        <v>3366</v>
+      <c r="C73" s="11" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="74" ht="11" customHeight="true" outlineLevel="3">
@@ -2173,15 +2191,15 @@
         <v>73</v>
       </c>
       <c r="C74" s="18" t="n">
-        <v>1325</v>
-      </c>
-    </row>
-    <row r="75" ht="22" customHeight="true" outlineLevel="3">
+        <v>1735</v>
+      </c>
+    </row>
+    <row r="75" ht="11" customHeight="true" outlineLevel="3">
       <c r="B75" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="C75" s="11" t="n">
-        <v>338</v>
+      <c r="C75" s="18" t="n">
+        <v>3084</v>
       </c>
     </row>
     <row r="76" ht="11" customHeight="true" outlineLevel="3">
@@ -2189,23 +2207,23 @@
         <v>75</v>
       </c>
       <c r="C76" s="18" t="n">
-        <v>1651</v>
-      </c>
-    </row>
-    <row r="77" ht="11" customHeight="true" outlineLevel="3">
+        <v>1888</v>
+      </c>
+    </row>
+    <row r="77" ht="22" customHeight="true" outlineLevel="3">
       <c r="B77" s="17" t="s">
         <v>76</v>
       </c>
       <c r="C77" s="11" t="n">
-        <v>256</v>
+        <v>336</v>
       </c>
     </row>
     <row r="78" ht="11" customHeight="true" outlineLevel="3">
       <c r="B78" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="C78" s="11" t="n">
-        <v>209</v>
+      <c r="C78" s="18" t="n">
+        <v>2704</v>
       </c>
     </row>
     <row r="79" ht="11" customHeight="true" outlineLevel="3">
@@ -2213,7 +2231,7 @@
         <v>78</v>
       </c>
       <c r="C79" s="11" t="n">
-        <v>377</v>
+        <v>256</v>
       </c>
     </row>
     <row r="80" ht="11" customHeight="true" outlineLevel="3">
@@ -2221,7 +2239,7 @@
         <v>79</v>
       </c>
       <c r="C80" s="18" t="n">
-        <v>11168</v>
+        <v>3489</v>
       </c>
     </row>
     <row r="81" ht="11" customHeight="true" outlineLevel="3">
@@ -2229,31 +2247,31 @@
         <v>80</v>
       </c>
       <c r="C81" s="11" t="n">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="82" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B82" s="16" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="82" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B82" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="C82" s="12" t="n">
-        <v>63448</v>
+      <c r="C82" s="18" t="n">
+        <v>5587</v>
       </c>
     </row>
     <row r="83" ht="11" customHeight="true" outlineLevel="3">
       <c r="B83" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="C83" s="18" t="n">
-        <v>2645</v>
-      </c>
-    </row>
-    <row r="84" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B84" s="17" t="s">
+      <c r="C83" s="11" t="n">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="84" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B84" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="C84" s="18" t="n">
-        <v>6542</v>
+      <c r="C84" s="12" t="n">
+        <v>57774</v>
       </c>
     </row>
     <row r="85" ht="11" customHeight="true" outlineLevel="3">
@@ -2261,7 +2279,7 @@
         <v>84</v>
       </c>
       <c r="C85" s="18" t="n">
-        <v>3418</v>
+        <v>1363</v>
       </c>
     </row>
     <row r="86" ht="11" customHeight="true" outlineLevel="3">
@@ -2269,7 +2287,7 @@
         <v>85</v>
       </c>
       <c r="C86" s="18" t="n">
-        <v>3777</v>
+        <v>5899</v>
       </c>
     </row>
     <row r="87" ht="11" customHeight="true" outlineLevel="3">
@@ -2277,7 +2295,7 @@
         <v>86</v>
       </c>
       <c r="C87" s="18" t="n">
-        <v>9021</v>
+        <v>2388</v>
       </c>
     </row>
     <row r="88" ht="11" customHeight="true" outlineLevel="3">
@@ -2285,7 +2303,7 @@
         <v>87</v>
       </c>
       <c r="C88" s="18" t="n">
-        <v>3177</v>
+        <v>2332</v>
       </c>
     </row>
     <row r="89" ht="11" customHeight="true" outlineLevel="3">
@@ -2293,7 +2311,7 @@
         <v>88</v>
       </c>
       <c r="C89" s="18" t="n">
-        <v>7029</v>
+        <v>5589</v>
       </c>
     </row>
     <row r="90" ht="11" customHeight="true" outlineLevel="3">
@@ -2301,7 +2319,7 @@
         <v>89</v>
       </c>
       <c r="C90" s="18" t="n">
-        <v>3670</v>
+        <v>1739</v>
       </c>
     </row>
     <row r="91" ht="11" customHeight="true" outlineLevel="3">
@@ -2309,7 +2327,7 @@
         <v>90</v>
       </c>
       <c r="C91" s="18" t="n">
-        <v>1276</v>
+        <v>5846</v>
       </c>
     </row>
     <row r="92" ht="11" customHeight="true" outlineLevel="3">
@@ -2317,7 +2335,7 @@
         <v>91</v>
       </c>
       <c r="C92" s="18" t="n">
-        <v>4004</v>
+        <v>2269</v>
       </c>
     </row>
     <row r="93" ht="11" customHeight="true" outlineLevel="3">
@@ -2325,7 +2343,7 @@
         <v>92</v>
       </c>
       <c r="C93" s="18" t="n">
-        <v>1123</v>
+        <v>3360</v>
       </c>
     </row>
     <row r="94" ht="11" customHeight="true" outlineLevel="3">
@@ -2333,15 +2351,15 @@
         <v>93</v>
       </c>
       <c r="C94" s="18" t="n">
-        <v>10321</v>
+        <v>2265</v>
       </c>
     </row>
     <row r="95" ht="11" customHeight="true" outlineLevel="3">
       <c r="B95" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="C95" s="18" t="n">
-        <v>3703</v>
+      <c r="C95" s="11" t="n">
+        <v>931</v>
       </c>
     </row>
     <row r="96" ht="11" customHeight="true" outlineLevel="3">
@@ -2349,15 +2367,15 @@
         <v>95</v>
       </c>
       <c r="C96" s="18" t="n">
-        <v>1875</v>
+        <v>19059</v>
       </c>
     </row>
     <row r="97" ht="11" customHeight="true" outlineLevel="3">
       <c r="B97" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="C97" s="11" t="n">
-        <v>247</v>
+      <c r="C97" s="18" t="n">
+        <v>1601</v>
       </c>
     </row>
     <row r="98" ht="11" customHeight="true" outlineLevel="3">
@@ -2365,95 +2383,95 @@
         <v>97</v>
       </c>
       <c r="C98" s="18" t="n">
-        <v>1620</v>
-      </c>
-    </row>
-    <row r="99" ht="11" customHeight="true" outlineLevel="1">
-      <c r="B99" s="13" t="s">
+        <v>2283</v>
+      </c>
+    </row>
+    <row r="99" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B99" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="C99" s="12" t="n">
-        <v>675516</v>
-      </c>
-    </row>
-    <row r="100" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B100" s="16" t="s">
+      <c r="C99" s="11" t="n">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="100" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B100" s="17" t="s">
         <v>99</v>
       </c>
-      <c r="C100" s="12" t="n">
-        <v>117575</v>
-      </c>
-    </row>
-    <row r="101" ht="22" customHeight="true" outlineLevel="3">
-      <c r="B101" s="17" t="s">
+      <c r="C100" s="11" t="n">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="101" ht="11" customHeight="true" outlineLevel="1">
+      <c r="B101" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="C101" s="18" t="n">
-        <v>25214</v>
-      </c>
-    </row>
-    <row r="102" ht="22" customHeight="true" outlineLevel="3">
-      <c r="B102" s="17" t="s">
+      <c r="C101" s="12" t="n">
+        <v>709349</v>
+      </c>
+    </row>
+    <row r="102" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B102" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="C102" s="11" t="n">
-        <v>880</v>
-      </c>
-    </row>
-    <row r="103" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C102" s="12" t="n">
+        <v>112847</v>
+      </c>
+    </row>
+    <row r="103" ht="22" customHeight="true" outlineLevel="3">
       <c r="B103" s="17" t="s">
         <v>102</v>
       </c>
       <c r="C103" s="18" t="n">
-        <v>21637</v>
-      </c>
-    </row>
-    <row r="104" ht="11" customHeight="true" outlineLevel="3">
+        <v>12669</v>
+      </c>
+    </row>
+    <row r="104" ht="22" customHeight="true" outlineLevel="3">
       <c r="B104" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="C104" s="11" t="n">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="105" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C104" s="18" t="n">
+        <v>2570</v>
+      </c>
+    </row>
+    <row r="105" ht="22" customHeight="true" outlineLevel="3">
       <c r="B105" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="C105" s="11" t="n">
-        <v>24</v>
+      <c r="C105" s="18" t="n">
+        <v>2160</v>
       </c>
     </row>
     <row r="106" ht="22" customHeight="true" outlineLevel="3">
       <c r="B106" s="17" t="s">
         <v>105</v>
       </c>
-      <c r="C106" s="11" t="n">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="107" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C106" s="18" t="n">
+        <v>2110</v>
+      </c>
+    </row>
+    <row r="107" ht="11" customHeight="true" outlineLevel="3">
       <c r="B107" s="17" t="s">
         <v>106</v>
       </c>
       <c r="C107" s="18" t="n">
-        <v>2086</v>
-      </c>
-    </row>
-    <row r="108" ht="22" customHeight="true" outlineLevel="3">
+        <v>10672</v>
+      </c>
+    </row>
+    <row r="108" ht="11" customHeight="true" outlineLevel="3">
       <c r="B108" s="17" t="s">
         <v>107</v>
       </c>
       <c r="C108" s="18" t="n">
-        <v>1410</v>
-      </c>
-    </row>
-    <row r="109" ht="22" customHeight="true" outlineLevel="3">
+        <v>12330</v>
+      </c>
+    </row>
+    <row r="109" ht="11" customHeight="true" outlineLevel="3">
       <c r="B109" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="C109" s="11" t="n">
-        <v>11</v>
+      <c r="C109" s="18" t="n">
+        <v>2040</v>
       </c>
     </row>
     <row r="110" ht="22" customHeight="true" outlineLevel="3">
@@ -2461,7 +2479,7 @@
         <v>109</v>
       </c>
       <c r="C110" s="18" t="n">
-        <v>11884</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="111" ht="22" customHeight="true" outlineLevel="3">
@@ -2469,23 +2487,23 @@
         <v>110</v>
       </c>
       <c r="C111" s="18" t="n">
-        <v>5320</v>
+        <v>6601</v>
       </c>
     </row>
     <row r="112" ht="22" customHeight="true" outlineLevel="3">
       <c r="B112" s="17" t="s">
         <v>111</v>
       </c>
-      <c r="C112" s="11" t="n">
-        <v>900</v>
+      <c r="C112" s="18" t="n">
+        <v>3212</v>
       </c>
     </row>
     <row r="113" ht="22" customHeight="true" outlineLevel="3">
       <c r="B113" s="17" t="s">
         <v>112</v>
       </c>
-      <c r="C113" s="11" t="n">
-        <v>30</v>
+      <c r="C113" s="18" t="n">
+        <v>2520</v>
       </c>
     </row>
     <row r="114" ht="22" customHeight="true" outlineLevel="3">
@@ -2493,15 +2511,15 @@
         <v>113</v>
       </c>
       <c r="C114" s="18" t="n">
-        <v>23446</v>
+        <v>5900</v>
       </c>
     </row>
     <row r="115" ht="22" customHeight="true" outlineLevel="3">
       <c r="B115" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="C115" s="18" t="n">
-        <v>1500</v>
+      <c r="C115" s="11" t="n">
+        <v>480</v>
       </c>
     </row>
     <row r="116" ht="22" customHeight="true" outlineLevel="3">
@@ -2509,7 +2527,7 @@
         <v>115</v>
       </c>
       <c r="C116" s="18" t="n">
-        <v>21345</v>
+        <v>24359</v>
       </c>
     </row>
     <row r="117" ht="22" customHeight="true" outlineLevel="3">
@@ -2517,55 +2535,55 @@
         <v>116</v>
       </c>
       <c r="C117" s="18" t="n">
-        <v>1140</v>
-      </c>
-    </row>
-    <row r="118" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B118" s="16" t="s">
+        <v>2510</v>
+      </c>
+    </row>
+    <row r="118" ht="22" customHeight="true" outlineLevel="3">
+      <c r="B118" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="C118" s="12" t="n">
-        <v>7571</v>
-      </c>
-    </row>
-    <row r="119" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C118" s="18" t="n">
+        <v>3210</v>
+      </c>
+    </row>
+    <row r="119" ht="22" customHeight="true" outlineLevel="3">
       <c r="B119" s="17" t="s">
         <v>118</v>
       </c>
       <c r="C119" s="18" t="n">
-        <v>1136</v>
-      </c>
-    </row>
-    <row r="120" ht="11" customHeight="true" outlineLevel="3">
+        <v>17284</v>
+      </c>
+    </row>
+    <row r="120" ht="22" customHeight="true" outlineLevel="3">
       <c r="B120" s="17" t="s">
         <v>119</v>
       </c>
-      <c r="C120" s="11" t="n">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="121" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B121" s="17" t="s">
+      <c r="C120" s="18" t="n">
+        <v>1050</v>
+      </c>
+    </row>
+    <row r="121" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B121" s="16" t="s">
         <v>120</v>
       </c>
-      <c r="C121" s="11" t="n">
-        <v>540</v>
+      <c r="C121" s="12" t="n">
+        <v>10876</v>
       </c>
     </row>
     <row r="122" ht="11" customHeight="true" outlineLevel="3">
       <c r="B122" s="17" t="s">
         <v>121</v>
       </c>
-      <c r="C122" s="11" t="n">
-        <v>429</v>
+      <c r="C122" s="18" t="n">
+        <v>1202</v>
       </c>
     </row>
     <row r="123" ht="11" customHeight="true" outlineLevel="3">
       <c r="B123" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="C123" s="18" t="n">
-        <v>1616</v>
+      <c r="C123" s="11" t="n">
+        <v>234</v>
       </c>
     </row>
     <row r="124" ht="11" customHeight="true" outlineLevel="3">
@@ -2573,7 +2591,7 @@
         <v>123</v>
       </c>
       <c r="C124" s="11" t="n">
-        <v>712</v>
+        <v>669</v>
       </c>
     </row>
     <row r="125" ht="11" customHeight="true" outlineLevel="3">
@@ -2581,39 +2599,39 @@
         <v>124</v>
       </c>
       <c r="C125" s="18" t="n">
-        <v>2081</v>
+        <v>2386</v>
       </c>
     </row>
     <row r="126" ht="11" customHeight="true" outlineLevel="3">
       <c r="B126" s="17" t="s">
         <v>125</v>
       </c>
-      <c r="C126" s="11" t="n">
-        <v>170</v>
+      <c r="C126" s="18" t="n">
+        <v>1093</v>
       </c>
     </row>
     <row r="127" ht="11" customHeight="true" outlineLevel="3">
       <c r="B127" s="17" t="s">
         <v>126</v>
       </c>
-      <c r="C127" s="11" t="n">
-        <v>352</v>
+      <c r="C127" s="18" t="n">
+        <v>1471</v>
       </c>
     </row>
     <row r="128" ht="11" customHeight="true" outlineLevel="3">
       <c r="B128" s="17" t="s">
         <v>127</v>
       </c>
-      <c r="C128" s="11" t="n">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="129" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B129" s="16" t="s">
+      <c r="C128" s="18" t="n">
+        <v>1543</v>
+      </c>
+    </row>
+    <row r="129" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B129" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="C129" s="12" t="n">
-        <v>175424</v>
+      <c r="C129" s="18" t="n">
+        <v>1366</v>
       </c>
     </row>
     <row r="130" ht="11" customHeight="true" outlineLevel="3">
@@ -2621,15 +2639,15 @@
         <v>129</v>
       </c>
       <c r="C130" s="11" t="n">
-        <v>986</v>
-      </c>
-    </row>
-    <row r="131" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B131" s="17" t="s">
+        <v>912</v>
+      </c>
+    </row>
+    <row r="131" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B131" s="16" t="s">
         <v>130</v>
       </c>
-      <c r="C131" s="11" t="n">
-        <v>934</v>
+      <c r="C131" s="12" t="n">
+        <v>161755</v>
       </c>
     </row>
     <row r="132" ht="11" customHeight="true" outlineLevel="3">
@@ -2637,7 +2655,7 @@
         <v>131</v>
       </c>
       <c r="C132" s="11" t="n">
-        <v>535</v>
+        <v>818</v>
       </c>
     </row>
     <row r="133" ht="11" customHeight="true" outlineLevel="3">
@@ -2645,23 +2663,23 @@
         <v>132</v>
       </c>
       <c r="C133" s="11" t="n">
-        <v>60</v>
+        <v>694</v>
       </c>
     </row>
     <row r="134" ht="11" customHeight="true" outlineLevel="3">
       <c r="B134" s="17" t="s">
         <v>133</v>
       </c>
-      <c r="C134" s="18" t="n">
-        <v>1223</v>
+      <c r="C134" s="11" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="135" ht="11" customHeight="true" outlineLevel="3">
       <c r="B135" s="17" t="s">
         <v>134</v>
       </c>
-      <c r="C135" s="18" t="n">
-        <v>1501</v>
+      <c r="C135" s="11" t="n">
+        <v>687</v>
       </c>
     </row>
     <row r="136" ht="11" customHeight="true" outlineLevel="3">
@@ -2669,15 +2687,15 @@
         <v>135</v>
       </c>
       <c r="C136" s="18" t="n">
-        <v>66283</v>
+        <v>3049</v>
       </c>
     </row>
     <row r="137" ht="11" customHeight="true" outlineLevel="3">
       <c r="B137" s="17" t="s">
         <v>136</v>
       </c>
-      <c r="C137" s="18" t="n">
-        <v>22782</v>
+      <c r="C137" s="11" t="n">
+        <v>720</v>
       </c>
     </row>
     <row r="138" ht="11" customHeight="true" outlineLevel="3">
@@ -2685,7 +2703,7 @@
         <v>137</v>
       </c>
       <c r="C138" s="18" t="n">
-        <v>16475</v>
+        <v>61323</v>
       </c>
     </row>
     <row r="139" ht="11" customHeight="true" outlineLevel="3">
@@ -2693,15 +2711,15 @@
         <v>138</v>
       </c>
       <c r="C139" s="18" t="n">
-        <v>36904</v>
+        <v>19457</v>
       </c>
     </row>
     <row r="140" ht="11" customHeight="true" outlineLevel="3">
       <c r="B140" s="17" t="s">
         <v>139</v>
       </c>
-      <c r="C140" s="11" t="n">
-        <v>235</v>
+      <c r="C140" s="18" t="n">
+        <v>17100</v>
       </c>
     </row>
     <row r="141" ht="11" customHeight="true" outlineLevel="3">
@@ -2709,7 +2727,7 @@
         <v>140</v>
       </c>
       <c r="C141" s="18" t="n">
-        <v>3432</v>
+        <v>33604</v>
       </c>
     </row>
     <row r="142" ht="11" customHeight="true" outlineLevel="3">
@@ -2717,7 +2735,7 @@
         <v>141</v>
       </c>
       <c r="C142" s="11" t="n">
-        <v>93</v>
+        <v>100</v>
       </c>
     </row>
     <row r="143" ht="11" customHeight="true" outlineLevel="3">
@@ -2725,7 +2743,7 @@
         <v>142</v>
       </c>
       <c r="C143" s="18" t="n">
-        <v>1491</v>
+        <v>1590</v>
       </c>
     </row>
     <row r="144" ht="11" customHeight="true" outlineLevel="3">
@@ -2733,15 +2751,15 @@
         <v>143</v>
       </c>
       <c r="C144" s="11" t="n">
-        <v>136</v>
+        <v>438</v>
       </c>
     </row>
     <row r="145" ht="11" customHeight="true" outlineLevel="3">
       <c r="B145" s="17" t="s">
         <v>144</v>
       </c>
-      <c r="C145" s="18" t="n">
-        <v>1446</v>
+      <c r="C145" s="11" t="n">
+        <v>92</v>
       </c>
     </row>
     <row r="146" ht="11" customHeight="true" outlineLevel="3">
@@ -2749,15 +2767,15 @@
         <v>145</v>
       </c>
       <c r="C146" s="11" t="n">
-        <v>759</v>
+        <v>709</v>
       </c>
     </row>
     <row r="147" ht="11" customHeight="true" outlineLevel="3">
       <c r="B147" s="17" t="s">
         <v>146</v>
       </c>
-      <c r="C147" s="18" t="n">
-        <v>2051</v>
+      <c r="C147" s="11" t="n">
+        <v>991</v>
       </c>
     </row>
     <row r="148" ht="11" customHeight="true" outlineLevel="3">
@@ -2765,7 +2783,7 @@
         <v>147</v>
       </c>
       <c r="C148" s="11" t="n">
-        <v>263</v>
+        <v>221</v>
       </c>
     </row>
     <row r="149" ht="22" customHeight="true" outlineLevel="3">
@@ -2773,15 +2791,15 @@
         <v>148</v>
       </c>
       <c r="C149" s="18" t="n">
-        <v>4433</v>
+        <v>2655</v>
       </c>
     </row>
     <row r="150" ht="11" customHeight="true" outlineLevel="3">
       <c r="B150" s="17" t="s">
         <v>149</v>
       </c>
-      <c r="C150" s="18" t="n">
-        <v>1364</v>
+      <c r="C150" s="11" t="n">
+        <v>790</v>
       </c>
     </row>
     <row r="151" ht="11" customHeight="true" outlineLevel="3">
@@ -2789,15 +2807,15 @@
         <v>150</v>
       </c>
       <c r="C151" s="18" t="n">
-        <v>2431</v>
+        <v>1508</v>
       </c>
     </row>
     <row r="152" ht="11" customHeight="true" outlineLevel="3">
       <c r="B152" s="17" t="s">
         <v>151</v>
       </c>
-      <c r="C152" s="11" t="n">
-        <v>236</v>
+      <c r="C152" s="18" t="n">
+        <v>1891</v>
       </c>
     </row>
     <row r="153" ht="11" customHeight="true" outlineLevel="3">
@@ -2805,23 +2823,23 @@
         <v>152</v>
       </c>
       <c r="C153" s="18" t="n">
-        <v>1241</v>
+        <v>2366</v>
       </c>
     </row>
     <row r="154" ht="11" customHeight="true" outlineLevel="3">
       <c r="B154" s="17" t="s">
         <v>153</v>
       </c>
-      <c r="C154" s="11" t="n">
-        <v>6</v>
+      <c r="C154" s="18" t="n">
+        <v>2354</v>
       </c>
     </row>
     <row r="155" ht="11" customHeight="true" outlineLevel="3">
       <c r="B155" s="17" t="s">
         <v>154</v>
       </c>
-      <c r="C155" s="18" t="n">
-        <v>1592</v>
+      <c r="C155" s="11" t="n">
+        <v>490</v>
       </c>
     </row>
     <row r="156" ht="11" customHeight="true" outlineLevel="3">
@@ -2829,79 +2847,79 @@
         <v>155</v>
       </c>
       <c r="C156" s="11" t="n">
-        <v>243</v>
+        <v>760</v>
       </c>
     </row>
     <row r="157" ht="11" customHeight="true" outlineLevel="3">
       <c r="B157" s="17" t="s">
         <v>156</v>
       </c>
-      <c r="C157" s="11" t="n">
-        <v>634</v>
+      <c r="C157" s="18" t="n">
+        <v>1602</v>
       </c>
     </row>
     <row r="158" ht="11" customHeight="true" outlineLevel="3">
       <c r="B158" s="17" t="s">
         <v>157</v>
       </c>
-      <c r="C158" s="18" t="n">
-        <v>1156</v>
+      <c r="C158" s="11" t="n">
+        <v>922</v>
       </c>
     </row>
     <row r="159" ht="11" customHeight="true" outlineLevel="3">
       <c r="B159" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="C159" s="11" t="n">
-        <v>563</v>
+      <c r="C159" s="18" t="n">
+        <v>3118</v>
       </c>
     </row>
     <row r="160" ht="11" customHeight="true" outlineLevel="3">
       <c r="B160" s="17" t="s">
         <v>159</v>
       </c>
-      <c r="C160" s="18" t="n">
-        <v>1682</v>
+      <c r="C160" s="11" t="n">
+        <v>37</v>
       </c>
     </row>
     <row r="161" ht="11" customHeight="true" outlineLevel="3">
       <c r="B161" s="17" t="s">
         <v>160</v>
       </c>
-      <c r="C161" s="11" t="n">
-        <v>6</v>
+      <c r="C161" s="18" t="n">
+        <v>1371</v>
       </c>
     </row>
     <row r="162" ht="11" customHeight="true" outlineLevel="3">
       <c r="B162" s="17" t="s">
         <v>161</v>
       </c>
-      <c r="C162" s="18" t="n">
-        <v>1936</v>
-      </c>
-    </row>
-    <row r="163" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B163" s="17" t="s">
+      <c r="C162" s="11" t="n">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="163" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B163" s="16" t="s">
         <v>162</v>
       </c>
-      <c r="C163" s="11" t="n">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="164" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B164" s="16" t="s">
+      <c r="C163" s="12" t="n">
+        <v>147670</v>
+      </c>
+    </row>
+    <row r="164" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B164" s="17" t="s">
         <v>163</v>
       </c>
-      <c r="C164" s="12" t="n">
-        <v>157091</v>
+      <c r="C164" s="18" t="n">
+        <v>1370</v>
       </c>
     </row>
     <row r="165" ht="11" customHeight="true" outlineLevel="3">
       <c r="B165" s="17" t="s">
         <v>164</v>
       </c>
-      <c r="C165" s="18" t="n">
-        <v>2156</v>
+      <c r="C165" s="11" t="n">
+        <v>255</v>
       </c>
     </row>
     <row r="166" ht="11" customHeight="true" outlineLevel="3">
@@ -2909,7 +2927,7 @@
         <v>165</v>
       </c>
       <c r="C166" s="11" t="n">
-        <v>357</v>
+        <v>266</v>
       </c>
     </row>
     <row r="167" ht="11" customHeight="true" outlineLevel="3">
@@ -2917,23 +2935,23 @@
         <v>166</v>
       </c>
       <c r="C167" s="11" t="n">
-        <v>358</v>
+        <v>715</v>
       </c>
     </row>
     <row r="168" ht="11" customHeight="true" outlineLevel="3">
       <c r="B168" s="17" t="s">
         <v>167</v>
       </c>
-      <c r="C168" s="11" t="n">
-        <v>625</v>
+      <c r="C168" s="18" t="n">
+        <v>4162</v>
       </c>
     </row>
     <row r="169" ht="11" customHeight="true" outlineLevel="3">
       <c r="B169" s="17" t="s">
         <v>168</v>
       </c>
-      <c r="C169" s="18" t="n">
-        <v>2041</v>
+      <c r="C169" s="11" t="n">
+        <v>641</v>
       </c>
     </row>
     <row r="170" ht="11" customHeight="true" outlineLevel="3">
@@ -2941,15 +2959,15 @@
         <v>169</v>
       </c>
       <c r="C170" s="11" t="n">
-        <v>600</v>
+        <v>376</v>
       </c>
     </row>
     <row r="171" ht="11" customHeight="true" outlineLevel="3">
       <c r="B171" s="17" t="s">
         <v>170</v>
       </c>
-      <c r="C171" s="11" t="n">
-        <v>904</v>
+      <c r="C171" s="18" t="n">
+        <v>1286</v>
       </c>
     </row>
     <row r="172" ht="11" customHeight="true" outlineLevel="3">
@@ -2957,7 +2975,7 @@
         <v>171</v>
       </c>
       <c r="C172" s="11" t="n">
-        <v>541</v>
+        <v>816</v>
       </c>
     </row>
     <row r="173" ht="11" customHeight="true" outlineLevel="3">
@@ -2965,31 +2983,31 @@
         <v>172</v>
       </c>
       <c r="C173" s="11" t="n">
-        <v>881</v>
+        <v>490</v>
       </c>
     </row>
     <row r="174" ht="11" customHeight="true" outlineLevel="3">
       <c r="B174" s="17" t="s">
         <v>173</v>
       </c>
-      <c r="C174" s="11" t="n">
-        <v>64</v>
+      <c r="C174" s="18" t="n">
+        <v>4397</v>
       </c>
     </row>
     <row r="175" ht="11" customHeight="true" outlineLevel="3">
       <c r="B175" s="17" t="s">
         <v>174</v>
       </c>
-      <c r="C175" s="11" t="n">
-        <v>17</v>
+      <c r="C175" s="18" t="n">
+        <v>1242</v>
       </c>
     </row>
     <row r="176" ht="11" customHeight="true" outlineLevel="3">
       <c r="B176" s="17" t="s">
         <v>175</v>
       </c>
-      <c r="C176" s="18" t="n">
-        <v>4958</v>
+      <c r="C176" s="11" t="n">
+        <v>871</v>
       </c>
     </row>
     <row r="177" ht="11" customHeight="true" outlineLevel="3">
@@ -2997,15 +3015,15 @@
         <v>176</v>
       </c>
       <c r="C177" s="11" t="n">
-        <v>305</v>
+        <v>511</v>
       </c>
     </row>
     <row r="178" ht="11" customHeight="true" outlineLevel="3">
       <c r="B178" s="17" t="s">
         <v>177</v>
       </c>
-      <c r="C178" s="18" t="n">
-        <v>1084</v>
+      <c r="C178" s="11" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="179" ht="11" customHeight="true" outlineLevel="3">
@@ -3013,7 +3031,7 @@
         <v>178</v>
       </c>
       <c r="C179" s="11" t="n">
-        <v>155</v>
+        <v>426</v>
       </c>
     </row>
     <row r="180" ht="11" customHeight="true" outlineLevel="3">
@@ -3021,31 +3039,31 @@
         <v>179</v>
       </c>
       <c r="C180" s="11" t="n">
-        <v>776</v>
+        <v>332</v>
       </c>
     </row>
     <row r="181" ht="11" customHeight="true" outlineLevel="3">
       <c r="B181" s="17" t="s">
         <v>180</v>
       </c>
-      <c r="C181" s="11" t="n">
-        <v>870</v>
+      <c r="C181" s="18" t="n">
+        <v>1251</v>
       </c>
     </row>
     <row r="182" ht="11" customHeight="true" outlineLevel="3">
       <c r="B182" s="17" t="s">
         <v>181</v>
       </c>
-      <c r="C182" s="18" t="n">
-        <v>1033</v>
+      <c r="C182" s="11" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="183" ht="11" customHeight="true" outlineLevel="3">
       <c r="B183" s="17" t="s">
         <v>182</v>
       </c>
-      <c r="C183" s="11" t="n">
-        <v>583</v>
+      <c r="C183" s="18" t="n">
+        <v>1431</v>
       </c>
     </row>
     <row r="184" ht="11" customHeight="true" outlineLevel="3">
@@ -3053,7 +3071,7 @@
         <v>183</v>
       </c>
       <c r="C184" s="11" t="n">
-        <v>183</v>
+        <v>58</v>
       </c>
     </row>
     <row r="185" ht="11" customHeight="true" outlineLevel="3">
@@ -3061,15 +3079,15 @@
         <v>184</v>
       </c>
       <c r="C185" s="11" t="n">
-        <v>685</v>
+        <v>864</v>
       </c>
     </row>
     <row r="186" ht="11" customHeight="true" outlineLevel="3">
       <c r="B186" s="17" t="s">
         <v>185</v>
       </c>
-      <c r="C186" s="11" t="n">
-        <v>15</v>
+      <c r="C186" s="18" t="n">
+        <v>1232</v>
       </c>
     </row>
     <row r="187" ht="11" customHeight="true" outlineLevel="3">
@@ -3077,15 +3095,15 @@
         <v>186</v>
       </c>
       <c r="C187" s="11" t="n">
-        <v>91</v>
+        <v>-77</v>
       </c>
     </row>
     <row r="188" ht="11" customHeight="true" outlineLevel="3">
       <c r="B188" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="C188" s="11" t="n">
-        <v>946</v>
+      <c r="C188" s="18" t="n">
+        <v>3060</v>
       </c>
     </row>
     <row r="189" ht="11" customHeight="true" outlineLevel="3">
@@ -3093,7 +3111,7 @@
         <v>188</v>
       </c>
       <c r="C189" s="18" t="n">
-        <v>1374</v>
+        <v>1603</v>
       </c>
     </row>
     <row r="190" ht="11" customHeight="true" outlineLevel="3">
@@ -3101,31 +3119,31 @@
         <v>189</v>
       </c>
       <c r="C190" s="11" t="n">
-        <v>247</v>
+        <v>89</v>
       </c>
     </row>
     <row r="191" ht="11" customHeight="true" outlineLevel="3">
       <c r="B191" s="17" t="s">
         <v>190</v>
       </c>
-      <c r="C191" s="18" t="n">
-        <v>3659</v>
-      </c>
-    </row>
-    <row r="192" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C191" s="11" t="n">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="192" ht="22" customHeight="true" outlineLevel="3">
       <c r="B192" s="17" t="s">
         <v>191</v>
       </c>
       <c r="C192" s="18" t="n">
-        <v>1393</v>
-      </c>
-    </row>
-    <row r="193" ht="11" customHeight="true" outlineLevel="3">
+        <v>20736</v>
+      </c>
+    </row>
+    <row r="193" ht="22" customHeight="true" outlineLevel="3">
       <c r="B193" s="17" t="s">
         <v>192</v>
       </c>
-      <c r="C193" s="11" t="n">
-        <v>125</v>
+      <c r="C193" s="18" t="n">
+        <v>7819</v>
       </c>
     </row>
     <row r="194" ht="11" customHeight="true" outlineLevel="3">
@@ -3136,60 +3154,60 @@
         <v>522</v>
       </c>
     </row>
-    <row r="195" ht="22" customHeight="true" outlineLevel="3">
+    <row r="195" ht="11" customHeight="true" outlineLevel="3">
       <c r="B195" s="17" t="s">
         <v>194</v>
       </c>
       <c r="C195" s="18" t="n">
-        <v>22265</v>
+        <v>25007</v>
       </c>
     </row>
     <row r="196" ht="22" customHeight="true" outlineLevel="3">
       <c r="B196" s="17" t="s">
         <v>195</v>
       </c>
-      <c r="C196" s="11" t="n">
-        <v>54</v>
+      <c r="C196" s="18" t="n">
+        <v>4101</v>
       </c>
     </row>
     <row r="197" ht="22" customHeight="true" outlineLevel="3">
       <c r="B197" s="17" t="s">
         <v>196</v>
       </c>
-      <c r="C197" s="18" t="n">
-        <v>9161</v>
+      <c r="C197" s="11" t="n">
+        <v>298</v>
       </c>
     </row>
     <row r="198" ht="11" customHeight="true" outlineLevel="3">
       <c r="B198" s="17" t="s">
         <v>197</v>
       </c>
-      <c r="C198" s="18" t="n">
-        <v>26215</v>
+      <c r="C198" s="11" t="n">
+        <v>577</v>
       </c>
     </row>
     <row r="199" ht="11" customHeight="true" outlineLevel="3">
       <c r="B199" s="17" t="s">
         <v>198</v>
       </c>
-      <c r="C199" s="11" t="n">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="200" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C199" s="18" t="n">
+        <v>15017</v>
+      </c>
+    </row>
+    <row r="200" ht="11" customHeight="true" outlineLevel="3">
       <c r="B200" s="17" t="s">
         <v>199</v>
       </c>
-      <c r="C200" s="18" t="n">
-        <v>4761</v>
-      </c>
-    </row>
-    <row r="201" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C200" s="11" t="n">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="201" ht="11" customHeight="true" outlineLevel="3">
       <c r="B201" s="17" t="s">
         <v>200</v>
       </c>
       <c r="C201" s="11" t="n">
-        <v>298</v>
+        <v>86</v>
       </c>
     </row>
     <row r="202" ht="11" customHeight="true" outlineLevel="3">
@@ -3197,15 +3215,15 @@
         <v>201</v>
       </c>
       <c r="C202" s="11" t="n">
-        <v>611</v>
+        <v>444</v>
       </c>
     </row>
     <row r="203" ht="11" customHeight="true" outlineLevel="3">
       <c r="B203" s="17" t="s">
         <v>202</v>
       </c>
-      <c r="C203" s="18" t="n">
-        <v>16187</v>
+      <c r="C203" s="11" t="n">
+        <v>161</v>
       </c>
     </row>
     <row r="204" ht="11" customHeight="true" outlineLevel="3">
@@ -3213,7 +3231,7 @@
         <v>203</v>
       </c>
       <c r="C204" s="11" t="n">
-        <v>861</v>
+        <v>556</v>
       </c>
     </row>
     <row r="205" ht="11" customHeight="true" outlineLevel="3">
@@ -3221,7 +3239,7 @@
         <v>204</v>
       </c>
       <c r="C205" s="11" t="n">
-        <v>86</v>
+        <v>608</v>
       </c>
     </row>
     <row r="206" ht="11" customHeight="true" outlineLevel="3">
@@ -3229,7 +3247,7 @@
         <v>205</v>
       </c>
       <c r="C206" s="11" t="n">
-        <v>577</v>
+        <v>470</v>
       </c>
     </row>
     <row r="207" ht="11" customHeight="true" outlineLevel="3">
@@ -3237,7 +3255,7 @@
         <v>206</v>
       </c>
       <c r="C207" s="11" t="n">
-        <v>929</v>
+        <v>430</v>
       </c>
     </row>
     <row r="208" ht="11" customHeight="true" outlineLevel="3">
@@ -3245,7 +3263,7 @@
         <v>207</v>
       </c>
       <c r="C208" s="18" t="n">
-        <v>1009</v>
+        <v>1775</v>
       </c>
     </row>
     <row r="209" ht="11" customHeight="true" outlineLevel="3">
@@ -3253,15 +3271,15 @@
         <v>208</v>
       </c>
       <c r="C209" s="11" t="n">
-        <v>773</v>
+        <v>962</v>
       </c>
     </row>
     <row r="210" ht="11" customHeight="true" outlineLevel="3">
       <c r="B210" s="17" t="s">
         <v>209</v>
       </c>
-      <c r="C210" s="11" t="n">
-        <v>26</v>
+      <c r="C210" s="18" t="n">
+        <v>1259</v>
       </c>
     </row>
     <row r="211" ht="11" customHeight="true" outlineLevel="3">
@@ -3269,63 +3287,63 @@
         <v>210</v>
       </c>
       <c r="C211" s="18" t="n">
-        <v>2564</v>
+        <v>1218</v>
       </c>
     </row>
     <row r="212" ht="11" customHeight="true" outlineLevel="3">
       <c r="B212" s="17" t="s">
         <v>211</v>
       </c>
-      <c r="C212" s="18" t="n">
-        <v>1577</v>
+      <c r="C212" s="11" t="n">
+        <v>701</v>
       </c>
     </row>
     <row r="213" ht="11" customHeight="true" outlineLevel="3">
       <c r="B213" s="17" t="s">
         <v>212</v>
       </c>
-      <c r="C213" s="18" t="n">
-        <v>1292</v>
+      <c r="C213" s="11" t="n">
+        <v>668</v>
       </c>
     </row>
     <row r="214" ht="11" customHeight="true" outlineLevel="3">
       <c r="B214" s="17" t="s">
         <v>213</v>
       </c>
-      <c r="C214" s="18" t="n">
-        <v>1547</v>
+      <c r="C214" s="11" t="n">
+        <v>656</v>
       </c>
     </row>
     <row r="215" ht="11" customHeight="true" outlineLevel="3">
       <c r="B215" s="17" t="s">
         <v>214</v>
       </c>
-      <c r="C215" s="18" t="n">
-        <v>1068</v>
+      <c r="C215" s="11" t="n">
+        <v>125</v>
       </c>
     </row>
     <row r="216" ht="11" customHeight="true" outlineLevel="3">
       <c r="B216" s="17" t="s">
         <v>215</v>
       </c>
-      <c r="C216" s="11" t="n">
-        <v>850</v>
+      <c r="C216" s="18" t="n">
+        <v>1410</v>
       </c>
     </row>
     <row r="217" ht="11" customHeight="true" outlineLevel="3">
       <c r="B217" s="17" t="s">
         <v>216</v>
       </c>
-      <c r="C217" s="11" t="n">
-        <v>799</v>
+      <c r="C217" s="18" t="n">
+        <v>2238</v>
       </c>
     </row>
     <row r="218" ht="11" customHeight="true" outlineLevel="3">
       <c r="B218" s="17" t="s">
         <v>217</v>
       </c>
-      <c r="C218" s="18" t="n">
-        <v>2064</v>
+      <c r="C218" s="11" t="n">
+        <v>785</v>
       </c>
     </row>
     <row r="219" ht="11" customHeight="true" outlineLevel="3">
@@ -3333,7 +3351,7 @@
         <v>218</v>
       </c>
       <c r="C219" s="18" t="n">
-        <v>2273</v>
+        <v>1830</v>
       </c>
     </row>
     <row r="220" ht="11" customHeight="true" outlineLevel="3">
@@ -3341,7 +3359,7 @@
         <v>219</v>
       </c>
       <c r="C220" s="11" t="n">
-        <v>828</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="221" ht="11" customHeight="true" outlineLevel="3">
@@ -3349,7 +3367,7 @@
         <v>220</v>
       </c>
       <c r="C221" s="11" t="n">
-        <v>327</v>
+        <v>234</v>
       </c>
     </row>
     <row r="222" ht="11" customHeight="true" outlineLevel="3">
@@ -3357,23 +3375,23 @@
         <v>221</v>
       </c>
       <c r="C222" s="18" t="n">
-        <v>1057</v>
+        <v>17231</v>
       </c>
     </row>
     <row r="223" ht="11" customHeight="true" outlineLevel="3">
       <c r="B223" s="17" t="s">
         <v>222</v>
       </c>
-      <c r="C223" s="18" t="n">
-        <v>17708</v>
+      <c r="C223" s="11" t="n">
+        <v>382</v>
       </c>
     </row>
     <row r="224" ht="11" customHeight="true" outlineLevel="3">
       <c r="B224" s="17" t="s">
         <v>223</v>
       </c>
-      <c r="C224" s="11" t="n">
-        <v>407</v>
+      <c r="C224" s="18" t="n">
+        <v>1015</v>
       </c>
     </row>
     <row r="225" ht="11" customHeight="true" outlineLevel="3">
@@ -3381,7 +3399,7 @@
         <v>224</v>
       </c>
       <c r="C225" s="11" t="n">
-        <v>609</v>
+        <v>529</v>
       </c>
     </row>
     <row r="226" ht="11" customHeight="true" outlineLevel="3">
@@ -3389,7 +3407,7 @@
         <v>225</v>
       </c>
       <c r="C226" s="18" t="n">
-        <v>1889</v>
+        <v>1166</v>
       </c>
     </row>
     <row r="227" ht="11" customHeight="true" outlineLevel="3">
@@ -3397,7 +3415,7 @@
         <v>226</v>
       </c>
       <c r="C227" s="18" t="n">
-        <v>2274</v>
+        <v>2683</v>
       </c>
     </row>
     <row r="228" ht="11" customHeight="true" outlineLevel="3">
@@ -3413,15 +3431,15 @@
         <v>228</v>
       </c>
       <c r="C229" s="11" t="n">
-        <v>225</v>
+        <v>201</v>
       </c>
     </row>
     <row r="230" ht="11" customHeight="true" outlineLevel="3">
       <c r="B230" s="17" t="s">
         <v>229</v>
       </c>
-      <c r="C230" s="18" t="n">
-        <v>1539</v>
+      <c r="C230" s="11" t="n">
+        <v>748</v>
       </c>
     </row>
     <row r="231" ht="11" customHeight="true" outlineLevel="3">
@@ -3429,7 +3447,7 @@
         <v>230</v>
       </c>
       <c r="C231" s="11" t="n">
-        <v>445</v>
+        <v>395</v>
       </c>
     </row>
     <row r="232" ht="11" customHeight="true" outlineLevel="3">
@@ -3437,7 +3455,7 @@
         <v>231</v>
       </c>
       <c r="C232" s="18" t="n">
-        <v>3918</v>
+        <v>3300</v>
       </c>
     </row>
     <row r="233" ht="11" customHeight="true" outlineLevel="3">
@@ -3445,7 +3463,7 @@
         <v>232</v>
       </c>
       <c r="C233" s="11" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
     </row>
     <row r="234" ht="11" customHeight="true" outlineLevel="2">
@@ -3453,7 +3471,7 @@
         <v>233</v>
       </c>
       <c r="C234" s="12" t="n">
-        <v>53483</v>
+        <v>75273</v>
       </c>
     </row>
     <row r="235" ht="11" customHeight="true" outlineLevel="3">
@@ -3461,7 +3479,7 @@
         <v>234</v>
       </c>
       <c r="C235" s="18" t="n">
-        <v>1009</v>
+        <v>1430</v>
       </c>
     </row>
     <row r="236" ht="11" customHeight="true" outlineLevel="3">
@@ -3469,7 +3487,7 @@
         <v>235</v>
       </c>
       <c r="C236" s="11" t="n">
-        <v>428</v>
+        <v>462</v>
       </c>
     </row>
     <row r="237" ht="11" customHeight="true" outlineLevel="3">
@@ -3477,7 +3495,7 @@
         <v>236</v>
       </c>
       <c r="C237" s="18" t="n">
-        <v>1275</v>
+        <v>2796</v>
       </c>
     </row>
     <row r="238" ht="11" customHeight="true" outlineLevel="3">
@@ -3485,23 +3503,23 @@
         <v>237</v>
       </c>
       <c r="C238" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="239" ht="11" customHeight="true" outlineLevel="3">
       <c r="B239" s="17" t="s">
         <v>238</v>
       </c>
-      <c r="C239" s="11" t="n">
-        <v>369</v>
+      <c r="C239" s="18" t="n">
+        <v>1493</v>
       </c>
     </row>
     <row r="240" ht="11" customHeight="true" outlineLevel="3">
       <c r="B240" s="17" t="s">
         <v>239</v>
       </c>
-      <c r="C240" s="11" t="n">
-        <v>769</v>
+      <c r="C240" s="18" t="n">
+        <v>1339</v>
       </c>
     </row>
     <row r="241" ht="11" customHeight="true" outlineLevel="3">
@@ -3509,7 +3527,7 @@
         <v>240</v>
       </c>
       <c r="C241" s="18" t="n">
-        <v>5334</v>
+        <v>6777</v>
       </c>
     </row>
     <row r="242" ht="11" customHeight="true" outlineLevel="3">
@@ -3517,7 +3535,7 @@
         <v>241</v>
       </c>
       <c r="C242" s="11" t="n">
-        <v>320</v>
+        <v>300</v>
       </c>
     </row>
     <row r="243" ht="11" customHeight="true" outlineLevel="3">
@@ -3533,7 +3551,7 @@
         <v>243</v>
       </c>
       <c r="C244" s="11" t="n">
-        <v>457</v>
+        <v>398</v>
       </c>
     </row>
     <row r="245" ht="11" customHeight="true" outlineLevel="3">
@@ -3541,7 +3559,7 @@
         <v>244</v>
       </c>
       <c r="C245" s="11" t="n">
-        <v>206</v>
+        <v>226</v>
       </c>
     </row>
     <row r="246" ht="11" customHeight="true" outlineLevel="3">
@@ -3549,7 +3567,7 @@
         <v>245</v>
       </c>
       <c r="C246" s="11" t="n">
-        <v>706</v>
+        <v>974</v>
       </c>
     </row>
     <row r="247" ht="11" customHeight="true" outlineLevel="3">
@@ -3557,7 +3575,7 @@
         <v>246</v>
       </c>
       <c r="C247" s="11" t="n">
-        <v>400</v>
+        <v>318</v>
       </c>
     </row>
     <row r="248" ht="11" customHeight="true" outlineLevel="3">
@@ -3565,7 +3583,7 @@
         <v>247</v>
       </c>
       <c r="C248" s="18" t="n">
-        <v>1340</v>
+        <v>2096</v>
       </c>
     </row>
     <row r="249" ht="11" customHeight="true" outlineLevel="3">
@@ -3573,7 +3591,7 @@
         <v>248</v>
       </c>
       <c r="C249" s="18" t="n">
-        <v>1894</v>
+        <v>1763</v>
       </c>
     </row>
     <row r="250" ht="11" customHeight="true" outlineLevel="3">
@@ -3581,23 +3599,23 @@
         <v>249</v>
       </c>
       <c r="C250" s="18" t="n">
-        <v>1626</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="251" ht="11" customHeight="true" outlineLevel="3">
       <c r="B251" s="17" t="s">
         <v>250</v>
       </c>
-      <c r="C251" s="11" t="n">
-        <v>723</v>
+      <c r="C251" s="18" t="n">
+        <v>1093</v>
       </c>
     </row>
     <row r="252" ht="11" customHeight="true" outlineLevel="3">
       <c r="B252" s="17" t="s">
         <v>251</v>
       </c>
-      <c r="C252" s="11" t="n">
-        <v>719</v>
+      <c r="C252" s="18" t="n">
+        <v>1565</v>
       </c>
     </row>
     <row r="253" ht="11" customHeight="true" outlineLevel="3">
@@ -3605,15 +3623,15 @@
         <v>252</v>
       </c>
       <c r="C253" s="11" t="n">
-        <v>571</v>
+        <v>321</v>
       </c>
     </row>
     <row r="254" ht="11" customHeight="true" outlineLevel="3">
       <c r="B254" s="17" t="s">
         <v>253</v>
       </c>
-      <c r="C254" s="18" t="n">
-        <v>1471</v>
+      <c r="C254" s="11" t="n">
+        <v>981</v>
       </c>
     </row>
     <row r="255" ht="11" customHeight="true" outlineLevel="3">
@@ -3621,7 +3639,7 @@
         <v>254</v>
       </c>
       <c r="C255" s="18" t="n">
-        <v>1265</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="256" ht="11" customHeight="true" outlineLevel="3">
@@ -3629,7 +3647,7 @@
         <v>255</v>
       </c>
       <c r="C256" s="11" t="n">
-        <v>678</v>
+        <v>434</v>
       </c>
     </row>
     <row r="257" ht="11" customHeight="true" outlineLevel="3">
@@ -3637,7 +3655,7 @@
         <v>256</v>
       </c>
       <c r="C257" s="18" t="n">
-        <v>1181</v>
+        <v>1906</v>
       </c>
     </row>
     <row r="258" ht="11" customHeight="true" outlineLevel="3">
@@ -3645,7 +3663,7 @@
         <v>257</v>
       </c>
       <c r="C258" s="18" t="n">
-        <v>2687</v>
+        <v>2094</v>
       </c>
     </row>
     <row r="259" ht="11" customHeight="true" outlineLevel="3">
@@ -3653,7 +3671,7 @@
         <v>258</v>
       </c>
       <c r="C259" s="18" t="n">
-        <v>3283</v>
+        <v>4659</v>
       </c>
     </row>
     <row r="260" ht="11" customHeight="true" outlineLevel="3">
@@ -3661,7 +3679,7 @@
         <v>259</v>
       </c>
       <c r="C260" s="18" t="n">
-        <v>1735</v>
+        <v>3289</v>
       </c>
     </row>
     <row r="261" ht="11" customHeight="true" outlineLevel="3">
@@ -3669,7 +3687,7 @@
         <v>260</v>
       </c>
       <c r="C261" s="18" t="n">
-        <v>2396</v>
+        <v>4344</v>
       </c>
     </row>
     <row r="262" ht="11" customHeight="true" outlineLevel="3">
@@ -3677,7 +3695,7 @@
         <v>261</v>
       </c>
       <c r="C262" s="18" t="n">
-        <v>2629</v>
+        <v>4597</v>
       </c>
     </row>
     <row r="263" ht="11" customHeight="true" outlineLevel="3">
@@ -3685,7 +3703,7 @@
         <v>262</v>
       </c>
       <c r="C263" s="18" t="n">
-        <v>1491</v>
+        <v>1755</v>
       </c>
     </row>
     <row r="264" ht="11" customHeight="true" outlineLevel="3">
@@ -3693,7 +3711,7 @@
         <v>263</v>
       </c>
       <c r="C264" s="18" t="n">
-        <v>1349</v>
+        <v>1913</v>
       </c>
     </row>
     <row r="265" ht="11" customHeight="true" outlineLevel="3">
@@ -3701,7 +3719,7 @@
         <v>264</v>
       </c>
       <c r="C265" s="18" t="n">
-        <v>2704</v>
+        <v>3346</v>
       </c>
     </row>
     <row r="266" ht="11" customHeight="true" outlineLevel="3">
@@ -3709,7 +3727,7 @@
         <v>265</v>
       </c>
       <c r="C266" s="18" t="n">
-        <v>1643</v>
+        <v>3599</v>
       </c>
     </row>
     <row r="267" ht="11" customHeight="true" outlineLevel="3">
@@ -3717,7 +3735,7 @@
         <v>266</v>
       </c>
       <c r="C267" s="18" t="n">
-        <v>3356</v>
+        <v>4605</v>
       </c>
     </row>
     <row r="268" ht="11" customHeight="true" outlineLevel="3">
@@ -3725,7 +3743,7 @@
         <v>267</v>
       </c>
       <c r="C268" s="18" t="n">
-        <v>1696</v>
+        <v>2845</v>
       </c>
     </row>
     <row r="269" ht="11" customHeight="true" outlineLevel="3">
@@ -3733,7 +3751,7 @@
         <v>268</v>
       </c>
       <c r="C269" s="18" t="n">
-        <v>4500</v>
+        <v>6236</v>
       </c>
     </row>
     <row r="270" ht="11" customHeight="true" outlineLevel="3">
@@ -3741,7 +3759,7 @@
         <v>269</v>
       </c>
       <c r="C270" s="18" t="n">
-        <v>1223</v>
+        <v>1629</v>
       </c>
     </row>
     <row r="271" ht="11" customHeight="true" outlineLevel="2">
@@ -3749,7 +3767,7 @@
         <v>270</v>
       </c>
       <c r="C271" s="12" t="n">
-        <v>5095</v>
+        <v>5857</v>
       </c>
     </row>
     <row r="272" ht="11" customHeight="true" outlineLevel="3">
@@ -3757,7 +3775,7 @@
         <v>271</v>
       </c>
       <c r="C272" s="11" t="n">
-        <v>35</v>
+        <v>272</v>
       </c>
     </row>
     <row r="273" ht="11" customHeight="true" outlineLevel="3">
@@ -3765,7 +3783,7 @@
         <v>272</v>
       </c>
       <c r="C273" s="11" t="n">
-        <v>97</v>
+        <v>55</v>
       </c>
     </row>
     <row r="274" ht="11" customHeight="true" outlineLevel="3">
@@ -3773,7 +3791,7 @@
         <v>273</v>
       </c>
       <c r="C274" s="11" t="n">
-        <v>80</v>
+        <v>69</v>
       </c>
     </row>
     <row r="275" ht="11" customHeight="true" outlineLevel="3">
@@ -3781,7 +3799,7 @@
         <v>274</v>
       </c>
       <c r="C275" s="11" t="n">
-        <v>165</v>
+        <v>498</v>
       </c>
     </row>
     <row r="276" ht="11" customHeight="true" outlineLevel="3">
@@ -3789,7 +3807,7 @@
         <v>275</v>
       </c>
       <c r="C276" s="11" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="277" ht="11" customHeight="true" outlineLevel="3">
@@ -3797,7 +3815,7 @@
         <v>276</v>
       </c>
       <c r="C277" s="11" t="n">
-        <v>5</v>
+        <v>384</v>
       </c>
     </row>
     <row r="278" ht="11" customHeight="true" outlineLevel="3">
@@ -3805,7 +3823,7 @@
         <v>277</v>
       </c>
       <c r="C278" s="11" t="n">
-        <v>418</v>
+        <v>16</v>
       </c>
     </row>
     <row r="279" ht="11" customHeight="true" outlineLevel="3">
@@ -3813,7 +3831,7 @@
         <v>278</v>
       </c>
       <c r="C279" s="11" t="n">
-        <v>390</v>
+        <v>194</v>
       </c>
     </row>
     <row r="280" ht="11" customHeight="true" outlineLevel="3">
@@ -3821,7 +3839,7 @@
         <v>279</v>
       </c>
       <c r="C280" s="11" t="n">
-        <v>49</v>
+        <v>275</v>
       </c>
     </row>
     <row r="281" ht="11" customHeight="true" outlineLevel="3">
@@ -3829,7 +3847,7 @@
         <v>280</v>
       </c>
       <c r="C281" s="11" t="n">
-        <v>437</v>
+        <v>569</v>
       </c>
     </row>
     <row r="282" ht="11" customHeight="true" outlineLevel="3">
@@ -3837,7 +3855,7 @@
         <v>281</v>
       </c>
       <c r="C282" s="11" t="n">
-        <v>286</v>
+        <v>661</v>
       </c>
     </row>
     <row r="283" ht="11" customHeight="true" outlineLevel="3">
@@ -3845,7 +3863,7 @@
         <v>282</v>
       </c>
       <c r="C283" s="11" t="n">
-        <v>555</v>
+        <v>345</v>
       </c>
     </row>
     <row r="284" ht="11" customHeight="true" outlineLevel="3">
@@ -3853,7 +3871,7 @@
         <v>283</v>
       </c>
       <c r="C284" s="11" t="n">
-        <v>829</v>
+        <v>258</v>
       </c>
     </row>
     <row r="285" ht="11" customHeight="true" outlineLevel="3">
@@ -3861,7 +3879,7 @@
         <v>284</v>
       </c>
       <c r="C285" s="11" t="n">
-        <v>345</v>
+        <v>60</v>
       </c>
     </row>
     <row r="286" ht="11" customHeight="true" outlineLevel="3">
@@ -3869,7 +3887,7 @@
         <v>285</v>
       </c>
       <c r="C286" s="11" t="n">
-        <v>312</v>
+        <v>455</v>
       </c>
     </row>
     <row r="287" ht="11" customHeight="true" outlineLevel="3">
@@ -3877,7 +3895,7 @@
         <v>286</v>
       </c>
       <c r="C287" s="11" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
     </row>
     <row r="288" ht="11" customHeight="true" outlineLevel="3">
@@ -3885,7 +3903,7 @@
         <v>287</v>
       </c>
       <c r="C288" s="11" t="n">
-        <v>429</v>
+        <v>960</v>
       </c>
     </row>
     <row r="289" ht="11" customHeight="true" outlineLevel="3">
@@ -3893,7 +3911,7 @@
         <v>288</v>
       </c>
       <c r="C289" s="11" t="n">
-        <v>35</v>
+        <v>22</v>
       </c>
     </row>
     <row r="290" ht="11" customHeight="true" outlineLevel="3">
@@ -3901,7 +3919,7 @@
         <v>289</v>
       </c>
       <c r="C290" s="11" t="n">
-        <v>142</v>
+        <v>557</v>
       </c>
     </row>
     <row r="291" ht="11" customHeight="true" outlineLevel="3">
@@ -3909,7 +3927,7 @@
         <v>290</v>
       </c>
       <c r="C291" s="11" t="n">
-        <v>50</v>
+        <v>7</v>
       </c>
     </row>
     <row r="292" ht="11" customHeight="true" outlineLevel="3">
@@ -3917,15 +3935,15 @@
         <v>291</v>
       </c>
       <c r="C292" s="11" t="n">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="293" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B293" s="17" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="293" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B293" s="16" t="s">
         <v>292</v>
       </c>
-      <c r="C293" s="11" t="n">
-        <v>7</v>
+      <c r="C293" s="12" t="n">
+        <v>63144</v>
       </c>
     </row>
     <row r="294" ht="11" customHeight="true" outlineLevel="3">
@@ -3933,15 +3951,15 @@
         <v>293</v>
       </c>
       <c r="C294" s="11" t="n">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="295" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B295" s="16" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="295" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B295" s="17" t="s">
         <v>294</v>
       </c>
-      <c r="C295" s="12" t="n">
-        <v>53377</v>
+      <c r="C295" s="11" t="n">
+        <v>990</v>
       </c>
     </row>
     <row r="296" ht="11" customHeight="true" outlineLevel="3">
@@ -3949,7 +3967,7 @@
         <v>295</v>
       </c>
       <c r="C296" s="11" t="n">
-        <v>485</v>
+        <v>340</v>
       </c>
     </row>
     <row r="297" ht="11" customHeight="true" outlineLevel="3">
@@ -3957,7 +3975,7 @@
         <v>296</v>
       </c>
       <c r="C297" s="11" t="n">
-        <v>114</v>
+        <v>78</v>
       </c>
     </row>
     <row r="298" ht="11" customHeight="true" outlineLevel="3">
@@ -3965,7 +3983,7 @@
         <v>297</v>
       </c>
       <c r="C298" s="11" t="n">
-        <v>409</v>
+        <v>269</v>
       </c>
     </row>
     <row r="299" ht="11" customHeight="true" outlineLevel="3">
@@ -3973,7 +3991,7 @@
         <v>298</v>
       </c>
       <c r="C299" s="11" t="n">
-        <v>78</v>
+        <v>151</v>
       </c>
     </row>
     <row r="300" ht="11" customHeight="true" outlineLevel="3">
@@ -3981,7 +3999,7 @@
         <v>299</v>
       </c>
       <c r="C300" s="11" t="n">
-        <v>490</v>
+        <v>775</v>
       </c>
     </row>
     <row r="301" ht="11" customHeight="true" outlineLevel="3">
@@ -3989,7 +4007,7 @@
         <v>300</v>
       </c>
       <c r="C301" s="11" t="n">
-        <v>349</v>
+        <v>604</v>
       </c>
     </row>
     <row r="302" ht="11" customHeight="true" outlineLevel="3">
@@ -3997,15 +4015,15 @@
         <v>301</v>
       </c>
       <c r="C302" s="11" t="n">
-        <v>504</v>
-      </c>
-    </row>
-    <row r="303" ht="11" customHeight="true" outlineLevel="3">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="303" ht="22" customHeight="true" outlineLevel="3">
       <c r="B303" s="17" t="s">
         <v>302</v>
       </c>
       <c r="C303" s="11" t="n">
-        <v>129</v>
+        <v>215</v>
       </c>
     </row>
     <row r="304" ht="11" customHeight="true" outlineLevel="3">
@@ -4013,15 +4031,15 @@
         <v>303</v>
       </c>
       <c r="C304" s="11" t="n">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="305" ht="22" customHeight="true" outlineLevel="3">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="305" ht="11" customHeight="true" outlineLevel="3">
       <c r="B305" s="17" t="s">
         <v>304</v>
       </c>
       <c r="C305" s="11" t="n">
-        <v>365</v>
+        <v>188</v>
       </c>
     </row>
     <row r="306" ht="11" customHeight="true" outlineLevel="3">
@@ -4029,15 +4047,15 @@
         <v>305</v>
       </c>
       <c r="C306" s="11" t="n">
-        <v>73</v>
+        <v>657</v>
       </c>
     </row>
     <row r="307" ht="11" customHeight="true" outlineLevel="3">
       <c r="B307" s="17" t="s">
         <v>306</v>
       </c>
-      <c r="C307" s="11" t="n">
-        <v>292</v>
+      <c r="C307" s="18" t="n">
+        <v>1547</v>
       </c>
     </row>
     <row r="308" ht="11" customHeight="true" outlineLevel="3">
@@ -4045,31 +4063,31 @@
         <v>307</v>
       </c>
       <c r="C308" s="11" t="n">
-        <v>820</v>
-      </c>
-    </row>
-    <row r="309" ht="11" customHeight="true" outlineLevel="3">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="309" ht="22" customHeight="true" outlineLevel="3">
       <c r="B309" s="17" t="s">
         <v>308</v>
       </c>
-      <c r="C309" s="18" t="n">
-        <v>1794</v>
-      </c>
-    </row>
-    <row r="310" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C309" s="11" t="n">
+        <v>854</v>
+      </c>
+    </row>
+    <row r="310" ht="22" customHeight="true" outlineLevel="3">
       <c r="B310" s="17" t="s">
         <v>309</v>
       </c>
-      <c r="C310" s="18" t="n">
-        <v>1044</v>
+      <c r="C310" s="11" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="311" ht="22" customHeight="true" outlineLevel="3">
       <c r="B311" s="17" t="s">
         <v>310</v>
       </c>
-      <c r="C311" s="11" t="n">
-        <v>982</v>
+      <c r="C311" s="18" t="n">
+        <v>1266</v>
       </c>
     </row>
     <row r="312" ht="22" customHeight="true" outlineLevel="3">
@@ -4077,15 +4095,15 @@
         <v>311</v>
       </c>
       <c r="C312" s="11" t="n">
-        <v>31</v>
+        <v>42</v>
       </c>
     </row>
     <row r="313" ht="22" customHeight="true" outlineLevel="3">
       <c r="B313" s="17" t="s">
         <v>312</v>
       </c>
-      <c r="C313" s="11" t="n">
-        <v>464</v>
+      <c r="C313" s="18" t="n">
+        <v>1282</v>
       </c>
     </row>
     <row r="314" ht="22" customHeight="true" outlineLevel="3">
@@ -4093,7 +4111,7 @@
         <v>313</v>
       </c>
       <c r="C314" s="11" t="n">
-        <v>108</v>
+        <v>186</v>
       </c>
     </row>
     <row r="315" ht="22" customHeight="true" outlineLevel="3">
@@ -4101,7 +4119,7 @@
         <v>314</v>
       </c>
       <c r="C315" s="11" t="n">
-        <v>400</v>
+        <v>151</v>
       </c>
     </row>
     <row r="316" ht="22" customHeight="true" outlineLevel="3">
@@ -4109,15 +4127,15 @@
         <v>315</v>
       </c>
       <c r="C316" s="11" t="n">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="317" ht="22" customHeight="true" outlineLevel="3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="317" ht="11" customHeight="true" outlineLevel="3">
       <c r="B317" s="17" t="s">
         <v>316</v>
       </c>
       <c r="C317" s="11" t="n">
-        <v>92</v>
+        <v>657</v>
       </c>
     </row>
     <row r="318" ht="11" customHeight="true" outlineLevel="3">
@@ -4125,7 +4143,7 @@
         <v>317</v>
       </c>
       <c r="C318" s="11" t="n">
-        <v>354</v>
+        <v>52</v>
       </c>
     </row>
     <row r="319" ht="11" customHeight="true" outlineLevel="3">
@@ -4133,7 +4151,7 @@
         <v>318</v>
       </c>
       <c r="C319" s="11" t="n">
-        <v>442</v>
+        <v>928</v>
       </c>
     </row>
     <row r="320" ht="11" customHeight="true" outlineLevel="3">
@@ -4141,15 +4159,15 @@
         <v>319</v>
       </c>
       <c r="C320" s="11" t="n">
-        <v>386</v>
+        <v>148</v>
       </c>
     </row>
     <row r="321" ht="11" customHeight="true" outlineLevel="3">
       <c r="B321" s="17" t="s">
         <v>320</v>
       </c>
-      <c r="C321" s="11" t="n">
-        <v>275</v>
+      <c r="C321" s="18" t="n">
+        <v>2601</v>
       </c>
     </row>
     <row r="322" ht="11" customHeight="true" outlineLevel="3">
@@ -4157,15 +4175,15 @@
         <v>321</v>
       </c>
       <c r="C322" s="18" t="n">
-        <v>4258</v>
+        <v>2570</v>
       </c>
     </row>
     <row r="323" ht="11" customHeight="true" outlineLevel="3">
       <c r="B323" s="17" t="s">
         <v>322</v>
       </c>
-      <c r="C323" s="18" t="n">
-        <v>2451</v>
+      <c r="C323" s="11" t="n">
+        <v>765</v>
       </c>
     </row>
     <row r="324" ht="11" customHeight="true" outlineLevel="3">
@@ -4173,15 +4191,15 @@
         <v>323</v>
       </c>
       <c r="C324" s="18" t="n">
-        <v>2039</v>
+        <v>1960</v>
       </c>
     </row>
     <row r="325" ht="11" customHeight="true" outlineLevel="3">
       <c r="B325" s="17" t="s">
         <v>324</v>
       </c>
-      <c r="C325" s="18" t="n">
-        <v>1322</v>
+      <c r="C325" s="11" t="n">
+        <v>741</v>
       </c>
     </row>
     <row r="326" ht="11" customHeight="true" outlineLevel="3">
@@ -4189,23 +4207,23 @@
         <v>325</v>
       </c>
       <c r="C326" s="18" t="n">
-        <v>4238</v>
+        <v>1940</v>
       </c>
     </row>
     <row r="327" ht="11" customHeight="true" outlineLevel="3">
       <c r="B327" s="17" t="s">
         <v>326</v>
       </c>
-      <c r="C327" s="11" t="n">
-        <v>7</v>
+      <c r="C327" s="18" t="n">
+        <v>4702</v>
       </c>
     </row>
     <row r="328" ht="11" customHeight="true" outlineLevel="3">
       <c r="B328" s="17" t="s">
         <v>327</v>
       </c>
-      <c r="C328" s="18" t="n">
-        <v>3750</v>
+      <c r="C328" s="11" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="329" ht="11" customHeight="true" outlineLevel="3">
@@ -4213,7 +4231,7 @@
         <v>328</v>
       </c>
       <c r="C329" s="18" t="n">
-        <v>17195</v>
+        <v>3628</v>
       </c>
     </row>
     <row r="330" ht="11" customHeight="true" outlineLevel="3">
@@ -4221,47 +4239,47 @@
         <v>329</v>
       </c>
       <c r="C330" s="18" t="n">
-        <v>1195</v>
+        <v>21479</v>
       </c>
     </row>
     <row r="331" ht="11" customHeight="true" outlineLevel="3">
       <c r="B331" s="17" t="s">
         <v>330</v>
       </c>
-      <c r="C331" s="11" t="n">
-        <v>194</v>
+      <c r="C331" s="18" t="n">
+        <v>1151</v>
       </c>
     </row>
     <row r="332" ht="11" customHeight="true" outlineLevel="3">
       <c r="B332" s="17" t="s">
         <v>331</v>
       </c>
-      <c r="C332" s="18" t="n">
-        <v>5687</v>
-      </c>
-    </row>
-    <row r="333" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B333" s="16" t="s">
+      <c r="C332" s="11" t="n">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="333" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B333" s="17" t="s">
         <v>332</v>
       </c>
-      <c r="C333" s="12" t="n">
-        <v>60967</v>
-      </c>
-    </row>
-    <row r="334" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B334" s="17" t="s">
+      <c r="C333" s="18" t="n">
+        <v>7716</v>
+      </c>
+    </row>
+    <row r="334" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B334" s="16" t="s">
         <v>333</v>
       </c>
-      <c r="C334" s="18" t="n">
-        <v>2253</v>
+      <c r="C334" s="12" t="n">
+        <v>69209</v>
       </c>
     </row>
     <row r="335" ht="11" customHeight="true" outlineLevel="3">
       <c r="B335" s="17" t="s">
         <v>334</v>
       </c>
-      <c r="C335" s="11" t="n">
-        <v>382</v>
+      <c r="C335" s="18" t="n">
+        <v>1745</v>
       </c>
     </row>
     <row r="336" ht="11" customHeight="true" outlineLevel="3">
@@ -4269,31 +4287,31 @@
         <v>335</v>
       </c>
       <c r="C336" s="11" t="n">
-        <v>694</v>
-      </c>
-    </row>
-    <row r="337" ht="22" customHeight="true" outlineLevel="3">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="337" ht="11" customHeight="true" outlineLevel="3">
       <c r="B337" s="17" t="s">
         <v>336</v>
       </c>
-      <c r="C337" s="11" t="n">
-        <v>376</v>
+      <c r="C337" s="18" t="n">
+        <v>1507</v>
       </c>
     </row>
     <row r="338" ht="22" customHeight="true" outlineLevel="3">
       <c r="B338" s="17" t="s">
         <v>337</v>
       </c>
-      <c r="C338" s="18" t="n">
-        <v>1288</v>
-      </c>
-    </row>
-    <row r="339" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C338" s="11" t="n">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="339" ht="22" customHeight="true" outlineLevel="3">
       <c r="B339" s="17" t="s">
         <v>338</v>
       </c>
-      <c r="C339" s="11" t="n">
-        <v>839</v>
+      <c r="C339" s="18" t="n">
+        <v>1183</v>
       </c>
     </row>
     <row r="340" ht="11" customHeight="true" outlineLevel="3">
@@ -4301,7 +4319,7 @@
         <v>339</v>
       </c>
       <c r="C340" s="11" t="n">
-        <v>511</v>
+        <v>527</v>
       </c>
     </row>
     <row r="341" ht="11" customHeight="true" outlineLevel="3">
@@ -4309,23 +4327,23 @@
         <v>340</v>
       </c>
       <c r="C341" s="11" t="n">
-        <v>556</v>
+        <v>551</v>
       </c>
     </row>
     <row r="342" ht="11" customHeight="true" outlineLevel="3">
       <c r="B342" s="17" t="s">
         <v>341</v>
       </c>
-      <c r="C342" s="18" t="n">
-        <v>1655</v>
+      <c r="C342" s="11" t="n">
+        <v>958</v>
       </c>
     </row>
     <row r="343" ht="11" customHeight="true" outlineLevel="3">
       <c r="B343" s="17" t="s">
         <v>342</v>
       </c>
-      <c r="C343" s="11" t="n">
-        <v>830</v>
+      <c r="C343" s="18" t="n">
+        <v>2786</v>
       </c>
     </row>
     <row r="344" ht="11" customHeight="true" outlineLevel="3">
@@ -4333,15 +4351,15 @@
         <v>343</v>
       </c>
       <c r="C344" s="11" t="n">
-        <v>678</v>
+        <v>708</v>
       </c>
     </row>
     <row r="345" ht="11" customHeight="true" outlineLevel="3">
       <c r="B345" s="17" t="s">
         <v>344</v>
       </c>
-      <c r="C345" s="11" t="n">
-        <v>297</v>
+      <c r="C345" s="18" t="n">
+        <v>1092</v>
       </c>
     </row>
     <row r="346" ht="11" customHeight="true" outlineLevel="3">
@@ -4349,7 +4367,7 @@
         <v>345</v>
       </c>
       <c r="C346" s="11" t="n">
-        <v>78</v>
+        <v>436</v>
       </c>
     </row>
     <row r="347" ht="11" customHeight="true" outlineLevel="3">
@@ -4357,7 +4375,7 @@
         <v>346</v>
       </c>
       <c r="C347" s="11" t="n">
-        <v>703</v>
+        <v>78</v>
       </c>
     </row>
     <row r="348" ht="11" customHeight="true" outlineLevel="3">
@@ -4365,7 +4383,7 @@
         <v>347</v>
       </c>
       <c r="C348" s="11" t="n">
-        <v>295</v>
+        <v>754</v>
       </c>
     </row>
     <row r="349" ht="11" customHeight="true" outlineLevel="3">
@@ -4373,15 +4391,15 @@
         <v>348</v>
       </c>
       <c r="C349" s="11" t="n">
-        <v>427</v>
+        <v>295</v>
       </c>
     </row>
     <row r="350" ht="11" customHeight="true" outlineLevel="3">
       <c r="B350" s="17" t="s">
         <v>349</v>
       </c>
-      <c r="C350" s="11" t="n">
-        <v>17</v>
+      <c r="C350" s="18" t="n">
+        <v>1143</v>
       </c>
     </row>
     <row r="351" ht="11" customHeight="true" outlineLevel="3">
@@ -4389,15 +4407,15 @@
         <v>350</v>
       </c>
       <c r="C351" s="11" t="n">
-        <v>397</v>
+        <v>703</v>
       </c>
     </row>
     <row r="352" ht="11" customHeight="true" outlineLevel="3">
       <c r="B352" s="17" t="s">
         <v>351</v>
       </c>
-      <c r="C352" s="18" t="n">
-        <v>1297</v>
+      <c r="C352" s="11" t="n">
+        <v>926</v>
       </c>
     </row>
     <row r="353" ht="11" customHeight="true" outlineLevel="3">
@@ -4405,7 +4423,7 @@
         <v>352</v>
       </c>
       <c r="C353" s="11" t="n">
-        <v>498</v>
+        <v>442</v>
       </c>
     </row>
     <row r="354" ht="11" customHeight="true" outlineLevel="3">
@@ -4413,7 +4431,7 @@
         <v>353</v>
       </c>
       <c r="C354" s="18" t="n">
-        <v>1061</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="355" ht="11" customHeight="true" outlineLevel="3">
@@ -4421,7 +4439,7 @@
         <v>354</v>
       </c>
       <c r="C355" s="11" t="n">
-        <v>491</v>
+        <v>764</v>
       </c>
     </row>
     <row r="356" ht="11" customHeight="true" outlineLevel="3">
@@ -4429,7 +4447,7 @@
         <v>355</v>
       </c>
       <c r="C356" s="11" t="n">
-        <v>828</v>
+        <v>784</v>
       </c>
     </row>
     <row r="357" ht="11" customHeight="true" outlineLevel="3">
@@ -4437,7 +4455,7 @@
         <v>356</v>
       </c>
       <c r="C357" s="11" t="n">
-        <v>140</v>
+        <v>130</v>
       </c>
     </row>
     <row r="358" ht="11" customHeight="true" outlineLevel="3">
@@ -4445,7 +4463,7 @@
         <v>357</v>
       </c>
       <c r="C358" s="18" t="n">
-        <v>3324</v>
+        <v>2529</v>
       </c>
     </row>
     <row r="359" ht="11" customHeight="true" outlineLevel="3">
@@ -4453,7 +4471,7 @@
         <v>358</v>
       </c>
       <c r="C359" s="18" t="n">
-        <v>1002</v>
+        <v>2126</v>
       </c>
     </row>
     <row r="360" ht="11" customHeight="true" outlineLevel="3">
@@ -4461,18 +4479,18 @@
         <v>359</v>
       </c>
       <c r="C360" s="11" t="n">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="361" ht="22" customHeight="true" outlineLevel="3">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="361" ht="11" customHeight="true" outlineLevel="3">
       <c r="B361" s="17" t="s">
         <v>360</v>
       </c>
       <c r="C361" s="11" t="n">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="362" ht="22" customHeight="true" outlineLevel="3">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="362" ht="11" customHeight="true" outlineLevel="3">
       <c r="B362" s="17" t="s">
         <v>361</v>
       </c>
@@ -4480,12 +4498,12 @@
         <v>104</v>
       </c>
     </row>
-    <row r="363" ht="11" customHeight="true" outlineLevel="3">
+    <row r="363" ht="22" customHeight="true" outlineLevel="3">
       <c r="B363" s="17" t="s">
         <v>362</v>
       </c>
       <c r="C363" s="11" t="n">
-        <v>231</v>
+        <v>38</v>
       </c>
     </row>
     <row r="364" ht="11" customHeight="true" outlineLevel="3">
@@ -4493,7 +4511,7 @@
         <v>363</v>
       </c>
       <c r="C364" s="11" t="n">
-        <v>245</v>
+        <v>164</v>
       </c>
     </row>
     <row r="365" ht="22" customHeight="true" outlineLevel="3">
@@ -4501,7 +4519,7 @@
         <v>364</v>
       </c>
       <c r="C365" s="11" t="n">
-        <v>124</v>
+        <v>660</v>
       </c>
     </row>
     <row r="366" ht="11" customHeight="true" outlineLevel="3">
@@ -4509,7 +4527,7 @@
         <v>365</v>
       </c>
       <c r="C366" s="11" t="n">
-        <v>257</v>
+        <v>186</v>
       </c>
     </row>
     <row r="367" ht="22" customHeight="true" outlineLevel="3">
@@ -4517,7 +4535,7 @@
         <v>366</v>
       </c>
       <c r="C367" s="11" t="n">
-        <v>754</v>
+        <v>843</v>
       </c>
     </row>
     <row r="368" ht="11" customHeight="true" outlineLevel="3">
@@ -4525,7 +4543,7 @@
         <v>367</v>
       </c>
       <c r="C368" s="11" t="n">
-        <v>253</v>
+        <v>270</v>
       </c>
     </row>
     <row r="369" ht="22" customHeight="true" outlineLevel="3">
@@ -4533,47 +4551,47 @@
         <v>368</v>
       </c>
       <c r="C369" s="11" t="n">
-        <v>818</v>
+        <v>745</v>
       </c>
     </row>
     <row r="370" ht="11" customHeight="true" outlineLevel="3">
       <c r="B370" s="17" t="s">
         <v>369</v>
       </c>
-      <c r="C370" s="11" t="n">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="371" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C370" s="18" t="n">
+        <v>11999</v>
+      </c>
+    </row>
+    <row r="371" ht="11" customHeight="true" outlineLevel="3">
       <c r="B371" s="17" t="s">
         <v>370</v>
       </c>
       <c r="C371" s="11" t="n">
-        <v>559</v>
+        <v>450</v>
       </c>
     </row>
     <row r="372" ht="11" customHeight="true" outlineLevel="3">
       <c r="B372" s="17" t="s">
         <v>371</v>
       </c>
-      <c r="C372" s="18" t="n">
-        <v>7892</v>
+      <c r="C372" s="11" t="n">
+        <v>299</v>
       </c>
     </row>
     <row r="373" ht="11" customHeight="true" outlineLevel="3">
       <c r="B373" s="17" t="s">
         <v>372</v>
       </c>
-      <c r="C373" s="11" t="n">
-        <v>480</v>
+      <c r="C373" s="18" t="n">
+        <v>17694</v>
       </c>
     </row>
     <row r="374" ht="11" customHeight="true" outlineLevel="3">
       <c r="B374" s="17" t="s">
         <v>373</v>
       </c>
-      <c r="C374" s="11" t="n">
-        <v>521</v>
+      <c r="C374" s="18" t="n">
+        <v>7860</v>
       </c>
     </row>
     <row r="375" ht="11" customHeight="true" outlineLevel="3">
@@ -4581,31 +4599,31 @@
         <v>374</v>
       </c>
       <c r="C375" s="18" t="n">
-        <v>18805</v>
+        <v>2823</v>
       </c>
     </row>
     <row r="376" ht="11" customHeight="true" outlineLevel="3">
       <c r="B376" s="17" t="s">
         <v>375</v>
       </c>
-      <c r="C376" s="18" t="n">
-        <v>5837</v>
+      <c r="C376" s="11" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="377" ht="11" customHeight="true" outlineLevel="3">
       <c r="B377" s="17" t="s">
         <v>376</v>
       </c>
-      <c r="C377" s="18" t="n">
-        <v>1430</v>
-      </c>
-    </row>
-    <row r="378" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B378" s="17" t="s">
+      <c r="C377" s="11" t="n">
+        <v>929</v>
+      </c>
+    </row>
+    <row r="378" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B378" s="16" t="s">
         <v>377</v>
       </c>
-      <c r="C378" s="11" t="n">
-        <v>93</v>
+      <c r="C378" s="14" t="n">
+        <v>880</v>
       </c>
     </row>
     <row r="379" ht="11" customHeight="true" outlineLevel="3">
@@ -4613,15 +4631,15 @@
         <v>378</v>
       </c>
       <c r="C379" s="11" t="n">
-        <v>984</v>
-      </c>
-    </row>
-    <row r="380" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B380" s="16" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="380" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B380" s="17" t="s">
         <v>379</v>
       </c>
-      <c r="C380" s="14" t="n">
-        <v>253</v>
+      <c r="C380" s="11" t="n">
+        <v>85</v>
       </c>
     </row>
     <row r="381" ht="11" customHeight="true" outlineLevel="3">
@@ -4629,7 +4647,7 @@
         <v>380</v>
       </c>
       <c r="C381" s="11" t="n">
-        <v>37</v>
+        <v>295</v>
       </c>
     </row>
     <row r="382" ht="11" customHeight="true" outlineLevel="3">
@@ -4637,15 +4655,15 @@
         <v>381</v>
       </c>
       <c r="C382" s="11" t="n">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="383" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B383" s="17" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="383" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B383" s="16" t="s">
         <v>382</v>
       </c>
-      <c r="C383" s="11" t="n">
-        <v>43</v>
+      <c r="C383" s="12" t="n">
+        <v>61838</v>
       </c>
     </row>
     <row r="384" ht="11" customHeight="true" outlineLevel="3">
@@ -4653,39 +4671,39 @@
         <v>383</v>
       </c>
       <c r="C384" s="11" t="n">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="385" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B385" s="16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="385" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B385" s="17" t="s">
         <v>384</v>
       </c>
-      <c r="C385" s="12" t="n">
-        <v>44680</v>
-      </c>
-    </row>
-    <row r="386" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C385" s="11" t="n">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="386" ht="22" customHeight="true" outlineLevel="3">
       <c r="B386" s="17" t="s">
         <v>385</v>
       </c>
-      <c r="C386" s="11" t="n">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="387" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C386" s="18" t="n">
+        <v>3362</v>
+      </c>
+    </row>
+    <row r="387" ht="22" customHeight="true" outlineLevel="3">
       <c r="B387" s="17" t="s">
         <v>386</v>
       </c>
-      <c r="C387" s="11" t="n">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="388" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C387" s="18" t="n">
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="388" ht="22" customHeight="true" outlineLevel="3">
       <c r="B388" s="17" t="s">
         <v>387</v>
       </c>
       <c r="C388" s="11" t="n">
-        <v>190</v>
+        <v>84</v>
       </c>
     </row>
     <row r="389" ht="22" customHeight="true" outlineLevel="3">
@@ -4693,15 +4711,15 @@
         <v>388</v>
       </c>
       <c r="C389" s="11" t="n">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="390" ht="22" customHeight="true" outlineLevel="3">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="390" ht="11" customHeight="true" outlineLevel="3">
       <c r="B390" s="17" t="s">
         <v>389</v>
       </c>
-      <c r="C390" s="11" t="n">
-        <v>169</v>
+      <c r="C390" s="18" t="n">
+        <v>3128</v>
       </c>
     </row>
     <row r="391" ht="11" customHeight="true" outlineLevel="3">
@@ -4709,55 +4727,55 @@
         <v>390</v>
       </c>
       <c r="C391" s="11" t="n">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="392" ht="11" customHeight="true" outlineLevel="3">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="392" ht="22" customHeight="true" outlineLevel="3">
       <c r="B392" s="17" t="s">
         <v>391</v>
       </c>
-      <c r="C392" s="11" t="n">
-        <v>44</v>
+      <c r="C392" s="18" t="n">
+        <v>5233</v>
       </c>
     </row>
     <row r="393" ht="22" customHeight="true" outlineLevel="3">
       <c r="B393" s="17" t="s">
         <v>392</v>
       </c>
-      <c r="C393" s="18" t="n">
-        <v>3896</v>
-      </c>
-    </row>
-    <row r="394" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C393" s="11" t="n">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="394" ht="11" customHeight="true" outlineLevel="3">
       <c r="B394" s="17" t="s">
         <v>393</v>
       </c>
       <c r="C394" s="11" t="n">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="395" ht="22" customHeight="true" outlineLevel="3">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="395" ht="11" customHeight="true" outlineLevel="3">
       <c r="B395" s="17" t="s">
         <v>394</v>
       </c>
       <c r="C395" s="11" t="n">
-        <v>51</v>
+        <v>231</v>
       </c>
     </row>
     <row r="396" ht="11" customHeight="true" outlineLevel="3">
       <c r="B396" s="17" t="s">
         <v>395</v>
       </c>
-      <c r="C396" s="11" t="n">
-        <v>48</v>
+      <c r="C396" s="18" t="n">
+        <v>2624</v>
       </c>
     </row>
     <row r="397" ht="11" customHeight="true" outlineLevel="3">
       <c r="B397" s="17" t="s">
         <v>396</v>
       </c>
-      <c r="C397" s="11" t="n">
-        <v>59</v>
+      <c r="C397" s="18" t="n">
+        <v>1760</v>
       </c>
     </row>
     <row r="398" ht="11" customHeight="true" outlineLevel="3">
@@ -4765,15 +4783,15 @@
         <v>397</v>
       </c>
       <c r="C398" s="11" t="n">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="399" ht="11" customHeight="true" outlineLevel="3">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="399" ht="22" customHeight="true" outlineLevel="3">
       <c r="B399" s="17" t="s">
         <v>398</v>
       </c>
       <c r="C399" s="11" t="n">
-        <v>251</v>
+        <v>36</v>
       </c>
     </row>
     <row r="400" ht="22" customHeight="true" outlineLevel="3">
@@ -4781,7 +4799,7 @@
         <v>399</v>
       </c>
       <c r="C400" s="11" t="n">
-        <v>587</v>
+        <v>28</v>
       </c>
     </row>
     <row r="401" ht="22" customHeight="true" outlineLevel="3">
@@ -4789,15 +4807,15 @@
         <v>400</v>
       </c>
       <c r="C401" s="11" t="n">
-        <v>42</v>
+        <v>168</v>
       </c>
     </row>
     <row r="402" ht="22" customHeight="true" outlineLevel="3">
       <c r="B402" s="17" t="s">
         <v>401</v>
       </c>
-      <c r="C402" s="18" t="n">
-        <v>4214</v>
+      <c r="C402" s="11" t="n">
+        <v>961</v>
       </c>
     </row>
     <row r="403" ht="22" customHeight="true" outlineLevel="3">
@@ -4813,23 +4831,23 @@
         <v>403</v>
       </c>
       <c r="C404" s="11" t="n">
-        <v>110</v>
+        <v>44</v>
       </c>
     </row>
     <row r="405" ht="22" customHeight="true" outlineLevel="3">
       <c r="B405" s="17" t="s">
         <v>404</v>
       </c>
-      <c r="C405" s="18" t="n">
-        <v>3915</v>
+      <c r="C405" s="11" t="n">
+        <v>660</v>
       </c>
     </row>
     <row r="406" ht="22" customHeight="true" outlineLevel="3">
       <c r="B406" s="17" t="s">
         <v>405</v>
       </c>
-      <c r="C406" s="18" t="n">
-        <v>4023</v>
+      <c r="C406" s="11" t="n">
+        <v>458</v>
       </c>
     </row>
     <row r="407" ht="22" customHeight="true" outlineLevel="3">
@@ -4837,15 +4855,15 @@
         <v>406</v>
       </c>
       <c r="C407" s="11" t="n">
-        <v>74</v>
+        <v>528</v>
       </c>
     </row>
     <row r="408" ht="22" customHeight="true" outlineLevel="3">
       <c r="B408" s="17" t="s">
         <v>407</v>
       </c>
-      <c r="C408" s="11" t="n">
-        <v>36</v>
+      <c r="C408" s="18" t="n">
+        <v>2177</v>
       </c>
     </row>
     <row r="409" ht="22" customHeight="true" outlineLevel="3">
@@ -4853,7 +4871,7 @@
         <v>408</v>
       </c>
       <c r="C409" s="11" t="n">
-        <v>107</v>
+        <v>38</v>
       </c>
     </row>
     <row r="410" ht="22" customHeight="true" outlineLevel="3">
@@ -4861,7 +4879,7 @@
         <v>409</v>
       </c>
       <c r="C410" s="11" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
     </row>
     <row r="411" ht="22" customHeight="true" outlineLevel="3">
@@ -4869,7 +4887,7 @@
         <v>410</v>
       </c>
       <c r="C411" s="11" t="n">
-        <v>18</v>
+        <v>354</v>
       </c>
     </row>
     <row r="412" ht="22" customHeight="true" outlineLevel="3">
@@ -4877,7 +4895,7 @@
         <v>411</v>
       </c>
       <c r="C412" s="11" t="n">
-        <v>35</v>
+        <v>360</v>
       </c>
     </row>
     <row r="413" ht="22" customHeight="true" outlineLevel="3">
@@ -4885,15 +4903,15 @@
         <v>412</v>
       </c>
       <c r="C413" s="11" t="n">
-        <v>79</v>
+        <v>50</v>
       </c>
     </row>
     <row r="414" ht="22" customHeight="true" outlineLevel="3">
       <c r="B414" s="17" t="s">
         <v>413</v>
       </c>
-      <c r="C414" s="11" t="n">
-        <v>543</v>
+      <c r="C414" s="18" t="n">
+        <v>3797</v>
       </c>
     </row>
     <row r="415" ht="22" customHeight="true" outlineLevel="3">
@@ -4901,7 +4919,7 @@
         <v>414</v>
       </c>
       <c r="C415" s="11" t="n">
-        <v>198</v>
+        <v>726</v>
       </c>
     </row>
     <row r="416" ht="22" customHeight="true" outlineLevel="3">
@@ -4909,7 +4927,7 @@
         <v>415</v>
       </c>
       <c r="C416" s="11" t="n">
-        <v>2</v>
+        <v>50</v>
       </c>
     </row>
     <row r="417" ht="22" customHeight="true" outlineLevel="3">
@@ -4917,15 +4935,15 @@
         <v>416</v>
       </c>
       <c r="C417" s="11" t="n">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="418" ht="11" customHeight="true" outlineLevel="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="418" ht="22" customHeight="true" outlineLevel="3">
       <c r="B418" s="17" t="s">
         <v>417</v>
       </c>
       <c r="C418" s="11" t="n">
-        <v>209</v>
+        <v>26</v>
       </c>
     </row>
     <row r="419" ht="11" customHeight="true" outlineLevel="3">
@@ -4933,15 +4951,15 @@
         <v>418</v>
       </c>
       <c r="C419" s="11" t="n">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="420" ht="22" customHeight="true" outlineLevel="3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="420" ht="11" customHeight="true" outlineLevel="3">
       <c r="B420" s="17" t="s">
         <v>419</v>
       </c>
       <c r="C420" s="11" t="n">
-        <v>66</v>
+        <v>922</v>
       </c>
     </row>
     <row r="421" ht="22" customHeight="true" outlineLevel="3">
@@ -4949,7 +4967,7 @@
         <v>420</v>
       </c>
       <c r="C421" s="11" t="n">
-        <v>24</v>
+        <v>59</v>
       </c>
     </row>
     <row r="422" ht="22" customHeight="true" outlineLevel="3">
@@ -4957,15 +4975,15 @@
         <v>421</v>
       </c>
       <c r="C422" s="11" t="n">
-        <v>77</v>
+        <v>23</v>
       </c>
     </row>
     <row r="423" ht="22" customHeight="true" outlineLevel="3">
       <c r="B423" s="17" t="s">
         <v>422</v>
       </c>
-      <c r="C423" s="11" t="n">
-        <v>20</v>
+      <c r="C423" s="18" t="n">
+        <v>1416</v>
       </c>
     </row>
     <row r="424" ht="22" customHeight="true" outlineLevel="3">
@@ -4973,7 +4991,7 @@
         <v>423</v>
       </c>
       <c r="C424" s="11" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="425" ht="22" customHeight="true" outlineLevel="3">
@@ -4981,15 +4999,15 @@
         <v>424</v>
       </c>
       <c r="C425" s="11" t="n">
-        <v>140</v>
+        <v>72</v>
       </c>
     </row>
     <row r="426" ht="22" customHeight="true" outlineLevel="3">
       <c r="B426" s="17" t="s">
         <v>425</v>
       </c>
-      <c r="C426" s="18" t="n">
-        <v>4489</v>
+      <c r="C426" s="11" t="n">
+        <v>260</v>
       </c>
     </row>
     <row r="427" ht="22" customHeight="true" outlineLevel="3">
@@ -4997,39 +5015,39 @@
         <v>426</v>
       </c>
       <c r="C427" s="11" t="n">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="428" ht="11" customHeight="true" outlineLevel="3">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="428" ht="22" customHeight="true" outlineLevel="3">
       <c r="B428" s="17" t="s">
         <v>427</v>
       </c>
-      <c r="C428" s="11" t="n">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="429" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C428" s="18" t="n">
+        <v>3914</v>
+      </c>
+    </row>
+    <row r="429" ht="22" customHeight="true" outlineLevel="3">
       <c r="B429" s="17" t="s">
         <v>428</v>
       </c>
       <c r="C429" s="11" t="n">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="430" ht="22" customHeight="true" outlineLevel="3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="430" ht="11" customHeight="true" outlineLevel="3">
       <c r="B430" s="17" t="s">
         <v>429</v>
       </c>
-      <c r="C430" s="11" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="431" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C430" s="18" t="n">
+        <v>1722</v>
+      </c>
+    </row>
+    <row r="431" ht="22" customHeight="true" outlineLevel="3">
       <c r="B431" s="17" t="s">
         <v>430</v>
       </c>
       <c r="C431" s="11" t="n">
-        <v>195</v>
+        <v>500</v>
       </c>
     </row>
     <row r="432" ht="11" customHeight="true" outlineLevel="3">
@@ -5037,39 +5055,39 @@
         <v>431</v>
       </c>
       <c r="C432" s="11" t="n">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="433" ht="11" customHeight="true" outlineLevel="3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="433" ht="22" customHeight="true" outlineLevel="3">
       <c r="B433" s="17" t="s">
         <v>432</v>
       </c>
       <c r="C433" s="11" t="n">
-        <v>-8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="434" ht="11" customHeight="true" outlineLevel="3">
       <c r="B434" s="17" t="s">
         <v>433</v>
       </c>
-      <c r="C434" s="11" t="n">
-        <v>241</v>
+      <c r="C434" s="18" t="n">
+        <v>1666</v>
       </c>
     </row>
     <row r="435" ht="11" customHeight="true" outlineLevel="3">
       <c r="B435" s="17" t="s">
         <v>434</v>
       </c>
-      <c r="C435" s="18" t="n">
-        <v>5067</v>
-      </c>
-    </row>
-    <row r="436" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C435" s="11" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="436" ht="11" customHeight="true" outlineLevel="3">
       <c r="B436" s="17" t="s">
         <v>435</v>
       </c>
       <c r="C436" s="11" t="n">
-        <v>801</v>
+        <v>32</v>
       </c>
     </row>
     <row r="437" ht="11" customHeight="true" outlineLevel="3">
@@ -5077,47 +5095,47 @@
         <v>436</v>
       </c>
       <c r="C437" s="11" t="n">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="438" ht="22" customHeight="true" outlineLevel="3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="438" ht="11" customHeight="true" outlineLevel="3">
       <c r="B438" s="17" t="s">
         <v>437</v>
       </c>
-      <c r="C438" s="11" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="439" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C438" s="18" t="n">
+        <v>4001</v>
+      </c>
+    </row>
+    <row r="439" ht="22" customHeight="true" outlineLevel="3">
       <c r="B439" s="17" t="s">
         <v>438</v>
       </c>
       <c r="C439" s="11" t="n">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="440" ht="11" customHeight="true" outlineLevel="3">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="440" ht="22" customHeight="true" outlineLevel="3">
       <c r="B440" s="17" t="s">
         <v>439</v>
       </c>
       <c r="C440" s="11" t="n">
-        <v>708</v>
+        <v>2</v>
       </c>
     </row>
     <row r="441" ht="11" customHeight="true" outlineLevel="3">
       <c r="B441" s="17" t="s">
         <v>440</v>
       </c>
-      <c r="C441" s="11" t="n">
-        <v>785</v>
-      </c>
-    </row>
-    <row r="442" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C441" s="18" t="n">
+        <v>4385</v>
+      </c>
+    </row>
+    <row r="442" ht="22" customHeight="true" outlineLevel="3">
       <c r="B442" s="17" t="s">
         <v>441</v>
       </c>
       <c r="C442" s="11" t="n">
-        <v>42</v>
+        <v>4</v>
       </c>
     </row>
     <row r="443" ht="11" customHeight="true" outlineLevel="3">
@@ -5125,7 +5143,7 @@
         <v>442</v>
       </c>
       <c r="C443" s="11" t="n">
-        <v>222</v>
+        <v>45</v>
       </c>
     </row>
     <row r="444" ht="11" customHeight="true" outlineLevel="3">
@@ -5133,23 +5151,71 @@
         <v>443</v>
       </c>
       <c r="C444" s="18" t="n">
-        <v>6160</v>
-      </c>
-    </row>
-    <row r="445" ht="22" customHeight="true" outlineLevel="3">
+        <v>1085</v>
+      </c>
+    </row>
+    <row r="445" ht="11" customHeight="true" outlineLevel="3">
       <c r="B445" s="17" t="s">
         <v>444</v>
       </c>
       <c r="C445" s="11" t="n">
-        <v>888</v>
+        <v>624</v>
       </c>
     </row>
     <row r="446" ht="11" customHeight="true" outlineLevel="3">
       <c r="B446" s="17" t="s">
         <v>445</v>
       </c>
-      <c r="C446" s="18" t="n">
-        <v>3408</v>
+      <c r="C446" s="11" t="n">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="447" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B447" s="17" t="s">
+        <v>446</v>
+      </c>
+      <c r="C447" s="11" t="n">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="448" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B448" s="17" t="s">
+        <v>447</v>
+      </c>
+      <c r="C448" s="18" t="n">
+        <v>1863</v>
+      </c>
+    </row>
+    <row r="449" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B449" s="17" t="s">
+        <v>448</v>
+      </c>
+      <c r="C449" s="11" t="n">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="450" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B450" s="17" t="s">
+        <v>449</v>
+      </c>
+      <c r="C450" s="18" t="n">
+        <v>3946</v>
+      </c>
+    </row>
+    <row r="451" ht="22" customHeight="true" outlineLevel="3">
+      <c r="B451" s="17" t="s">
+        <v>450</v>
+      </c>
+      <c r="C451" s="11" t="n">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="452" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B452" s="17" t="s">
+        <v>451</v>
+      </c>
+      <c r="C452" s="18" t="n">
+        <v>1828</v>
       </c>
     </row>
   </sheetData>

</xml_diff>